<commit_message>
Conducted extractions for 4 PDFs. Added 3 new PDFs to extraction list.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B4DB32A-2912-44D5-91C2-92F843E5A14D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C281114D-EEC9-4F30-9F9E-4ECD04BF7EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="57">
   <si>
     <t>PMID</t>
   </si>
@@ -138,6 +138,60 @@
   </si>
   <si>
     <t>Antiphage; Nuclease</t>
+  </si>
+  <si>
+    <t>Paper_title</t>
+  </si>
+  <si>
+    <t>Uniprot_accession</t>
+  </si>
+  <si>
+    <t>Uniparc_accession</t>
+  </si>
+  <si>
+    <t>The pan-immune system of bacteria: antiviral defence as a community resource</t>
+  </si>
+  <si>
+    <t>tadA, an essential tRNA-specific adenosine deaminase from Escherichia coli</t>
+  </si>
+  <si>
+    <t>tadA</t>
+  </si>
+  <si>
+    <t>P68398</t>
+  </si>
+  <si>
+    <t>No obvious immune function</t>
+  </si>
+  <si>
+    <t>Not assesed</t>
+  </si>
+  <si>
+    <t>Not assessed</t>
+  </si>
+  <si>
+    <t>tRNA binding; tRNA deamination</t>
+  </si>
+  <si>
+    <t>34% sequence-similar to yeast tRNA deaminase subunit Tad2p.</t>
+  </si>
+  <si>
+    <t>Abortive Infection: Bacterial Suicide as an Antiviral Immune Strategy</t>
+  </si>
+  <si>
+    <t>CBASS</t>
+  </si>
+  <si>
+    <t>Intracellular pathogen sensing; abortive infection</t>
+  </si>
+  <si>
+    <t>Diversity and classification of cyclic-oligonucleotide-based anti-phage signalling systems</t>
+  </si>
+  <si>
+    <t>Does not meet gold standard; in-silico analysis only</t>
+  </si>
+  <si>
+    <t>In-silico analysis only; leads into PMIDs 31533127, 30787435, 31932165, 32544385</t>
   </si>
 </sst>
 </file>
@@ -998,171 +1052,362 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="8" max="9" width="17.36328125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>31695182</v>
+        <v>12110595</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="b">
+        <v>43</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="b">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
       <c r="E2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>17</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
       </c>
       <c r="I2" t="s">
         <v>15</v>
       </c>
       <c r="J2" t="s">
+        <v>47</v>
+      </c>
+      <c r="K2" t="s">
+        <v>47</v>
+      </c>
+      <c r="L2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2" t="s">
+        <v>49</v>
+      </c>
+      <c r="N2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>31695182</v>
+      </c>
+      <c r="B6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" t="s">
         <v>15</v>
       </c>
-      <c r="K2" t="s">
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" t="s">
+        <v>47</v>
+      </c>
+      <c r="K6" t="s">
+        <v>47</v>
+      </c>
+      <c r="L6" t="s">
+        <v>47</v>
+      </c>
+      <c r="M6" t="s">
+        <v>48</v>
+      </c>
+      <c r="N6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>31695182</v>
+      </c>
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" t="s">
         <v>15</v>
       </c>
-      <c r="L2" t="s">
+      <c r="H7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" t="s">
+        <v>47</v>
+      </c>
+      <c r="K7" t="s">
+        <v>47</v>
+      </c>
+      <c r="L7" t="s">
+        <v>47</v>
+      </c>
+      <c r="M7" t="s">
+        <v>48</v>
+      </c>
+      <c r="N7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>31695182</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" t="s">
         <v>15</v>
       </c>
-      <c r="M2" t="s">
+      <c r="H8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" t="s">
+        <v>47</v>
+      </c>
+      <c r="K8" t="s">
+        <v>47</v>
+      </c>
+      <c r="L8" t="s">
+        <v>47</v>
+      </c>
+      <c r="M8" t="s">
+        <v>48</v>
+      </c>
+      <c r="N8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>31695182</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" t="b">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" t="s">
+        <v>48</v>
+      </c>
+      <c r="K9" t="s">
+        <v>48</v>
+      </c>
+      <c r="L9" t="s">
+        <v>48</v>
+      </c>
+      <c r="M9" t="s">
+        <v>48</v>
+      </c>
+      <c r="N9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>32559405</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J10" t="s">
+        <v>48</v>
+      </c>
+      <c r="K10" t="s">
+        <v>48</v>
+      </c>
+      <c r="L10" t="s">
+        <v>48</v>
+      </c>
+      <c r="M10" t="s">
+        <v>48</v>
+      </c>
+      <c r="N10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>32839535</v>
+      </c>
+      <c r="B11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" t="s">
+        <v>48</v>
+      </c>
+      <c r="I11" t="s">
+        <v>52</v>
+      </c>
+      <c r="J11" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>31695182</v>
-      </c>
-      <c r="B3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" t="b">
+      <c r="K11" t="s">
+        <v>15</v>
+      </c>
+      <c r="L11" t="b">
         <v>0</v>
       </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L3" t="s">
-        <v>15</v>
-      </c>
-      <c r="M3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>31695182</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L4" t="s">
-        <v>15</v>
-      </c>
-      <c r="M4" t="s">
-        <v>24</v>
+      <c r="M11" t="s">
+        <v>53</v>
+      </c>
+      <c r="N11" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Conducted extractions for PDF 30787435.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C281114D-EEC9-4F30-9F9E-4ECD04BF7EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D36D5610-973E-4DEC-8A46-DEB4BB59412F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="70">
   <si>
     <t>PMID</t>
   </si>
@@ -95,9 +95,6 @@
     <t>Streptococcus pyogenes serotype M1</t>
   </si>
   <si>
-    <t>Cas9 is not endogenously expressed in E. coli.</t>
-  </si>
-  <si>
     <t>Data_source</t>
   </si>
   <si>
@@ -173,9 +170,6 @@
     <t>tRNA binding; tRNA deamination</t>
   </si>
   <si>
-    <t>34% sequence-similar to yeast tRNA deaminase subunit Tad2p.</t>
-  </si>
-  <si>
     <t>Abortive Infection: Bacterial Suicide as an Antiviral Immune Strategy</t>
   </si>
   <si>
@@ -192,6 +186,51 @@
   </si>
   <si>
     <t>In-silico analysis only; leads into PMIDs 31533127, 30787435, 31932165, 32544385</t>
+  </si>
+  <si>
+    <t>Bacterial cGAS-like enzymes synthesize diverse nucleotide signals</t>
+  </si>
+  <si>
+    <t>dncV</t>
+  </si>
+  <si>
+    <t>Q9KVG7</t>
+  </si>
+  <si>
+    <t>Vibrio cholerae</t>
+  </si>
+  <si>
+    <t>Meets gold standard</t>
+  </si>
+  <si>
+    <t>Protein full name: Cyclic GMP-AMP synthase</t>
+  </si>
+  <si>
+    <t>34% sequence-similar to yeast tRNA deaminase subunit Tad2p</t>
+  </si>
+  <si>
+    <t>Cas9 is not endogenously expressed in E. coli</t>
+  </si>
+  <si>
+    <t>cdnE</t>
+  </si>
+  <si>
+    <t>Q6XGD5</t>
+  </si>
+  <si>
+    <t>Intracellular pathogen sensing; cGAMP synthesis; phospholipase activation</t>
+  </si>
+  <si>
+    <t>Protein full name: Cyclic UMP-AMP synthase; homologue to dncV; crystal structure conducted on homologue in Rhodothermus marinus</t>
+  </si>
+  <si>
+    <t>biochemical deconvolution; active-site mutation; product radiolabelling</t>
+  </si>
+  <si>
+    <t>product radiolabelling</t>
+  </si>
+  <si>
+    <t>HEK293T</t>
   </si>
 </sst>
 </file>
@@ -1063,7 +1102,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1075,10 +1114,10 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" t="s">
         <v>40</v>
-      </c>
-      <c r="G1" t="s">
-        <v>41</v>
       </c>
       <c r="H1" t="s">
         <v>6</v>
@@ -1107,19 +1146,19 @@
         <v>12110595</v>
       </c>
       <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" t="s">
         <v>43</v>
-      </c>
-      <c r="C2" t="s">
-        <v>44</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G2" t="s">
         <v>15</v>
@@ -1131,19 +1170,107 @@
         <v>15</v>
       </c>
       <c r="J2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>30787435</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>58</v>
+      </c>
+      <c r="I3" t="s">
         <v>50</v>
+      </c>
+      <c r="J3" t="s">
+        <v>68</v>
+      </c>
+      <c r="K3" t="s">
+        <v>69</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>65</v>
+      </c>
+      <c r="N3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>30787435</v>
+      </c>
+      <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J4" t="s">
+        <v>67</v>
+      </c>
+      <c r="K4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
+        <v>36</v>
+      </c>
+      <c r="N4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
@@ -1151,7 +1278,7 @@
         <v>31695182</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -1175,19 +1302,19 @@
         <v>18</v>
       </c>
       <c r="J6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
@@ -1195,7 +1322,7 @@
         <v>31695182</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
         <v>19</v>
@@ -1219,19 +1346,19 @@
         <v>18</v>
       </c>
       <c r="J7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
@@ -1239,7 +1366,7 @@
         <v>31695182</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -1263,19 +1390,19 @@
         <v>18</v>
       </c>
       <c r="J8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N8" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
@@ -1283,10 +1410,10 @@
         <v>31695182</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D9" t="b">
         <v>0</v>
@@ -1295,31 +1422,31 @@
         <v>14</v>
       </c>
       <c r="F9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
@@ -1327,10 +1454,10 @@
         <v>32559405</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D10" t="b">
         <v>0</v>
@@ -1339,31 +1466,31 @@
         <v>14</v>
       </c>
       <c r="F10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
@@ -1371,28 +1498,28 @@
         <v>32839535</v>
       </c>
       <c r="B11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D11" t="b">
         <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J11" t="s">
         <v>15</v>
@@ -1404,10 +1531,10 @@
         <v>0</v>
       </c>
       <c r="M11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="N11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1437,10 +1564,10 @@
         <v>7</v>
       </c>
       <c r="F1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" t="s">
         <v>25</v>
-      </c>
-      <c r="G1" t="s">
-        <v>26</v>
       </c>
       <c r="H1" t="s">
         <v>8</v>
@@ -1472,7 +1599,7 @@
         <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G2" t="s">
         <v>14</v>
@@ -1481,13 +1608,13 @@
         <v>15</v>
       </c>
       <c r="I2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J2" t="b">
         <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
@@ -1507,7 +1634,7 @@
         <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G3" t="s">
         <v>14</v>
@@ -1519,7 +1646,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
@@ -1539,7 +1666,7 @@
         <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
         <v>14</v>
@@ -1551,18 +1678,18 @@
         <v>0</v>
       </c>
       <c r="K4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="D5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J5" t="s">
         <v>15</v>
       </c>
       <c r="K5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
@@ -1570,7 +1697,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
@@ -1578,7 +1705,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
@@ -1586,7 +1713,7 @@
         <v>15</v>
       </c>
       <c r="K8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
@@ -1594,7 +1721,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
@@ -1602,7 +1729,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Conducted extraction for 31932165. Added 1 more PDF to extraction list.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D36D5610-973E-4DEC-8A46-DEB4BB59412F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368A00CE-CBE0-4545-A027-64F42D07F7B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="88">
   <si>
     <t>PMID</t>
   </si>
@@ -176,9 +176,6 @@
     <t>CBASS</t>
   </si>
   <si>
-    <t>Intracellular pathogen sensing; abortive infection</t>
-  </si>
-  <si>
     <t>Diversity and classification of cyclic-oligonucleotide-based anti-phage signalling systems</t>
   </si>
   <si>
@@ -203,9 +200,6 @@
     <t>Meets gold standard</t>
   </si>
   <si>
-    <t>Protein full name: Cyclic GMP-AMP synthase</t>
-  </si>
-  <si>
     <t>34% sequence-similar to yeast tRNA deaminase subunit Tad2p</t>
   </si>
   <si>
@@ -218,12 +212,6 @@
     <t>Q6XGD5</t>
   </si>
   <si>
-    <t>Intracellular pathogen sensing; cGAMP synthesis; phospholipase activation</t>
-  </si>
-  <si>
-    <t>Protein full name: Cyclic UMP-AMP synthase; homologue to dncV; crystal structure conducted on homologue in Rhodothermus marinus</t>
-  </si>
-  <si>
     <t>biochemical deconvolution; active-site mutation; product radiolabelling</t>
   </si>
   <si>
@@ -231,6 +219,72 @@
   </si>
   <si>
     <t>HEK293T</t>
+  </si>
+  <si>
+    <t>abortive infection; intracellular pathogen sensing</t>
+  </si>
+  <si>
+    <t>HORMA Domain Proteins and a Trip13-like ATPase Regulate Bacterial cGAS-like Enzymes to Mediate Bacteriophage Immunity</t>
+  </si>
+  <si>
+    <t>cdnC</t>
+  </si>
+  <si>
+    <t>D7Y2H2</t>
+  </si>
+  <si>
+    <t>Pseudomonas aeruginosa</t>
+  </si>
+  <si>
+    <t>P0DTF7</t>
+  </si>
+  <si>
+    <t>cdnD</t>
+  </si>
+  <si>
+    <t>second-messenger synthesis assay</t>
+  </si>
+  <si>
+    <t>second-messenger synthesis assay; yeast two-hybrid assay; major-product liquid chromatography; major-product MS2 fragmentation</t>
+  </si>
+  <si>
+    <t>abortive infection; intracellular pathogen sensing; second messenger synthesis</t>
+  </si>
+  <si>
+    <t>abortive infection; intracellular pathogen sensing; second messenger synthesis; cGAMP synthesis; phospholipase activation</t>
+  </si>
+  <si>
+    <t>abortive infection; intracellular pathogen sensing; second-messenger synthesis</t>
+  </si>
+  <si>
+    <t>protein full name: Cyclic GMP-AMP synthase</t>
+  </si>
+  <si>
+    <t>protein full name: Cyclic UMP-AMP synthase; homologue to dncV; crystal structure conducted on homologue in Rhodothermus marinus</t>
+  </si>
+  <si>
+    <t>P0DTF6</t>
+  </si>
+  <si>
+    <t>cap7</t>
+  </si>
+  <si>
+    <t>AKA HORMA2</t>
+  </si>
+  <si>
+    <t>AKA HORMA1</t>
+  </si>
+  <si>
+    <t>induced immunity via abortive infection</t>
+  </si>
+  <si>
+    <t>No identifiable UniProt ID</t>
+  </si>
+  <si>
+    <t>Rhizobiales</t>
+  </si>
+  <si>
+    <t>AKA Trip13, Pch2; authors specify only organism genus</t>
   </si>
 </sst>
 </file>
@@ -1091,7 +1145,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="8" max="9" width="17.36328125" customWidth="1"/>
@@ -1182,7 +1236,7 @@
         <v>48</v>
       </c>
       <c r="N2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
@@ -1190,43 +1244,43 @@
         <v>30787435</v>
       </c>
       <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" t="s">
         <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>56</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
         <v>57</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>58</v>
       </c>
       <c r="I3" t="s">
         <v>50</v>
       </c>
       <c r="J3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="K3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="L3" t="b">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="N3" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
@@ -1234,19 +1288,19 @@
         <v>30787435</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G4" t="s">
         <v>15</v>
@@ -1258,7 +1312,7 @@
         <v>50</v>
       </c>
       <c r="J4" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="K4" t="s">
         <v>15</v>
@@ -1267,10 +1321,54 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="N4" t="s">
-        <v>66</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>31695182</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" t="s">
+        <v>46</v>
+      </c>
+      <c r="K5" t="s">
+        <v>46</v>
+      </c>
+      <c r="L5" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" t="s">
+        <v>47</v>
+      </c>
+      <c r="N5" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
@@ -1281,7 +1379,7 @@
         <v>41</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -1290,7 +1388,7 @@
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G6" t="s">
         <v>15</v>
@@ -1325,7 +1423,7 @@
         <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -1334,13 +1432,13 @@
         <v>14</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G7" t="s">
         <v>15</v>
       </c>
       <c r="H7" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="I7" t="s">
         <v>18</v>
@@ -1358,7 +1456,7 @@
         <v>47</v>
       </c>
       <c r="N7" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
@@ -1369,7 +1467,7 @@
         <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="D8" t="b">
         <v>0</v>
@@ -1378,163 +1476,339 @@
         <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="H8" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="I8" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="J8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M8" t="s">
         <v>47</v>
       </c>
       <c r="N8" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9">
-        <v>31695182</v>
+        <v>31932165</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>67</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="D9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="G9" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="H9" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="I9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J9" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="K9" t="s">
-        <v>47</v>
-      </c>
-      <c r="L9" t="s">
-        <v>47</v>
+        <v>17</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="N9" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10">
-        <v>32559405</v>
+        <v>31932165</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="D10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="F10" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="G10" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="H10" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="I10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J10" t="s">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="K10" t="s">
-        <v>47</v>
-      </c>
-      <c r="L10" t="s">
-        <v>47</v>
+        <v>17</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="N10" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11">
-        <v>32839535</v>
+        <v>31932165</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>81</v>
       </c>
       <c r="D11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F11" t="s">
-        <v>47</v>
+        <v>80</v>
       </c>
       <c r="G11" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="H11" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="I11" t="s">
         <v>50</v>
       </c>
       <c r="J11" t="s">
-        <v>15</v>
+        <v>84</v>
       </c>
       <c r="K11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>66</v>
+      </c>
+      <c r="N11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>31932165</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" t="b">
         <v>0</v>
       </c>
-      <c r="M11" t="s">
+      <c r="E12" t="s">
+        <v>85</v>
+      </c>
+      <c r="F12" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
+        <v>70</v>
+      </c>
+      <c r="I12" t="s">
+        <v>50</v>
+      </c>
+      <c r="J12" t="s">
+        <v>84</v>
+      </c>
+      <c r="K12" t="s">
+        <v>17</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>66</v>
+      </c>
+      <c r="N12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>31932165</v>
+      </c>
+      <c r="B13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>85</v>
+      </c>
+      <c r="F13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" t="s">
+        <v>50</v>
+      </c>
+      <c r="J13" t="s">
+        <v>84</v>
+      </c>
+      <c r="K13" t="s">
+        <v>17</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>66</v>
+      </c>
+      <c r="N13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>32559405</v>
+      </c>
+      <c r="B16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" t="s">
+        <v>47</v>
+      </c>
+      <c r="G16" t="s">
+        <v>47</v>
+      </c>
+      <c r="H16" t="s">
+        <v>47</v>
+      </c>
+      <c r="I16" t="s">
+        <v>47</v>
+      </c>
+      <c r="J16" t="s">
+        <v>47</v>
+      </c>
+      <c r="K16" t="s">
+        <v>47</v>
+      </c>
+      <c r="L16" t="s">
+        <v>47</v>
+      </c>
+      <c r="M16" t="s">
+        <v>47</v>
+      </c>
+      <c r="N16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>32839535</v>
+      </c>
+      <c r="B17" t="s">
         <v>51</v>
       </c>
-      <c r="N11" t="s">
-        <v>54</v>
+      <c r="C17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17" t="s">
+        <v>47</v>
+      </c>
+      <c r="H17" t="s">
+        <v>47</v>
+      </c>
+      <c r="I17" t="s">
+        <v>50</v>
+      </c>
+      <c r="J17" t="s">
+        <v>15</v>
+      </c>
+      <c r="K17" t="s">
+        <v>15</v>
+      </c>
+      <c r="L17" t="b">
+        <v>0</v>
+      </c>
+      <c r="M17" t="s">
+        <v>66</v>
+      </c>
+      <c r="N17" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added human homologue annotations to schema. Updated all previous extractions accordingly.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368A00CE-CBE0-4545-A027-64F42D07F7B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03065E6E-1611-4EB2-89D0-0D23B92A1A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="97">
   <si>
     <t>PMID</t>
   </si>
@@ -260,9 +260,6 @@
     <t>protein full name: Cyclic GMP-AMP synthase</t>
   </si>
   <si>
-    <t>protein full name: Cyclic UMP-AMP synthase; homologue to dncV; crystal structure conducted on homologue in Rhodothermus marinus</t>
-  </si>
-  <si>
     <t>P0DTF6</t>
   </si>
   <si>
@@ -285,6 +282,36 @@
   </si>
   <si>
     <t>AKA Trip13, Pch2; authors specify only organism genus</t>
+  </si>
+  <si>
+    <t>Similiarity_to_hs_note</t>
+  </si>
+  <si>
+    <t>No human similarity</t>
+  </si>
+  <si>
+    <t>overlaid Rhizobiales Pch2 with H. sapiens Trip13</t>
+  </si>
+  <si>
+    <t>Human_homologue</t>
+  </si>
+  <si>
+    <t>Q8N884</t>
+  </si>
+  <si>
+    <t>Sequence similarity and functional similarity; see Extended Data Fig. 3</t>
+  </si>
+  <si>
+    <t>protein full name: Cyclic UMP-AMP synthase; crystal structure conducted on homologue in Rhodothermus marinus</t>
+  </si>
+  <si>
+    <t>Rhodothermus marinus</t>
+  </si>
+  <si>
+    <t>G2SLH8</t>
+  </si>
+  <si>
+    <t>abortive infection; intracellular pathogen sensing; second messenger synthesis; cUMP-cAMP synthesis</t>
   </si>
 </sst>
 </file>
@@ -1145,13 +1172,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="8" max="9" width="17.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1192,10 +1219,16 @@
         <v>11</v>
       </c>
       <c r="N1" t="s">
+        <v>90</v>
+      </c>
+      <c r="O1" t="s">
+        <v>87</v>
+      </c>
+      <c r="P1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>12110595</v>
       </c>
@@ -1236,10 +1269,16 @@
         <v>48</v>
       </c>
       <c r="N2" t="s">
+        <v>47</v>
+      </c>
+      <c r="O2" t="s">
+        <v>47</v>
+      </c>
+      <c r="P2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>30787435</v>
       </c>
@@ -1280,10 +1319,16 @@
         <v>76</v>
       </c>
       <c r="N3" t="s">
+        <v>91</v>
+      </c>
+      <c r="O3" t="s">
+        <v>92</v>
+      </c>
+      <c r="P3" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>30787435</v>
       </c>
@@ -1324,54 +1369,66 @@
         <v>75</v>
       </c>
       <c r="N4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+      <c r="O4" t="s">
+        <v>92</v>
+      </c>
+      <c r="P4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>31695182</v>
+        <v>30787435</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="D5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="F5" t="s">
-        <v>16</v>
+        <v>95</v>
       </c>
       <c r="G5" t="s">
         <v>15</v>
       </c>
       <c r="H5" t="s">
-        <v>17</v>
+        <v>94</v>
       </c>
       <c r="I5" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="J5" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="K5" t="s">
-        <v>46</v>
-      </c>
-      <c r="L5" t="s">
-        <v>46</v>
+        <v>15</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
       <c r="N5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+      <c r="O5" t="s">
+        <v>92</v>
+      </c>
+      <c r="P5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>31695182</v>
       </c>
@@ -1379,7 +1436,7 @@
         <v>41</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -1388,7 +1445,7 @@
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
         <v>15</v>
@@ -1414,8 +1471,14 @@
       <c r="N6" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O6" t="s">
+        <v>47</v>
+      </c>
+      <c r="P6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>31695182</v>
       </c>
@@ -1423,7 +1486,7 @@
         <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -1432,13 +1495,13 @@
         <v>14</v>
       </c>
       <c r="F7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G7" t="s">
         <v>15</v>
       </c>
       <c r="H7" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I7" t="s">
         <v>18</v>
@@ -1456,10 +1519,16 @@
         <v>47</v>
       </c>
       <c r="N7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+      <c r="O7" t="s">
+        <v>47</v>
+      </c>
+      <c r="P7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>31695182</v>
       </c>
@@ -1467,7 +1536,7 @@
         <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="D8" t="b">
         <v>0</v>
@@ -1476,25 +1545,25 @@
         <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="H8" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="I8" t="s">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="J8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M8" t="s">
         <v>47</v>
@@ -1502,52 +1571,64 @@
       <c r="N8" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O8" t="s">
+        <v>47</v>
+      </c>
+      <c r="P8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9">
-        <v>31932165</v>
+        <v>31695182</v>
       </c>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="D9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="F9" t="s">
-        <v>69</v>
+        <v>47</v>
       </c>
       <c r="G9" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="H9" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="I9" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J9" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="K9" t="s">
-        <v>17</v>
-      </c>
-      <c r="L9" t="b">
-        <v>1</v>
+        <v>47</v>
+      </c>
+      <c r="L9" t="s">
+        <v>47</v>
       </c>
       <c r="M9" t="s">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="N9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+      <c r="O9" t="s">
+        <v>47</v>
+      </c>
+      <c r="P9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>31932165</v>
       </c>
@@ -1555,28 +1636,28 @@
         <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="s">
-        <v>58</v>
+        <v>88</v>
       </c>
       <c r="F10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G10" t="s">
         <v>15</v>
       </c>
       <c r="H10" t="s">
-        <v>70</v>
+        <v>17</v>
       </c>
       <c r="I10" t="s">
         <v>50</v>
       </c>
       <c r="J10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K10" t="s">
         <v>17</v>
@@ -1590,8 +1671,14 @@
       <c r="N10" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O10" t="s">
+        <v>15</v>
+      </c>
+      <c r="P10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>31932165</v>
       </c>
@@ -1599,16 +1686,16 @@
         <v>67</v>
       </c>
       <c r="C11" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="D11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>58</v>
+        <v>88</v>
       </c>
       <c r="F11" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="G11" t="s">
         <v>15</v>
@@ -1620,7 +1707,7 @@
         <v>50</v>
       </c>
       <c r="J11" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="K11" t="s">
         <v>17</v>
@@ -1629,13 +1716,19 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="N11" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="O11" t="s">
+        <v>15</v>
+      </c>
+      <c r="P11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>31932165</v>
       </c>
@@ -1643,16 +1736,16 @@
         <v>67</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>80</v>
       </c>
       <c r="D12" t="b">
         <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F12" t="s">
-        <v>15</v>
+        <v>79</v>
       </c>
       <c r="G12" t="s">
         <v>15</v>
@@ -1664,7 +1757,7 @@
         <v>50</v>
       </c>
       <c r="J12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K12" t="s">
         <v>17</v>
@@ -1676,10 +1769,16 @@
         <v>66</v>
       </c>
       <c r="N12" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="O12" t="s">
+        <v>15</v>
+      </c>
+      <c r="P12" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>31932165</v>
       </c>
@@ -1693,7 +1792,7 @@
         <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
         <v>15</v>
@@ -1702,13 +1801,13 @@
         <v>15</v>
       </c>
       <c r="H13" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="I13" t="s">
         <v>50</v>
       </c>
       <c r="J13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K13" t="s">
         <v>17</v>
@@ -1720,15 +1819,121 @@
         <v>66</v>
       </c>
       <c r="N13" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+      <c r="O13" t="s">
+        <v>47</v>
+      </c>
+      <c r="P13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>31932165</v>
+      </c>
+      <c r="B14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s">
+        <v>85</v>
+      </c>
+      <c r="I14" t="s">
+        <v>50</v>
+      </c>
+      <c r="J14" t="s">
+        <v>83</v>
+      </c>
+      <c r="K14" t="s">
+        <v>17</v>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="M14" t="s">
+        <v>66</v>
+      </c>
+      <c r="N14" t="s">
+        <v>15</v>
+      </c>
+      <c r="O14" t="s">
+        <v>89</v>
+      </c>
+      <c r="P14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>32559405</v>
+      </c>
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>47</v>
+      </c>
+      <c r="G15" t="s">
+        <v>47</v>
+      </c>
+      <c r="H15" t="s">
+        <v>47</v>
+      </c>
+      <c r="I15" t="s">
+        <v>47</v>
+      </c>
+      <c r="J15" t="s">
+        <v>47</v>
+      </c>
+      <c r="K15" t="s">
+        <v>47</v>
+      </c>
+      <c r="L15" t="s">
+        <v>47</v>
+      </c>
+      <c r="M15" t="s">
+        <v>47</v>
+      </c>
+      <c r="N15" t="s">
+        <v>47</v>
+      </c>
+      <c r="O15" t="s">
+        <v>47</v>
+      </c>
+      <c r="P15" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16">
-        <v>32559405</v>
+        <v>32839535</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C16" t="s">
         <v>47</v>
@@ -1737,7 +1942,7 @@
         <v>0</v>
       </c>
       <c r="E16" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="F16" t="s">
         <v>47</v>
@@ -1749,65 +1954,27 @@
         <v>47</v>
       </c>
       <c r="I16" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="K16" t="s">
-        <v>47</v>
-      </c>
-      <c r="L16" t="s">
-        <v>47</v>
+        <v>15</v>
+      </c>
+      <c r="L16" t="b">
+        <v>0</v>
       </c>
       <c r="M16" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="N16" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A17">
-        <v>32839535</v>
-      </c>
-      <c r="B17" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" t="b">
-        <v>0</v>
-      </c>
-      <c r="E17" t="s">
-        <v>52</v>
-      </c>
-      <c r="F17" t="s">
-        <v>47</v>
-      </c>
-      <c r="G17" t="s">
-        <v>47</v>
-      </c>
-      <c r="H17" t="s">
-        <v>47</v>
-      </c>
-      <c r="I17" t="s">
-        <v>50</v>
-      </c>
-      <c r="J17" t="s">
-        <v>15</v>
-      </c>
-      <c r="K17" t="s">
-        <v>15</v>
-      </c>
-      <c r="L17" t="b">
-        <v>0</v>
-      </c>
-      <c r="M17" t="s">
-        <v>66</v>
-      </c>
-      <c r="N17" t="s">
+      <c r="O16" t="s">
+        <v>47</v>
+      </c>
+      <c r="P16" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Conducted extractions for 39208803 as screened by M Uchmanowicz. No annotations that pass gold standard.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03065E6E-1611-4EB2-89D0-0D23B92A1A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C7407DC-7C76-4C77-910D-149025914962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -16,12 +16,25 @@
     <sheet name="gold_standard_manual" sheetId="1" r:id="rId1"/>
     <sheet name="notes" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="123">
   <si>
     <t>PMID</t>
   </si>
@@ -140,12 +153,6 @@
     <t>Paper_title</t>
   </si>
   <si>
-    <t>Uniprot_accession</t>
-  </si>
-  <si>
-    <t>Uniparc_accession</t>
-  </si>
-  <si>
     <t>The pan-immune system of bacteria: antiviral defence as a community resource</t>
   </si>
   <si>
@@ -197,9 +204,6 @@
     <t>Vibrio cholerae</t>
   </si>
   <si>
-    <t>Meets gold standard</t>
-  </si>
-  <si>
     <t>34% sequence-similar to yeast tRNA deaminase subunit Tad2p</t>
   </si>
   <si>
@@ -293,15 +297,9 @@
     <t>overlaid Rhizobiales Pch2 with H. sapiens Trip13</t>
   </si>
   <si>
-    <t>Human_homologue</t>
-  </si>
-  <si>
     <t>Q8N884</t>
   </si>
   <si>
-    <t>Sequence similarity and functional similarity; see Extended Data Fig. 3</t>
-  </si>
-  <si>
     <t>protein full name: Cyclic UMP-AMP synthase; crystal structure conducted on homologue in Rhodothermus marinus</t>
   </si>
   <si>
@@ -312,6 +310,99 @@
   </si>
   <si>
     <t>abortive infection; intracellular pathogen sensing; second messenger synthesis; cUMP-cAMP synthesis</t>
+  </si>
+  <si>
+    <t>Bacterial_gene_name</t>
+  </si>
+  <si>
+    <t>Bacterial_UniProt_accession</t>
+  </si>
+  <si>
+    <t>Q99895</t>
+  </si>
+  <si>
+    <t>lmuA</t>
+  </si>
+  <si>
+    <t>Conservation of antiviral systems across domains of life reveals immune genes in humans</t>
+  </si>
+  <si>
+    <t>Human_UniProt_accession</t>
+  </si>
+  <si>
+    <t>Human_gene_name</t>
+  </si>
+  <si>
+    <t>CGAS</t>
+  </si>
+  <si>
+    <t>CTRC</t>
+  </si>
+  <si>
+    <t>TM-score = 0.69 from structural comparison with alphafold structures</t>
+  </si>
+  <si>
+    <t>MOV10L1</t>
+  </si>
+  <si>
+    <t>PLD6</t>
+  </si>
+  <si>
+    <t>Mokosh</t>
+  </si>
+  <si>
+    <t>FHAD</t>
+  </si>
+  <si>
+    <t>In-silico analysis paper proving  bacterial-to-human homology only</t>
+  </si>
+  <si>
+    <t>mkoA</t>
+  </si>
+  <si>
+    <t>mkoB</t>
+  </si>
+  <si>
+    <t>Lamassu</t>
+  </si>
+  <si>
+    <t>lmuB</t>
+  </si>
+  <si>
+    <t>In-silico analysis paper proving  bacterial-to-human homology only; lmuA protein accession EEV5712270.1 as given by authors has no record outside of this paper</t>
+  </si>
+  <si>
+    <t>A0A556BFV1</t>
+  </si>
+  <si>
+    <t>GIMAP6</t>
+  </si>
+  <si>
+    <t>Bacillus sp. HY001</t>
+  </si>
+  <si>
+    <t>FOT98_29090</t>
+  </si>
+  <si>
+    <t>B4DH95</t>
+  </si>
+  <si>
+    <t>TM-score 0.4 from alphafold structures</t>
+  </si>
+  <si>
+    <t>Eleos</t>
+  </si>
+  <si>
+    <t>In-silico analysis paper proving  bacterial-to-human homology only; bacterial gene AKA LeoBC; I cannot find a paper proving this specific protein's antiphage activity with functional assays</t>
+  </si>
+  <si>
+    <t>Unquantified loose sequence similarity and functional similarity; see Extended Data Fig. 3</t>
+  </si>
+  <si>
+    <t>In-silico analysis only</t>
+  </si>
+  <si>
+    <t>Functional assay, homology to human protein; homology is unquantified and domain-specific</t>
   </si>
 </sst>
 </file>
@@ -1172,10 +1263,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="8" max="9" width="17.36328125" customWidth="1"/>
+    <col min="10" max="11" width="17.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">
@@ -1186,43 +1277,43 @@
         <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="I1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>10</v>
-      </c>
-      <c r="M1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" t="s">
-        <v>90</v>
-      </c>
-      <c r="O1" t="s">
-        <v>87</v>
       </c>
       <c r="P1" t="s">
         <v>12</v>
@@ -1233,49 +1324,49 @@
         <v>12110595</v>
       </c>
       <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
         <v>42</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
         <v>43</v>
       </c>
-      <c r="D2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F2" t="s">
-        <v>44</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>46</v>
-      </c>
       <c r="K2" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="L2" t="s">
         <v>46</v>
       </c>
       <c r="M2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="N2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="O2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="P2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
@@ -1283,49 +1374,49 @@
         <v>30787435</v>
       </c>
       <c r="B3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" t="s">
         <v>54</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" t="s">
+        <v>120</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
+        <v>122</v>
+      </c>
+      <c r="J3" t="s">
         <v>55</v>
       </c>
-      <c r="D3" t="b">
+      <c r="K3" t="s">
+        <v>48</v>
+      </c>
+      <c r="L3" t="s">
+        <v>73</v>
+      </c>
+      <c r="M3" t="s">
+        <v>61</v>
+      </c>
+      <c r="N3" t="s">
+        <v>62</v>
+      </c>
+      <c r="O3" t="b">
         <v>1</v>
       </c>
-      <c r="E3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>57</v>
-      </c>
-      <c r="I3" t="s">
-        <v>50</v>
-      </c>
-      <c r="J3" t="s">
-        <v>64</v>
-      </c>
-      <c r="K3" t="s">
-        <v>65</v>
-      </c>
-      <c r="L3" t="b">
-        <v>1</v>
-      </c>
-      <c r="M3" t="s">
-        <v>76</v>
-      </c>
-      <c r="N3" t="s">
-        <v>91</v>
-      </c>
-      <c r="O3" t="s">
-        <v>92</v>
-      </c>
       <c r="P3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
@@ -1333,49 +1424,49 @@
         <v>30787435</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D4" t="b">
+        <v>58</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" t="s">
+        <v>120</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
+        <v>122</v>
+      </c>
+      <c r="J4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" t="s">
+        <v>72</v>
+      </c>
+      <c r="M4" t="s">
+        <v>60</v>
+      </c>
+      <c r="N4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O4" t="b">
         <v>1</v>
       </c>
-      <c r="E4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J4" t="s">
-        <v>63</v>
-      </c>
-      <c r="K4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M4" t="s">
-        <v>75</v>
-      </c>
-      <c r="N4" t="s">
-        <v>91</v>
-      </c>
-      <c r="O4" t="s">
-        <v>92</v>
-      </c>
       <c r="P4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.35">
@@ -1383,46 +1474,46 @@
         <v>30787435</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F5" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>122</v>
+      </c>
+      <c r="J5" t="s">
+        <v>89</v>
+      </c>
+      <c r="K5" t="s">
+        <v>48</v>
+      </c>
+      <c r="L5" t="s">
+        <v>91</v>
+      </c>
+      <c r="M5" t="s">
         <v>61</v>
       </c>
-      <c r="D5" t="b">
+      <c r="N5" t="s">
+        <v>15</v>
+      </c>
+      <c r="O5" t="b">
         <v>1</v>
-      </c>
-      <c r="E5" t="s">
-        <v>58</v>
-      </c>
-      <c r="F5" t="s">
-        <v>95</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s">
-        <v>94</v>
-      </c>
-      <c r="I5" t="s">
-        <v>50</v>
-      </c>
-      <c r="J5" t="s">
-        <v>64</v>
-      </c>
-      <c r="K5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L5" t="b">
-        <v>1</v>
-      </c>
-      <c r="M5" t="s">
-        <v>96</v>
-      </c>
-      <c r="N5" t="s">
-        <v>91</v>
-      </c>
-      <c r="O5" t="s">
-        <v>92</v>
       </c>
       <c r="P5" t="s">
         <v>15</v>
@@ -1433,49 +1524,49 @@
         <v>31695182</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" t="b">
-        <v>0</v>
+      <c r="D6" t="s">
+        <v>16</v>
       </c>
       <c r="E6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" t="s">
+        <v>45</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="s">
         <v>14</v>
       </c>
-      <c r="F6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>17</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>18</v>
       </c>
-      <c r="J6" t="s">
-        <v>46</v>
-      </c>
-      <c r="K6" t="s">
-        <v>46</v>
-      </c>
       <c r="L6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="N6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="O6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="P6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.35">
@@ -1483,49 +1574,49 @@
         <v>31695182</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
         <v>19</v>
       </c>
-      <c r="D7" t="b">
-        <v>0</v>
+      <c r="D7" t="s">
+        <v>20</v>
       </c>
       <c r="E7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="s">
         <v>14</v>
       </c>
-      <c r="F7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="J7" t="s">
         <v>17</v>
       </c>
-      <c r="I7" t="s">
+      <c r="K7" t="s">
         <v>18</v>
       </c>
-      <c r="J7" t="s">
-        <v>46</v>
-      </c>
-      <c r="K7" t="s">
-        <v>46</v>
-      </c>
       <c r="L7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="N7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="O7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="P7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">
@@ -1533,49 +1624,49 @@
         <v>31695182</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
       </c>
-      <c r="D8" t="b">
-        <v>0</v>
+      <c r="D8" t="s">
+        <v>22</v>
       </c>
       <c r="E8" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="s">
         <v>14</v>
       </c>
-      <c r="F8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="J8" t="s">
         <v>23</v>
       </c>
-      <c r="I8" t="s">
+      <c r="K8" t="s">
         <v>18</v>
       </c>
-      <c r="J8" t="s">
-        <v>46</v>
-      </c>
-      <c r="K8" t="s">
-        <v>46</v>
-      </c>
       <c r="L8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="N8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="O8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="P8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
@@ -1583,49 +1674,49 @@
         <v>31695182</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" t="b">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="D9" t="s">
+        <v>45</v>
       </c>
       <c r="E9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" t="s">
+        <v>45</v>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="s">
         <v>14</v>
       </c>
-      <c r="F9" t="s">
-        <v>47</v>
-      </c>
-      <c r="G9" t="s">
-        <v>47</v>
-      </c>
-      <c r="H9" t="s">
-        <v>47</v>
-      </c>
-      <c r="I9" t="s">
-        <v>47</v>
-      </c>
       <c r="J9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="L9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="M9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="N9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="O9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
@@ -1633,46 +1724,46 @@
         <v>31932165</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D10" t="b">
-        <v>0</v>
+        <v>65</v>
+      </c>
+      <c r="D10" t="s">
+        <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>88</v>
+        <v>15</v>
       </c>
       <c r="F10" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="G10" t="s">
         <v>15</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="s">
+        <v>85</v>
+      </c>
+      <c r="J10" t="s">
         <v>17</v>
       </c>
-      <c r="I10" t="s">
-        <v>50</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
+        <v>48</v>
+      </c>
+      <c r="L10" t="s">
         <v>74</v>
       </c>
-      <c r="K10" t="s">
+      <c r="M10" t="s">
+        <v>71</v>
+      </c>
+      <c r="N10" t="s">
         <v>17</v>
       </c>
-      <c r="L10" t="b">
+      <c r="O10" t="b">
         <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>77</v>
-      </c>
-      <c r="N10" t="s">
-        <v>15</v>
-      </c>
-      <c r="O10" t="s">
-        <v>15</v>
       </c>
       <c r="P10" t="s">
         <v>15</v>
@@ -1683,46 +1774,46 @@
         <v>31932165</v>
       </c>
       <c r="B11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" t="s">
+        <v>68</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="s">
+        <v>85</v>
+      </c>
+      <c r="J11" t="s">
         <v>67</v>
       </c>
-      <c r="C11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" t="b">
-        <v>0</v>
-      </c>
-      <c r="E11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F11" t="s">
-        <v>71</v>
-      </c>
-      <c r="G11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="K11" t="s">
+        <v>48</v>
+      </c>
+      <c r="L11" t="s">
+        <v>74</v>
+      </c>
+      <c r="M11" t="s">
         <v>70</v>
       </c>
-      <c r="I11" t="s">
-        <v>50</v>
-      </c>
-      <c r="J11" t="s">
-        <v>73</v>
-      </c>
-      <c r="K11" t="s">
+      <c r="N11" t="s">
         <v>17</v>
       </c>
-      <c r="L11" t="b">
+      <c r="O11" t="b">
         <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>77</v>
-      </c>
-      <c r="N11" t="s">
-        <v>15</v>
-      </c>
-      <c r="O11" t="s">
-        <v>15</v>
       </c>
       <c r="P11" t="s">
         <v>15</v>
@@ -1733,49 +1824,49 @@
         <v>31932165</v>
       </c>
       <c r="B12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="s">
+        <v>85</v>
+      </c>
+      <c r="J12" t="s">
         <v>67</v>
       </c>
-      <c r="C12" t="s">
+      <c r="K12" t="s">
+        <v>48</v>
+      </c>
+      <c r="L12" t="s">
+        <v>63</v>
+      </c>
+      <c r="M12" t="s">
         <v>80</v>
       </c>
-      <c r="D12" t="b">
-        <v>0</v>
-      </c>
-      <c r="E12" t="s">
-        <v>88</v>
-      </c>
-      <c r="F12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s">
-        <v>70</v>
-      </c>
-      <c r="I12" t="s">
-        <v>50</v>
-      </c>
-      <c r="J12" t="s">
-        <v>83</v>
-      </c>
-      <c r="K12" t="s">
+      <c r="N12" t="s">
         <v>17</v>
       </c>
-      <c r="L12" t="b">
+      <c r="O12" t="b">
         <v>1</v>
       </c>
-      <c r="M12" t="s">
-        <v>66</v>
-      </c>
-      <c r="N12" t="s">
-        <v>15</v>
-      </c>
-      <c r="O12" t="s">
-        <v>15</v>
-      </c>
       <c r="P12" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
@@ -1783,49 +1874,49 @@
         <v>31932165</v>
       </c>
       <c r="B13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G13" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" t="s">
+        <v>81</v>
+      </c>
+      <c r="J13" t="s">
         <v>67</v>
       </c>
-      <c r="C13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" t="b">
-        <v>0</v>
-      </c>
-      <c r="E13" t="s">
-        <v>84</v>
-      </c>
-      <c r="F13" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" t="s">
-        <v>70</v>
-      </c>
-      <c r="I13" t="s">
-        <v>50</v>
-      </c>
-      <c r="J13" t="s">
-        <v>83</v>
-      </c>
       <c r="K13" t="s">
+        <v>48</v>
+      </c>
+      <c r="L13" t="s">
+        <v>63</v>
+      </c>
+      <c r="M13" t="s">
+        <v>80</v>
+      </c>
+      <c r="N13" t="s">
         <v>17</v>
       </c>
-      <c r="L13" t="b">
+      <c r="O13" t="b">
         <v>1</v>
       </c>
-      <c r="M13" t="s">
-        <v>66</v>
-      </c>
-      <c r="N13" t="s">
-        <v>47</v>
-      </c>
-      <c r="O13" t="s">
-        <v>47</v>
-      </c>
       <c r="P13" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
@@ -1833,49 +1924,49 @@
         <v>31932165</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C14" t="s">
         <v>15</v>
       </c>
-      <c r="D14" t="b">
-        <v>0</v>
+      <c r="D14" t="s">
+        <v>15</v>
       </c>
       <c r="E14" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
       </c>
       <c r="G14" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" t="s">
-        <v>85</v>
+        <v>86</v>
+      </c>
+      <c r="H14" t="b">
+        <v>0</v>
       </c>
       <c r="I14" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="J14" t="s">
+        <v>82</v>
+      </c>
+      <c r="K14" t="s">
+        <v>48</v>
+      </c>
+      <c r="L14" t="s">
+        <v>63</v>
+      </c>
+      <c r="M14" t="s">
+        <v>80</v>
+      </c>
+      <c r="N14" t="s">
+        <v>17</v>
+      </c>
+      <c r="O14" t="b">
+        <v>1</v>
+      </c>
+      <c r="P14" t="s">
         <v>83</v>
-      </c>
-      <c r="K14" t="s">
-        <v>17</v>
-      </c>
-      <c r="L14" t="b">
-        <v>1</v>
-      </c>
-      <c r="M14" t="s">
-        <v>66</v>
-      </c>
-      <c r="N14" t="s">
-        <v>15</v>
-      </c>
-      <c r="O14" t="s">
-        <v>89</v>
-      </c>
-      <c r="P14" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
@@ -1883,49 +1974,49 @@
         <v>32559405</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" t="b">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="D15" t="s">
+        <v>45</v>
       </c>
       <c r="E15" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" t="s">
+        <v>45</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" t="s">
         <v>14</v>
       </c>
-      <c r="F15" t="s">
-        <v>47</v>
-      </c>
-      <c r="G15" t="s">
-        <v>47</v>
-      </c>
-      <c r="H15" t="s">
-        <v>47</v>
-      </c>
-      <c r="I15" t="s">
-        <v>47</v>
-      </c>
       <c r="J15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="L15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="M15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="N15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="O15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
@@ -1933,49 +2024,287 @@
         <v>32839535</v>
       </c>
       <c r="B16" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
-      </c>
-      <c r="D16" t="b">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="D16" t="s">
+        <v>45</v>
       </c>
       <c r="E16" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="F16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G16" t="s">
-        <v>47</v>
-      </c>
-      <c r="H16" t="s">
-        <v>47</v>
+        <v>45</v>
+      </c>
+      <c r="H16" t="b">
+        <v>0</v>
       </c>
       <c r="I16" t="s">
         <v>50</v>
       </c>
       <c r="J16" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="K16" t="s">
-        <v>15</v>
-      </c>
-      <c r="L16" t="b">
-        <v>0</v>
+        <v>48</v>
+      </c>
+      <c r="L16" t="s">
+        <v>63</v>
       </c>
       <c r="M16" t="s">
-        <v>66</v>
+        <v>15</v>
       </c>
       <c r="N16" t="s">
-        <v>47</v>
-      </c>
-      <c r="O16" t="s">
-        <v>47</v>
+        <v>15</v>
+      </c>
+      <c r="O16" t="b">
+        <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>53</v>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>39208803</v>
+      </c>
+      <c r="B17" t="s">
+        <v>96</v>
+      </c>
+      <c r="C17" t="s">
+        <v>115</v>
+      </c>
+      <c r="D17" t="s">
+        <v>112</v>
+      </c>
+      <c r="E17" t="s">
+        <v>113</v>
+      </c>
+      <c r="F17" t="s">
+        <v>116</v>
+      </c>
+      <c r="G17" t="s">
+        <v>117</v>
+      </c>
+      <c r="H17" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" t="s">
+        <v>50</v>
+      </c>
+      <c r="J17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K17" t="s">
+        <v>118</v>
+      </c>
+      <c r="L17" t="s">
+        <v>15</v>
+      </c>
+      <c r="M17" t="s">
+        <v>15</v>
+      </c>
+      <c r="N17" t="s">
+        <v>15</v>
+      </c>
+      <c r="O17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P17" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>39208803</v>
+      </c>
+      <c r="B18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C18" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" t="s">
+        <v>105</v>
+      </c>
+      <c r="F18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="s">
+        <v>121</v>
+      </c>
+      <c r="K18" t="s">
+        <v>109</v>
+      </c>
+      <c r="L18" t="s">
+        <v>15</v>
+      </c>
+      <c r="M18" t="s">
+        <v>15</v>
+      </c>
+      <c r="N18" t="s">
+        <v>15</v>
+      </c>
+      <c r="O18" t="s">
+        <v>15</v>
+      </c>
+      <c r="P18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>39208803</v>
+      </c>
+      <c r="B19" t="s">
+        <v>96</v>
+      </c>
+      <c r="C19" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" t="s">
+        <v>100</v>
+      </c>
+      <c r="F19" t="s">
+        <v>94</v>
+      </c>
+      <c r="G19" t="s">
+        <v>101</v>
+      </c>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" t="s">
+        <v>81</v>
+      </c>
+      <c r="J19" t="s">
+        <v>17</v>
+      </c>
+      <c r="K19" t="s">
+        <v>109</v>
+      </c>
+      <c r="L19" t="s">
+        <v>15</v>
+      </c>
+      <c r="M19" t="s">
+        <v>15</v>
+      </c>
+      <c r="N19" t="s">
+        <v>15</v>
+      </c>
+      <c r="O19" t="s">
+        <v>15</v>
+      </c>
+      <c r="P19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>39208803</v>
+      </c>
+      <c r="B20" t="s">
+        <v>96</v>
+      </c>
+      <c r="C20" t="s">
+        <v>107</v>
+      </c>
+      <c r="D20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" t="s">
+        <v>102</v>
+      </c>
+      <c r="F20" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20" t="s">
+        <v>121</v>
+      </c>
+      <c r="K20" t="s">
+        <v>104</v>
+      </c>
+      <c r="L20" t="s">
+        <v>15</v>
+      </c>
+      <c r="M20" t="s">
+        <v>15</v>
+      </c>
+      <c r="N20" t="s">
+        <v>15</v>
+      </c>
+      <c r="O20" t="s">
+        <v>15</v>
+      </c>
+      <c r="P20" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>39208803</v>
+      </c>
+      <c r="B21" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" t="s">
+        <v>103</v>
+      </c>
+      <c r="F21" t="s">
+        <v>45</v>
+      </c>
+      <c r="G21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" t="s">
+        <v>121</v>
+      </c>
+      <c r="K21" t="s">
+        <v>104</v>
+      </c>
+      <c r="L21" t="s">
+        <v>15</v>
+      </c>
+      <c r="M21" t="s">
+        <v>15</v>
+      </c>
+      <c r="N21" t="s">
+        <v>15</v>
+      </c>
+      <c r="O21" t="s">
+        <v>15</v>
+      </c>
+      <c r="P21" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Performed extraction for PMID 40705877; J8G6Z1 to Q9BPY3 protein pair
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C7407DC-7C76-4C77-910D-149025914962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBCAB234-D081-4376-B350-F1AF57829A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="153">
   <si>
     <t>PMID</t>
   </si>
@@ -403,6 +403,96 @@
   </si>
   <si>
     <t>Functional assay, homology to human protein; homology is unquantified and domain-specific</t>
+  </si>
+  <si>
+    <t>A Bacterial Dynamin-Like Protein Confers a Novel Phage Resistance Strategy on the Population Level in Bacillus subtilis</t>
+  </si>
+  <si>
+    <t>dynA</t>
+  </si>
+  <si>
+    <t>P54159</t>
+  </si>
+  <si>
+    <t>Bacillus subtilis</t>
+  </si>
+  <si>
+    <t>Screening_source</t>
+  </si>
+  <si>
+    <t>C Trost</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>M Umanowicz</t>
+  </si>
+  <si>
+    <t>A human homolog of SIR2 antiphage proteins mediates immunity via the Toll- like receptor pathway</t>
+  </si>
+  <si>
+    <t>FAM118B</t>
+  </si>
+  <si>
+    <t>Human homology</t>
+  </si>
+  <si>
+    <t>Q9BPY3</t>
+  </si>
+  <si>
+    <t>"We first identified bacterial SIR2 proteins involved in documented antiphage systems with the program DefenseFinder";</t>
+  </si>
+  <si>
+    <t>Dsr 2</t>
+  </si>
+  <si>
+    <t>Citrobacter sp.</t>
+  </si>
+  <si>
+    <t>Treponema sp.</t>
+  </si>
+  <si>
+    <t>Bacillus cereus</t>
+  </si>
+  <si>
+    <t>Belliella baltica</t>
+  </si>
+  <si>
+    <t>Klebsiella pneumoniae</t>
+  </si>
+  <si>
+    <t>PD-T7-2 A</t>
+  </si>
+  <si>
+    <t>pAGO SIR2-APAZ</t>
+  </si>
+  <si>
+    <t>AbiH</t>
+  </si>
+  <si>
+    <t>ThsA</t>
+  </si>
+  <si>
+    <t>J8G6Z1</t>
+  </si>
+  <si>
+    <t>antiphage; NAD+ hydrolysis; NAD+ binding</t>
+  </si>
+  <si>
+    <t>SIR2 antiphage; Thoeris</t>
+  </si>
+  <si>
+    <t>AKA "Thoeris A" by authors; "We first identified bacterial SIR2 proteins involved in documented antiphage systems with the program DefenseFinder"; antiphage system words by NAD+ hyrolysis and binding; unclear whether working with predicted or experimental structures in this paper</t>
+  </si>
+  <si>
+    <t>Structural and functional evidence of bacterial antiphage protection by Thoeris defense system via NAD+ degradation</t>
+  </si>
+  <si>
+    <t>analytical size-exclusion chromatography; mutation analysis</t>
+  </si>
+  <si>
+    <t>"Fig. 2 Crystal structure of ThsA"; "The selenomethionyl proteins were expressed in E. coli BL21"; "To further study structural aspect of NAD+ cleavage by ThsA, we tried to crystallize NAD+-bound complexes of both wild-type and mutant ThsA proteins, but our attempts were not successful."</t>
   </si>
 </sst>
 </file>
@@ -1263,13 +1353,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="3" max="5" width="17.6328125" customWidth="1"/>
+    <col min="6" max="6" width="17.453125" customWidth="1"/>
+    <col min="9" max="9" width="8.7265625" customWidth="1"/>
     <col min="10" max="11" width="17.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1316,10 +1409,13 @@
         <v>10</v>
       </c>
       <c r="P1" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>12110595</v>
       </c>
@@ -1366,10 +1462,13 @@
         <v>44</v>
       </c>
       <c r="P2" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>30787435</v>
       </c>
@@ -1416,10 +1515,13 @@
         <v>1</v>
       </c>
       <c r="P3" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q3" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>30787435</v>
       </c>
@@ -1442,7 +1544,7 @@
         <v>120</v>
       </c>
       <c r="H4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="s">
         <v>122</v>
@@ -1466,10 +1568,13 @@
         <v>1</v>
       </c>
       <c r="P4" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>30787435</v>
       </c>
@@ -1492,7 +1597,7 @@
         <v>120</v>
       </c>
       <c r="H5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="s">
         <v>122</v>
@@ -1516,10 +1621,13 @@
         <v>1</v>
       </c>
       <c r="P5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>31695182</v>
       </c>
@@ -1566,10 +1674,13 @@
         <v>44</v>
       </c>
       <c r="P6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>31695182</v>
       </c>
@@ -1616,10 +1727,13 @@
         <v>44</v>
       </c>
       <c r="P7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>31695182</v>
       </c>
@@ -1666,10 +1780,13 @@
         <v>44</v>
       </c>
       <c r="P8" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>31695182</v>
       </c>
@@ -1716,10 +1833,13 @@
         <v>45</v>
       </c>
       <c r="P9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>31932165</v>
       </c>
@@ -1766,10 +1886,13 @@
         <v>1</v>
       </c>
       <c r="P10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>31932165</v>
       </c>
@@ -1816,10 +1939,13 @@
         <v>1</v>
       </c>
       <c r="P11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>31932165</v>
       </c>
@@ -1866,10 +1992,13 @@
         <v>1</v>
       </c>
       <c r="P12" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q12" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>31932165</v>
       </c>
@@ -1916,10 +2045,13 @@
         <v>1</v>
       </c>
       <c r="P13" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q13" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>31932165</v>
       </c>
@@ -1966,10 +2098,13 @@
         <v>1</v>
       </c>
       <c r="P14" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q14" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>32559405</v>
       </c>
@@ -2016,10 +2151,13 @@
         <v>45</v>
       </c>
       <c r="P15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>32839535</v>
       </c>
@@ -2066,10 +2204,13 @@
         <v>0</v>
       </c>
       <c r="P16" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q16" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>39208803</v>
       </c>
@@ -2116,10 +2257,13 @@
         <v>15</v>
       </c>
       <c r="P17" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q17" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>39208803</v>
       </c>
@@ -2138,12 +2282,18 @@
       <c r="F18" t="s">
         <v>15</v>
       </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
       <c r="H18" t="b">
         <v>0</v>
       </c>
       <c r="I18" t="s">
         <v>121</v>
       </c>
+      <c r="J18" t="s">
+        <v>45</v>
+      </c>
       <c r="K18" t="s">
         <v>109</v>
       </c>
@@ -2160,10 +2310,13 @@
         <v>15</v>
       </c>
       <c r="P18" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q18" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>39208803</v>
       </c>
@@ -2210,10 +2363,13 @@
         <v>15</v>
       </c>
       <c r="P19" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q19" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>39208803</v>
       </c>
@@ -2257,10 +2413,13 @@
         <v>15</v>
       </c>
       <c r="P20" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q20" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>39208803</v>
       </c>
@@ -2304,7 +2463,294 @@
         <v>15</v>
       </c>
       <c r="P21" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q21" t="s">
         <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>35164550</v>
+      </c>
+      <c r="B22" t="s">
+        <v>123</v>
+      </c>
+      <c r="C22" t="s">
+        <v>124</v>
+      </c>
+      <c r="D22" t="s">
+        <v>125</v>
+      </c>
+      <c r="E22" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" t="s">
+        <v>85</v>
+      </c>
+      <c r="J22" t="s">
+        <v>126</v>
+      </c>
+      <c r="K22" t="s">
+        <v>45</v>
+      </c>
+      <c r="L22" t="s">
+        <v>45</v>
+      </c>
+      <c r="M22" t="s">
+        <v>45</v>
+      </c>
+      <c r="N22" t="s">
+        <v>45</v>
+      </c>
+      <c r="O22" t="s">
+        <v>45</v>
+      </c>
+      <c r="P22" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>40705877</v>
+      </c>
+      <c r="B25" t="s">
+        <v>131</v>
+      </c>
+      <c r="C25" t="s">
+        <v>145</v>
+      </c>
+      <c r="D25" t="s">
+        <v>146</v>
+      </c>
+      <c r="E25" t="s">
+        <v>132</v>
+      </c>
+      <c r="F25" t="s">
+        <v>134</v>
+      </c>
+      <c r="H25" t="b">
+        <v>1</v>
+      </c>
+      <c r="I25" t="s">
+        <v>133</v>
+      </c>
+      <c r="J25" t="s">
+        <v>139</v>
+      </c>
+      <c r="K25" t="s">
+        <v>148</v>
+      </c>
+      <c r="L25" t="s">
+        <v>147</v>
+      </c>
+      <c r="M25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N25" t="s">
+        <v>15</v>
+      </c>
+      <c r="O25" t="s">
+        <v>15</v>
+      </c>
+      <c r="P25" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>32499527</v>
+      </c>
+      <c r="B26" t="s">
+        <v>150</v>
+      </c>
+      <c r="C26" t="s">
+        <v>145</v>
+      </c>
+      <c r="D26" t="s">
+        <v>146</v>
+      </c>
+      <c r="E26" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26" t="s">
+        <v>15</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" t="s">
+        <v>15</v>
+      </c>
+      <c r="J26" t="s">
+        <v>15</v>
+      </c>
+      <c r="K26" t="s">
+        <v>15</v>
+      </c>
+      <c r="L26" t="s">
+        <v>15</v>
+      </c>
+      <c r="M26" t="s">
+        <v>151</v>
+      </c>
+      <c r="N26" t="s">
+        <v>17</v>
+      </c>
+      <c r="O26" t="b">
+        <v>1</v>
+      </c>
+      <c r="P26" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>40705877</v>
+      </c>
+      <c r="B29" t="s">
+        <v>131</v>
+      </c>
+      <c r="C29" t="s">
+        <v>136</v>
+      </c>
+      <c r="E29" t="s">
+        <v>132</v>
+      </c>
+      <c r="F29" t="s">
+        <v>134</v>
+      </c>
+      <c r="H29" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" t="s">
+        <v>133</v>
+      </c>
+      <c r="J29" t="s">
+        <v>137</v>
+      </c>
+      <c r="P29" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>40705877</v>
+      </c>
+      <c r="B30" t="s">
+        <v>131</v>
+      </c>
+      <c r="C30" t="s">
+        <v>142</v>
+      </c>
+      <c r="E30" t="s">
+        <v>132</v>
+      </c>
+      <c r="F30" t="s">
+        <v>134</v>
+      </c>
+      <c r="H30" t="b">
+        <v>1</v>
+      </c>
+      <c r="I30" t="s">
+        <v>133</v>
+      </c>
+      <c r="J30" t="s">
+        <v>140</v>
+      </c>
+      <c r="P30" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>40705877</v>
+      </c>
+      <c r="B31" t="s">
+        <v>131</v>
+      </c>
+      <c r="C31" t="s">
+        <v>143</v>
+      </c>
+      <c r="E31" t="s">
+        <v>132</v>
+      </c>
+      <c r="F31" t="s">
+        <v>134</v>
+      </c>
+      <c r="H31" t="b">
+        <v>1</v>
+      </c>
+      <c r="I31" t="s">
+        <v>133</v>
+      </c>
+      <c r="J31" t="s">
+        <v>138</v>
+      </c>
+      <c r="P31" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>40705877</v>
+      </c>
+      <c r="B32" t="s">
+        <v>131</v>
+      </c>
+      <c r="C32" t="s">
+        <v>144</v>
+      </c>
+      <c r="E32" t="s">
+        <v>132</v>
+      </c>
+      <c r="F32" t="s">
+        <v>134</v>
+      </c>
+      <c r="H32" t="b">
+        <v>1</v>
+      </c>
+      <c r="I32" t="s">
+        <v>133</v>
+      </c>
+      <c r="J32" t="s">
+        <v>141</v>
+      </c>
+      <c r="P32" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed first round of extractions for 40705877; look again at SIR1, SIR2, etc. genes; proof of homology is in supplementaries.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBCAB234-D081-4376-B350-F1AF57829A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCF66B5D-7CC2-42C9-8A2D-DF6E2B5F9536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="159">
   <si>
     <t>PMID</t>
   </si>
@@ -441,9 +441,6 @@
     <t>Q9BPY3</t>
   </si>
   <si>
-    <t>"We first identified bacterial SIR2 proteins involved in documented antiphage systems with the program DefenseFinder";</t>
-  </si>
-  <si>
     <t>Dsr 2</t>
   </si>
   <si>
@@ -483,9 +480,6 @@
     <t>SIR2 antiphage; Thoeris</t>
   </si>
   <si>
-    <t>AKA "Thoeris A" by authors; "We first identified bacterial SIR2 proteins involved in documented antiphage systems with the program DefenseFinder"; antiphage system words by NAD+ hyrolysis and binding; unclear whether working with predicted or experimental structures in this paper</t>
-  </si>
-  <si>
     <t>Structural and functional evidence of bacterial antiphage protection by Thoeris defense system via NAD+ degradation</t>
   </si>
   <si>
@@ -493,6 +487,30 @@
   </si>
   <si>
     <t>"Fig. 2 Crystal structure of ThsA"; "The selenomethionyl proteins were expressed in E. coli BL21"; "To further study structural aspect of NAD+ cleavage by ThsA, we tried to crystallize NAD+-bound complexes of both wild-type and mutant ThsA proteins, but our attempts were not successful."</t>
+  </si>
+  <si>
+    <t>ID given by authors: R8X3J8; from UniProt: "Removed from UniProtKB because R8X3J8 is not part of a reference proteome"; from UinProt: "UniParc · UPI00032F70EF · R8X3J8"</t>
+  </si>
+  <si>
+    <t>I3Z638</t>
+  </si>
+  <si>
+    <t>No functional assays</t>
+  </si>
+  <si>
+    <t>AKA "Thoeris A" by authors; antiphage system words by NAD+ hyrolysis and binding; unclear whether working with predicted or experimental structures in this paper</t>
+  </si>
+  <si>
+    <t>No UniProt ID</t>
+  </si>
+  <si>
+    <t>EMBL ID given by authors as "AIW90156"; cannot translate to UniProt (tried the UniProt ID mapping tool)</t>
+  </si>
+  <si>
+    <t>AFDB ID given by authors as "A0A1V0M776" and organism given as "K. pneumoniae", but for A0A1V0M776  in AFDB the organism is Providencia rettgeri (https://alphafold.ebi.ac.uk/entry/AF-A0A1V0M776-F1)</t>
+  </si>
+  <si>
+    <t>Checked supplementaries for functional assays and found none</t>
   </si>
 </sst>
 </file>
@@ -1353,7 +1371,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="5" width="17.6328125" customWidth="1"/>
@@ -2522,6 +2540,112 @@
         <v>15</v>
       </c>
     </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>40705877</v>
+      </c>
+      <c r="B23" t="s">
+        <v>131</v>
+      </c>
+      <c r="C23" t="s">
+        <v>144</v>
+      </c>
+      <c r="D23" t="s">
+        <v>145</v>
+      </c>
+      <c r="E23" t="s">
+        <v>132</v>
+      </c>
+      <c r="F23" t="s">
+        <v>134</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" t="s">
+        <v>133</v>
+      </c>
+      <c r="J23" t="s">
+        <v>138</v>
+      </c>
+      <c r="K23" t="s">
+        <v>147</v>
+      </c>
+      <c r="L23" t="s">
+        <v>146</v>
+      </c>
+      <c r="M23" t="s">
+        <v>15</v>
+      </c>
+      <c r="N23" t="s">
+        <v>15</v>
+      </c>
+      <c r="O23" t="s">
+        <v>15</v>
+      </c>
+      <c r="P23" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>32499527</v>
+      </c>
+      <c r="B24" t="s">
+        <v>148</v>
+      </c>
+      <c r="C24" t="s">
+        <v>144</v>
+      </c>
+      <c r="D24" t="s">
+        <v>145</v>
+      </c>
+      <c r="E24" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="b">
+        <v>1</v>
+      </c>
+      <c r="I24" t="s">
+        <v>15</v>
+      </c>
+      <c r="J24" t="s">
+        <v>15</v>
+      </c>
+      <c r="K24" t="s">
+        <v>15</v>
+      </c>
+      <c r="L24" t="s">
+        <v>15</v>
+      </c>
+      <c r="M24" t="s">
+        <v>149</v>
+      </c>
+      <c r="N24" t="s">
+        <v>17</v>
+      </c>
+      <c r="O24" t="b">
+        <v>1</v>
+      </c>
+      <c r="P24" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>150</v>
+      </c>
+    </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>40705877</v>
@@ -2530,10 +2654,10 @@
         <v>131</v>
       </c>
       <c r="C25" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="D25" t="s">
-        <v>146</v>
+        <v>15</v>
       </c>
       <c r="E25" t="s">
         <v>132</v>
@@ -2541,20 +2665,23 @@
       <c r="F25" t="s">
         <v>134</v>
       </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
       <c r="H25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
       <c r="J25" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="K25" t="s">
-        <v>148</v>
+        <v>15</v>
       </c>
       <c r="L25" t="s">
-        <v>147</v>
+        <v>15</v>
       </c>
       <c r="M25" t="s">
         <v>15</v>
@@ -2569,188 +2696,166 @@
         <v>129</v>
       </c>
       <c r="Q25" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A26">
-        <v>32499527</v>
+        <v>40705877</v>
       </c>
       <c r="B26" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="C26" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D26" t="s">
-        <v>146</v>
+        <v>15</v>
       </c>
       <c r="E26" t="s">
-        <v>15</v>
+        <v>132</v>
       </c>
       <c r="F26" t="s">
-        <v>15</v>
+        <v>134</v>
       </c>
       <c r="G26" t="s">
         <v>15</v>
       </c>
       <c r="H26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I26" t="s">
-        <v>15</v>
+        <v>155</v>
       </c>
       <c r="J26" t="s">
-        <v>15</v>
+        <v>137</v>
       </c>
       <c r="K26" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="L26" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="M26" t="s">
-        <v>151</v>
+        <v>45</v>
       </c>
       <c r="N26" t="s">
-        <v>17</v>
-      </c>
-      <c r="O26" t="b">
-        <v>1</v>
+        <v>45</v>
+      </c>
+      <c r="O26" t="s">
+        <v>45</v>
       </c>
       <c r="P26" t="s">
         <v>129</v>
       </c>
       <c r="Q26" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>40705877</v>
+      </c>
+      <c r="B27" t="s">
+        <v>131</v>
+      </c>
+      <c r="C27" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" t="s">
+        <v>132</v>
+      </c>
+      <c r="F27" t="s">
+        <v>134</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" t="s">
+        <v>155</v>
+      </c>
+      <c r="J27" t="s">
+        <v>140</v>
+      </c>
+      <c r="K27" t="s">
+        <v>15</v>
+      </c>
+      <c r="L27" t="s">
+        <v>15</v>
+      </c>
+      <c r="M27" t="s">
+        <v>15</v>
+      </c>
+      <c r="N27" t="s">
+        <v>15</v>
+      </c>
+      <c r="O27" t="s">
+        <v>15</v>
+      </c>
+      <c r="P27" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>40705877</v>
+      </c>
+      <c r="B28" t="s">
+        <v>131</v>
+      </c>
+      <c r="C28" t="s">
+        <v>141</v>
+      </c>
+      <c r="D28" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A29">
-        <v>40705877</v>
-      </c>
-      <c r="B29" t="s">
-        <v>131</v>
-      </c>
-      <c r="C29" t="s">
-        <v>136</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="E28" t="s">
         <v>132</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F28" t="s">
         <v>134</v>
       </c>
-      <c r="H29" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" t="s">
-        <v>133</v>
-      </c>
-      <c r="J29" t="s">
-        <v>137</v>
-      </c>
-      <c r="P29" t="s">
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="s">
+        <v>153</v>
+      </c>
+      <c r="J28" t="s">
+        <v>139</v>
+      </c>
+      <c r="K28" t="s">
+        <v>15</v>
+      </c>
+      <c r="L28" t="s">
+        <v>15</v>
+      </c>
+      <c r="M28" t="s">
+        <v>15</v>
+      </c>
+      <c r="N28" t="s">
+        <v>15</v>
+      </c>
+      <c r="O28" t="s">
+        <v>15</v>
+      </c>
+      <c r="P28" t="s">
         <v>129</v>
       </c>
-      <c r="Q29" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A30">
-        <v>40705877</v>
-      </c>
-      <c r="B30" t="s">
-        <v>131</v>
-      </c>
-      <c r="C30" t="s">
-        <v>142</v>
-      </c>
-      <c r="E30" t="s">
-        <v>132</v>
-      </c>
-      <c r="F30" t="s">
-        <v>134</v>
-      </c>
-      <c r="H30" t="b">
-        <v>1</v>
-      </c>
-      <c r="I30" t="s">
-        <v>133</v>
-      </c>
-      <c r="J30" t="s">
-        <v>140</v>
-      </c>
-      <c r="P30" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q30" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A31">
-        <v>40705877</v>
-      </c>
-      <c r="B31" t="s">
-        <v>131</v>
-      </c>
-      <c r="C31" t="s">
-        <v>143</v>
-      </c>
-      <c r="E31" t="s">
-        <v>132</v>
-      </c>
-      <c r="F31" t="s">
-        <v>134</v>
-      </c>
-      <c r="H31" t="b">
-        <v>1</v>
-      </c>
-      <c r="I31" t="s">
-        <v>133</v>
-      </c>
-      <c r="J31" t="s">
-        <v>138</v>
-      </c>
-      <c r="P31" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q31" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A32">
-        <v>40705877</v>
-      </c>
-      <c r="B32" t="s">
-        <v>131</v>
-      </c>
-      <c r="C32" t="s">
-        <v>144</v>
-      </c>
-      <c r="E32" t="s">
-        <v>132</v>
-      </c>
-      <c r="F32" t="s">
-        <v>134</v>
-      </c>
-      <c r="H32" t="b">
-        <v>1</v>
-      </c>
-      <c r="I32" t="s">
-        <v>133</v>
-      </c>
-      <c r="J32" t="s">
-        <v>141</v>
-      </c>
-      <c r="P32" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>135</v>
+      <c r="Q28" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
For 40705877, 32499527, performed extractions for SERT1, 2, 4, 5, 6, 7.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCF66B5D-7CC2-42C9-8A2D-DF6E2B5F9536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E68A2B5-6791-4CB9-A35E-F50E4F33F508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="173">
   <si>
     <t>PMID</t>
   </si>
@@ -511,13 +511,55 @@
   </si>
   <si>
     <t>Checked supplementaries for functional assays and found none</t>
+  </si>
+  <si>
+    <t>Human protein AKA "SirAL" by authors</t>
+  </si>
+  <si>
+    <t>SIRT1</t>
+  </si>
+  <si>
+    <t>SIRT2</t>
+  </si>
+  <si>
+    <t>SIRT4</t>
+  </si>
+  <si>
+    <t>SIRT5</t>
+  </si>
+  <si>
+    <t>SIRT6</t>
+  </si>
+  <si>
+    <t>SIRT7</t>
+  </si>
+  <si>
+    <t>Q96EB6</t>
+  </si>
+  <si>
+    <t>Q8IXJ6</t>
+  </si>
+  <si>
+    <t>Q9NXA8</t>
+  </si>
+  <si>
+    <t>Q9NRC8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q8N6T7 </t>
+  </si>
+  <si>
+    <t>Q9Y6E7</t>
+  </si>
+  <si>
+    <t>Functional assays</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -648,6 +690,12 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1371,7 +1419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="5" width="17.6328125" customWidth="1"/>
@@ -2560,7 +2608,7 @@
         <v>134</v>
       </c>
       <c r="G23" t="s">
-        <v>15</v>
+        <v>159</v>
       </c>
       <c r="H23" t="b">
         <v>1</v>
@@ -2619,10 +2667,10 @@
         <v>1</v>
       </c>
       <c r="I24" t="s">
-        <v>15</v>
+        <v>172</v>
       </c>
       <c r="J24" t="s">
-        <v>15</v>
+        <v>138</v>
       </c>
       <c r="K24" t="s">
         <v>15</v>
@@ -2654,34 +2702,34 @@
         <v>131</v>
       </c>
       <c r="C25" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="D25" t="s">
-        <v>15</v>
+        <v>145</v>
       </c>
       <c r="E25" t="s">
-        <v>132</v>
+        <v>160</v>
       </c>
       <c r="F25" t="s">
-        <v>134</v>
+        <v>166</v>
       </c>
       <c r="G25" t="s">
         <v>15</v>
       </c>
       <c r="H25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" t="s">
-        <v>155</v>
+        <v>133</v>
       </c>
       <c r="J25" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="K25" t="s">
-        <v>15</v>
+        <v>147</v>
       </c>
       <c r="L25" t="s">
-        <v>15</v>
+        <v>146</v>
       </c>
       <c r="M25" t="s">
         <v>15</v>
@@ -2696,60 +2744,60 @@
         <v>129</v>
       </c>
       <c r="Q25" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A26">
-        <v>40705877</v>
+        <v>32499527</v>
       </c>
       <c r="B26" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="C26" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D26" t="s">
-        <v>15</v>
+        <v>145</v>
       </c>
       <c r="E26" t="s">
-        <v>132</v>
+        <v>15</v>
       </c>
       <c r="F26" t="s">
-        <v>134</v>
+        <v>15</v>
       </c>
       <c r="G26" t="s">
         <v>15</v>
       </c>
       <c r="H26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="J26" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K26" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="L26" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="M26" t="s">
-        <v>45</v>
+        <v>149</v>
       </c>
       <c r="N26" t="s">
-        <v>45</v>
-      </c>
-      <c r="O26" t="s">
-        <v>45</v>
+        <v>17</v>
+      </c>
+      <c r="O26" t="b">
+        <v>1</v>
       </c>
       <c r="P26" t="s">
         <v>129</v>
       </c>
       <c r="Q26" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.35">
@@ -2760,34 +2808,34 @@
         <v>131</v>
       </c>
       <c r="C27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D27" t="s">
-        <v>15</v>
+        <v>145</v>
       </c>
       <c r="E27" t="s">
-        <v>132</v>
+        <v>161</v>
       </c>
       <c r="F27" t="s">
-        <v>134</v>
+        <v>167</v>
       </c>
       <c r="G27" t="s">
         <v>15</v>
       </c>
       <c r="H27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" t="s">
-        <v>155</v>
+        <v>133</v>
       </c>
       <c r="J27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="K27" t="s">
-        <v>15</v>
+        <v>147</v>
       </c>
       <c r="L27" t="s">
-        <v>15</v>
+        <v>146</v>
       </c>
       <c r="M27" t="s">
         <v>15</v>
@@ -2802,39 +2850,39 @@
         <v>129</v>
       </c>
       <c r="Q27" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A28">
-        <v>40705877</v>
+        <v>32499527</v>
       </c>
       <c r="B28" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="C28" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D28" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="E28" t="s">
-        <v>132</v>
+        <v>15</v>
       </c>
       <c r="F28" t="s">
-        <v>134</v>
+        <v>15</v>
       </c>
       <c r="G28" t="s">
         <v>15</v>
       </c>
       <c r="H28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="J28" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K28" t="s">
         <v>15</v>
@@ -2843,22 +2891,606 @@
         <v>15</v>
       </c>
       <c r="M28" t="s">
-        <v>15</v>
+        <v>149</v>
       </c>
       <c r="N28" t="s">
-        <v>15</v>
-      </c>
-      <c r="O28" t="s">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="O28" t="b">
+        <v>1</v>
       </c>
       <c r="P28" t="s">
         <v>129</v>
       </c>
       <c r="Q28" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>40705877</v>
+      </c>
+      <c r="B29" t="s">
+        <v>131</v>
+      </c>
+      <c r="C29" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" t="s">
+        <v>145</v>
+      </c>
+      <c r="E29" t="s">
+        <v>162</v>
+      </c>
+      <c r="F29" t="s">
+        <v>171</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" t="s">
+        <v>133</v>
+      </c>
+      <c r="J29" t="s">
+        <v>138</v>
+      </c>
+      <c r="K29" t="s">
+        <v>147</v>
+      </c>
+      <c r="L29" t="s">
+        <v>146</v>
+      </c>
+      <c r="M29" t="s">
+        <v>15</v>
+      </c>
+      <c r="N29" t="s">
+        <v>15</v>
+      </c>
+      <c r="O29" t="s">
+        <v>15</v>
+      </c>
+      <c r="P29" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>32499527</v>
+      </c>
+      <c r="B30" t="s">
+        <v>148</v>
+      </c>
+      <c r="C30" t="s">
+        <v>144</v>
+      </c>
+      <c r="D30" t="s">
+        <v>145</v>
+      </c>
+      <c r="E30" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30" t="s">
+        <v>15</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" t="b">
+        <v>1</v>
+      </c>
+      <c r="I30" t="s">
+        <v>172</v>
+      </c>
+      <c r="J30" t="s">
+        <v>138</v>
+      </c>
+      <c r="K30" t="s">
+        <v>15</v>
+      </c>
+      <c r="L30" t="s">
+        <v>15</v>
+      </c>
+      <c r="M30" t="s">
+        <v>149</v>
+      </c>
+      <c r="N30" t="s">
+        <v>17</v>
+      </c>
+      <c r="O30" t="b">
+        <v>1</v>
+      </c>
+      <c r="P30" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>40705877</v>
+      </c>
+      <c r="B31" t="s">
+        <v>131</v>
+      </c>
+      <c r="C31" t="s">
+        <v>144</v>
+      </c>
+      <c r="D31" t="s">
+        <v>145</v>
+      </c>
+      <c r="E31" t="s">
+        <v>163</v>
+      </c>
+      <c r="F31" t="s">
+        <v>168</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" t="b">
+        <v>1</v>
+      </c>
+      <c r="I31" t="s">
+        <v>133</v>
+      </c>
+      <c r="J31" t="s">
+        <v>138</v>
+      </c>
+      <c r="K31" t="s">
+        <v>147</v>
+      </c>
+      <c r="L31" t="s">
+        <v>146</v>
+      </c>
+      <c r="M31" t="s">
+        <v>15</v>
+      </c>
+      <c r="N31" t="s">
+        <v>15</v>
+      </c>
+      <c r="O31" t="s">
+        <v>15</v>
+      </c>
+      <c r="P31" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>32499527</v>
+      </c>
+      <c r="B32" t="s">
+        <v>148</v>
+      </c>
+      <c r="C32" t="s">
+        <v>144</v>
+      </c>
+      <c r="D32" t="s">
+        <v>145</v>
+      </c>
+      <c r="E32" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" t="s">
+        <v>15</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" t="b">
+        <v>1</v>
+      </c>
+      <c r="I32" t="s">
+        <v>172</v>
+      </c>
+      <c r="J32" t="s">
+        <v>138</v>
+      </c>
+      <c r="K32" t="s">
+        <v>15</v>
+      </c>
+      <c r="L32" t="s">
+        <v>15</v>
+      </c>
+      <c r="M32" t="s">
+        <v>149</v>
+      </c>
+      <c r="N32" t="s">
+        <v>17</v>
+      </c>
+      <c r="O32" t="b">
+        <v>1</v>
+      </c>
+      <c r="P32" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>40705877</v>
+      </c>
+      <c r="B33" t="s">
+        <v>131</v>
+      </c>
+      <c r="C33" t="s">
+        <v>144</v>
+      </c>
+      <c r="D33" t="s">
+        <v>145</v>
+      </c>
+      <c r="E33" t="s">
+        <v>164</v>
+      </c>
+      <c r="F33" t="s">
+        <v>170</v>
+      </c>
+      <c r="G33" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" t="b">
+        <v>1</v>
+      </c>
+      <c r="I33" t="s">
+        <v>133</v>
+      </c>
+      <c r="J33" t="s">
+        <v>138</v>
+      </c>
+      <c r="K33" t="s">
+        <v>147</v>
+      </c>
+      <c r="L33" t="s">
+        <v>146</v>
+      </c>
+      <c r="M33" t="s">
+        <v>15</v>
+      </c>
+      <c r="N33" t="s">
+        <v>15</v>
+      </c>
+      <c r="O33" t="s">
+        <v>15</v>
+      </c>
+      <c r="P33" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>32499527</v>
+      </c>
+      <c r="B34" t="s">
+        <v>148</v>
+      </c>
+      <c r="C34" t="s">
+        <v>144</v>
+      </c>
+      <c r="D34" t="s">
+        <v>145</v>
+      </c>
+      <c r="E34" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" t="s">
+        <v>15</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" t="b">
+        <v>1</v>
+      </c>
+      <c r="I34" t="s">
+        <v>172</v>
+      </c>
+      <c r="J34" t="s">
+        <v>138</v>
+      </c>
+      <c r="K34" t="s">
+        <v>15</v>
+      </c>
+      <c r="L34" t="s">
+        <v>15</v>
+      </c>
+      <c r="M34" t="s">
+        <v>149</v>
+      </c>
+      <c r="N34" t="s">
+        <v>17</v>
+      </c>
+      <c r="O34" t="b">
+        <v>1</v>
+      </c>
+      <c r="P34" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>40705877</v>
+      </c>
+      <c r="B35" t="s">
+        <v>131</v>
+      </c>
+      <c r="C35" t="s">
+        <v>144</v>
+      </c>
+      <c r="D35" t="s">
+        <v>145</v>
+      </c>
+      <c r="E35" t="s">
+        <v>165</v>
+      </c>
+      <c r="F35" t="s">
+        <v>169</v>
+      </c>
+      <c r="G35" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" t="b">
+        <v>1</v>
+      </c>
+      <c r="I35" t="s">
+        <v>133</v>
+      </c>
+      <c r="J35" t="s">
+        <v>138</v>
+      </c>
+      <c r="K35" t="s">
+        <v>147</v>
+      </c>
+      <c r="L35" t="s">
+        <v>146</v>
+      </c>
+      <c r="M35" t="s">
+        <v>15</v>
+      </c>
+      <c r="N35" t="s">
+        <v>15</v>
+      </c>
+      <c r="O35" t="s">
+        <v>15</v>
+      </c>
+      <c r="P35" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>40705877</v>
+      </c>
+      <c r="B36" t="s">
+        <v>131</v>
+      </c>
+      <c r="C36" t="s">
+        <v>135</v>
+      </c>
+      <c r="D36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E36" t="s">
+        <v>132</v>
+      </c>
+      <c r="F36" t="s">
+        <v>134</v>
+      </c>
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" t="s">
+        <v>155</v>
+      </c>
+      <c r="J36" t="s">
+        <v>136</v>
+      </c>
+      <c r="K36" t="s">
+        <v>15</v>
+      </c>
+      <c r="L36" t="s">
+        <v>15</v>
+      </c>
+      <c r="M36" t="s">
+        <v>15</v>
+      </c>
+      <c r="N36" t="s">
+        <v>15</v>
+      </c>
+      <c r="O36" t="s">
+        <v>15</v>
+      </c>
+      <c r="P36" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>40705877</v>
+      </c>
+      <c r="B37" t="s">
+        <v>131</v>
+      </c>
+      <c r="C37" t="s">
+        <v>142</v>
+      </c>
+      <c r="D37" t="s">
+        <v>15</v>
+      </c>
+      <c r="E37" t="s">
+        <v>132</v>
+      </c>
+      <c r="F37" t="s">
+        <v>134</v>
+      </c>
+      <c r="G37" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" t="b">
+        <v>0</v>
+      </c>
+      <c r="I37" t="s">
+        <v>155</v>
+      </c>
+      <c r="J37" t="s">
+        <v>137</v>
+      </c>
+      <c r="K37" t="s">
+        <v>44</v>
+      </c>
+      <c r="L37" t="s">
+        <v>45</v>
+      </c>
+      <c r="M37" t="s">
+        <v>45</v>
+      </c>
+      <c r="N37" t="s">
+        <v>45</v>
+      </c>
+      <c r="O37" t="s">
+        <v>45</v>
+      </c>
+      <c r="P37" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>40705877</v>
+      </c>
+      <c r="B38" t="s">
+        <v>131</v>
+      </c>
+      <c r="C38" t="s">
+        <v>143</v>
+      </c>
+      <c r="D38" t="s">
+        <v>15</v>
+      </c>
+      <c r="E38" t="s">
+        <v>132</v>
+      </c>
+      <c r="F38" t="s">
+        <v>134</v>
+      </c>
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" t="s">
+        <v>155</v>
+      </c>
+      <c r="J38" t="s">
+        <v>140</v>
+      </c>
+      <c r="K38" t="s">
+        <v>15</v>
+      </c>
+      <c r="L38" t="s">
+        <v>15</v>
+      </c>
+      <c r="M38" t="s">
+        <v>15</v>
+      </c>
+      <c r="N38" t="s">
+        <v>15</v>
+      </c>
+      <c r="O38" t="s">
+        <v>15</v>
+      </c>
+      <c r="P38" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>40705877</v>
+      </c>
+      <c r="B39" t="s">
+        <v>131</v>
+      </c>
+      <c r="C39" t="s">
+        <v>141</v>
+      </c>
+      <c r="D39" t="s">
+        <v>152</v>
+      </c>
+      <c r="E39" t="s">
+        <v>132</v>
+      </c>
+      <c r="F39" t="s">
+        <v>134</v>
+      </c>
+      <c r="G39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" t="b">
+        <v>0</v>
+      </c>
+      <c r="I39" t="s">
+        <v>153</v>
+      </c>
+      <c r="J39" t="s">
+        <v>139</v>
+      </c>
+      <c r="K39" t="s">
+        <v>15</v>
+      </c>
+      <c r="L39" t="s">
+        <v>15</v>
+      </c>
+      <c r="M39" t="s">
+        <v>15</v>
+      </c>
+      <c r="N39" t="s">
+        <v>15</v>
+      </c>
+      <c r="O39" t="s">
+        <v>15</v>
+      </c>
+      <c r="P39" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q39" t="s">
         <v>158</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Performed first round of extractions for 32937646. Initiated EMBOSS NEEDLE record keeping for AA sequence alignment. Added AA sequence annotations for bacterial and human genes.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E68A2B5-6791-4CB9-A35E-F50E4F33F508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45B5BB3B-DAC7-4484-BB79-219AE9DEB743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="195">
   <si>
     <t>PMID</t>
   </si>
@@ -294,9 +294,6 @@
     <t>No human similarity</t>
   </si>
   <si>
-    <t>overlaid Rhizobiales Pch2 with H. sapiens Trip13</t>
-  </si>
-  <si>
     <t>Q8N884</t>
   </si>
   <si>
@@ -553,6 +550,75 @@
   </si>
   <si>
     <t>Functional assays</t>
+  </si>
+  <si>
+    <t>Overlaid Rhizobiales Pch2 with H. sapiens Trip13</t>
+  </si>
+  <si>
+    <t>Q8WXG1</t>
+  </si>
+  <si>
+    <t>Prokaryotic viperins produce diverse antiviral molecules</t>
+  </si>
+  <si>
+    <t>RSAD2</t>
+  </si>
+  <si>
+    <t>Vipirin</t>
+  </si>
+  <si>
+    <t>antiphage; RNA polymerase inihibition</t>
+  </si>
+  <si>
+    <t>Cloned_into_organism</t>
+  </si>
+  <si>
+    <t>Did_structural_validation</t>
+  </si>
+  <si>
+    <t>No human homology; claim is there but evidence is absent</t>
+  </si>
+  <si>
+    <t>Lutibacter oricola</t>
+  </si>
+  <si>
+    <t>A0A1H3CMF9</t>
+  </si>
+  <si>
+    <t>Authors claim human homology but provide no evidence; BLASTp of AA sequence and 30 to 60% identity filter yields no human matches</t>
+  </si>
+  <si>
+    <t>From fig 1 description: "Homologues of human viperin are shown in red, genes annotated as nucleotide kinase are brown, genes known to be involved in defence are yellow and genes with mobile genetic elements are dark grey"; "We first performed a profile-based search for viperin homologues in a database of more than 38,000 bacterial and archaeal genomes. This search yielded 1,724 genes (1,112 non-redundant sequences) homologous to the human viperin gene (RSAD2)"</t>
+  </si>
+  <si>
+    <t>A0A1N7JN37</t>
+  </si>
+  <si>
+    <t>Chryseobacterium gambrini</t>
+  </si>
+  <si>
+    <t>Bacterial_AA_sequence</t>
+  </si>
+  <si>
+    <t>MRNLVEKGIIPAVNFHLWKACNYKCKFCFGTFNDVKKNNLEYEEAKRTVQNLAGFGFEKITFSGGEPTLCKYLPKLLKIAKNAGMTTSIVTNGSMLNYDWLNENKDYLDWIAISIDSINIETNIRSGRFNKNNSFTEEIYIELIQLIKEIGFKLKINTVVSNFNKNEDFNEFINWVKPERWKIFQALPIEVQNDKYKDDFMVNQFEFNNYLKRHKSSSYIKESNYDMKGSYIMVDPIGRFFENSKGIHKYSSKINSVGVERALSEINYCFKKFINREGLYDWE</t>
+  </si>
+  <si>
+    <t>METSFEGIIPSVNYHLWEPCNMKCRFCFATFQEAKKILPKGHLPKEQSLELIKQIAGMGFKKITFAGGEPTICPWISDLIAAAKESGMTTMLVTNGTKLNETFFKKNQKNLDWIILSIDSLNDTTNIKSGRAFKGKEPLTAEAYKLLIDEIKRYGFQLKINTVVHHLNYNESLMDLILYAQPKRWKVFQVLPMKGENDEHIEEFIISQQQFDHFIANHQFLKDHEILVSEDNSEMKDSYVMIDPAGRFFTNKEGFQEYSRPILEAGAKKAYDEMDYSYRNFLDRGGLYQWD</t>
+  </si>
+  <si>
+    <t>MPTPSTIRSVNWHLISACNYSCRFCFARNLGETPVSFSEGCRILTRLVGAGMEKINFAGGEPLLHPQLFEYCRVAHDLGMTVSITTNGSRLTPELVRTHRGYIDWIALSVDSASEETEARLGRGDGQHVGHCIRLSDAIRETGIRLKINTTVTALSRDEDMTGFVRRTDPDRWKVLQMLHIRGENDGAVADLSVTDAEFRAFADRHAGVILRGGVLPVFESSAMIEGSYFMVTPGGRVKTDTGRVIRKYSLDEVLGSGVFAYVDEGQYLRRGGVYAW</t>
+  </si>
+  <si>
+    <t>Human_AA_sequence</t>
+  </si>
+  <si>
+    <t>MWVLTPAAFAGKLLSVFRQPLSSLWRSLVPLFCWLRATFWLLATKRRKQQLVLRGPDETKEEEEDPPLPTTPTSVNYHFTRQCNYKCGFCFHTAKTSFVLPLEEAKRGLLLLKEAGMEKINFSGGEPFLQDRGEYLGKLVRFCKVELRLPSVSIVSNGSLIRERWFQNYGEYLDILAISCDSFDEEVNVLIGRGQGKKNHVENLQKLRRWCRDYRVAFKINSVINRFNVEEDMTEQIKALNPVRWKVFQCLLIEGENCGEDALREAERFVIGDEEFERFLERHKEVSCLVPESNQKMKDSYLILDEYMRFLNCRKGRKDPSKSILDVGVEEAIKFSGFDEKMFLKRGGKYIWSKADLKLDW</t>
+  </si>
+  <si>
+    <t>Authors claim human homology but provide no evidence; EMBOSS NEEDLE shows sufficient homology</t>
+  </si>
+  <si>
+    <t>T7 plaque assay; mutation assay</t>
   </si>
 </sst>
 </file>
@@ -1419,16 +1485,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:S47"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="5" width="17.6328125" customWidth="1"/>
-    <col min="6" max="6" width="17.453125" customWidth="1"/>
-    <col min="9" max="9" width="8.7265625" customWidth="1"/>
-    <col min="10" max="11" width="17.36328125" customWidth="1"/>
+    <col min="3" max="3" width="17.6328125" customWidth="1"/>
+    <col min="4" max="4" width="17.36328125" customWidth="1"/>
+    <col min="5" max="5" width="17.6328125" customWidth="1"/>
+    <col min="6" max="6" width="17.36328125" customWidth="1"/>
+    <col min="7" max="7" width="17.6328125" customWidth="1"/>
+    <col min="8" max="9" width="17.453125" customWidth="1"/>
+    <col min="10" max="10" width="9.7265625" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="17.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1436,52 +1507,58 @@
         <v>38</v>
       </c>
       <c r="C1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E1" t="s">
-        <v>98</v>
-      </c>
       <c r="F1" t="s">
+        <v>187</v>
+      </c>
+      <c r="G1" t="s">
         <v>97</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I1" t="s">
+        <v>191</v>
+      </c>
+      <c r="J1" t="s">
         <v>84</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>3</v>
       </c>
-      <c r="J1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>8</v>
       </c>
-      <c r="N1" t="s">
-        <v>9</v>
-      </c>
-      <c r="O1" t="s">
-        <v>10</v>
-      </c>
       <c r="P1" t="s">
-        <v>127</v>
+        <v>178</v>
       </c>
       <c r="Q1" t="s">
+        <v>179</v>
+      </c>
+      <c r="R1" t="s">
+        <v>126</v>
+      </c>
+      <c r="S1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>12110595</v>
       </c>
@@ -1492,49 +1569,55 @@
         <v>41</v>
       </c>
       <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
         <v>42</v>
       </c>
-      <c r="E2" t="s">
-        <v>45</v>
-      </c>
       <c r="F2" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s">
         <v>45</v>
       </c>
-      <c r="H2" t="b">
+      <c r="H2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" t="b">
         <v>0</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
         <v>43</v>
       </c>
-      <c r="J2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" t="s">
         <v>46</v>
-      </c>
-      <c r="M2" t="s">
-        <v>44</v>
-      </c>
-      <c r="N2" t="s">
-        <v>44</v>
       </c>
       <c r="O2" t="s">
         <v>44</v>
       </c>
       <c r="P2" t="s">
-        <v>128</v>
+        <v>44</v>
       </c>
       <c r="Q2" t="s">
+        <v>44</v>
+      </c>
+      <c r="R2" t="s">
+        <v>127</v>
+      </c>
+      <c r="S2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>30787435</v>
       </c>
@@ -1545,49 +1628,55 @@
         <v>53</v>
       </c>
       <c r="D3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" t="s">
         <v>54</v>
       </c>
-      <c r="E3" t="s">
-        <v>99</v>
-      </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>15</v>
       </c>
       <c r="G3" t="s">
-        <v>120</v>
-      </c>
-      <c r="H3" t="b">
+        <v>98</v>
+      </c>
+      <c r="H3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" t="s">
+        <v>119</v>
+      </c>
+      <c r="K3" t="b">
         <v>0</v>
       </c>
-      <c r="I3" t="s">
-        <v>122</v>
-      </c>
-      <c r="J3" t="s">
-        <v>55</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
+        <v>121</v>
+      </c>
+      <c r="M3" t="s">
         <v>48</v>
       </c>
-      <c r="L3" t="s">
+      <c r="N3" t="s">
         <v>73</v>
       </c>
-      <c r="M3" t="s">
+      <c r="O3" t="s">
         <v>61</v>
       </c>
-      <c r="N3" t="s">
+      <c r="P3" t="s">
         <v>62</v>
       </c>
-      <c r="O3" t="b">
+      <c r="Q3" t="b">
         <v>1</v>
       </c>
-      <c r="P3" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
+        <v>127</v>
+      </c>
+      <c r="S3" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>30787435</v>
       </c>
@@ -1598,49 +1687,55 @@
         <v>58</v>
       </c>
       <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
         <v>59</v>
       </c>
-      <c r="E4" t="s">
-        <v>99</v>
-      </c>
       <c r="F4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" t="s">
+        <v>98</v>
+      </c>
+      <c r="H4" t="s">
+        <v>86</v>
+      </c>
+      <c r="I4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" t="s">
+        <v>119</v>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="s">
+        <v>121</v>
+      </c>
+      <c r="M4" t="s">
+        <v>48</v>
+      </c>
+      <c r="N4" t="s">
+        <v>72</v>
+      </c>
+      <c r="O4" t="s">
+        <v>60</v>
+      </c>
+      <c r="P4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q4" t="b">
+        <v>1</v>
+      </c>
+      <c r="R4" t="s">
+        <v>127</v>
+      </c>
+      <c r="S4" t="s">
         <v>87</v>
       </c>
-      <c r="G4" t="s">
-        <v>120</v>
-      </c>
-      <c r="H4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" t="s">
-        <v>122</v>
-      </c>
-      <c r="J4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" t="s">
-        <v>48</v>
-      </c>
-      <c r="L4" t="s">
-        <v>72</v>
-      </c>
-      <c r="M4" t="s">
-        <v>60</v>
-      </c>
-      <c r="N4" t="s">
-        <v>15</v>
-      </c>
-      <c r="O4" t="b">
-        <v>1</v>
-      </c>
-      <c r="P4" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>30787435</v>
       </c>
@@ -1651,49 +1746,55 @@
         <v>58</v>
       </c>
       <c r="D5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E5" t="s">
+        <v>89</v>
+      </c>
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" t="s">
+        <v>98</v>
+      </c>
+      <c r="H5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="s">
+        <v>121</v>
+      </c>
+      <c r="M5" t="s">
+        <v>48</v>
+      </c>
+      <c r="N5" t="s">
         <v>90</v>
       </c>
-      <c r="E5" t="s">
-        <v>99</v>
-      </c>
-      <c r="F5" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" t="s">
-        <v>120</v>
-      </c>
-      <c r="H5" t="b">
+      <c r="O5" t="s">
+        <v>61</v>
+      </c>
+      <c r="P5" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q5" t="b">
         <v>1</v>
       </c>
-      <c r="I5" t="s">
-        <v>122</v>
-      </c>
-      <c r="J5" t="s">
-        <v>89</v>
-      </c>
-      <c r="K5" t="s">
-        <v>48</v>
-      </c>
-      <c r="L5" t="s">
-        <v>91</v>
-      </c>
-      <c r="M5" t="s">
-        <v>61</v>
-      </c>
-      <c r="N5" t="s">
-        <v>15</v>
-      </c>
-      <c r="O5" t="b">
-        <v>1</v>
-      </c>
-      <c r="P5" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="R5" t="s">
+        <v>127</v>
+      </c>
+      <c r="S5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>31695182</v>
       </c>
@@ -1704,49 +1805,55 @@
         <v>13</v>
       </c>
       <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
         <v>16</v>
       </c>
-      <c r="E6" t="s">
-        <v>45</v>
-      </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G6" t="s">
         <v>45</v>
       </c>
-      <c r="H6" t="b">
+      <c r="H6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K6" t="b">
         <v>0</v>
       </c>
-      <c r="I6" t="s">
+      <c r="L6" t="s">
         <v>14</v>
       </c>
-      <c r="J6" t="s">
-        <v>17</v>
-      </c>
-      <c r="K6" t="s">
+      <c r="M6" t="s">
         <v>18</v>
       </c>
-      <c r="L6" t="s">
-        <v>45</v>
-      </c>
-      <c r="M6" t="s">
-        <v>44</v>
-      </c>
       <c r="N6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="O6" t="s">
         <v>44</v>
       </c>
       <c r="P6" t="s">
-        <v>128</v>
+        <v>44</v>
       </c>
       <c r="Q6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+      <c r="R6" t="s">
+        <v>127</v>
+      </c>
+      <c r="S6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>31695182</v>
       </c>
@@ -1757,49 +1864,55 @@
         <v>19</v>
       </c>
       <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" t="s">
         <v>20</v>
       </c>
-      <c r="E7" t="s">
-        <v>45</v>
-      </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G7" t="s">
         <v>45</v>
       </c>
-      <c r="H7" t="b">
+      <c r="H7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" t="s">
+        <v>45</v>
+      </c>
+      <c r="K7" t="b">
         <v>0</v>
       </c>
-      <c r="I7" t="s">
+      <c r="L7" t="s">
         <v>14</v>
       </c>
-      <c r="J7" t="s">
-        <v>17</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="M7" t="s">
         <v>18</v>
       </c>
-      <c r="L7" t="s">
-        <v>45</v>
-      </c>
-      <c r="M7" t="s">
-        <v>44</v>
-      </c>
       <c r="N7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="O7" t="s">
         <v>44</v>
       </c>
       <c r="P7" t="s">
-        <v>128</v>
+        <v>44</v>
       </c>
       <c r="Q7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+      <c r="R7" t="s">
+        <v>127</v>
+      </c>
+      <c r="S7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>31695182</v>
       </c>
@@ -1810,49 +1923,55 @@
         <v>21</v>
       </c>
       <c r="D8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" t="s">
         <v>22</v>
       </c>
-      <c r="E8" t="s">
-        <v>45</v>
-      </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G8" t="s">
         <v>45</v>
       </c>
-      <c r="H8" t="b">
+      <c r="H8" t="s">
+        <v>45</v>
+      </c>
+      <c r="I8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" t="s">
+        <v>45</v>
+      </c>
+      <c r="K8" t="b">
         <v>0</v>
       </c>
-      <c r="I8" t="s">
+      <c r="L8" t="s">
         <v>14</v>
       </c>
-      <c r="J8" t="s">
-        <v>23</v>
-      </c>
-      <c r="K8" t="s">
+      <c r="M8" t="s">
         <v>18</v>
       </c>
-      <c r="L8" t="s">
-        <v>45</v>
-      </c>
-      <c r="M8" t="s">
-        <v>44</v>
-      </c>
       <c r="N8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="O8" t="s">
         <v>44</v>
       </c>
       <c r="P8" t="s">
-        <v>128</v>
+        <v>44</v>
       </c>
       <c r="Q8" t="s">
+        <v>44</v>
+      </c>
+      <c r="R8" t="s">
+        <v>127</v>
+      </c>
+      <c r="S8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>31695182</v>
       </c>
@@ -1869,26 +1988,26 @@
         <v>45</v>
       </c>
       <c r="F9" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G9" t="s">
         <v>45</v>
       </c>
-      <c r="H9" t="b">
+      <c r="H9" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" t="s">
+        <v>45</v>
+      </c>
+      <c r="K9" t="b">
         <v>0</v>
       </c>
-      <c r="I9" t="s">
+      <c r="L9" t="s">
         <v>14</v>
       </c>
-      <c r="J9" t="s">
-        <v>45</v>
-      </c>
-      <c r="K9" t="s">
-        <v>45</v>
-      </c>
-      <c r="L9" t="s">
-        <v>45</v>
-      </c>
       <c r="M9" t="s">
         <v>45</v>
       </c>
@@ -1899,13 +2018,19 @@
         <v>45</v>
       </c>
       <c r="P9" t="s">
-        <v>128</v>
+        <v>45</v>
       </c>
       <c r="Q9" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="R9" t="s">
+        <v>127</v>
+      </c>
+      <c r="S9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>31932165</v>
       </c>
@@ -1916,49 +2041,55 @@
         <v>65</v>
       </c>
       <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
         <v>66</v>
       </c>
-      <c r="E10" t="s">
-        <v>15</v>
-      </c>
       <c r="F10" t="s">
         <v>15</v>
       </c>
       <c r="G10" t="s">
         <v>15</v>
       </c>
-      <c r="H10" t="b">
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" t="s">
+        <v>15</v>
+      </c>
+      <c r="K10" t="b">
         <v>0</v>
       </c>
-      <c r="I10" t="s">
+      <c r="L10" t="s">
         <v>85</v>
       </c>
-      <c r="J10" t="s">
+      <c r="M10" t="s">
+        <v>48</v>
+      </c>
+      <c r="N10" t="s">
+        <v>74</v>
+      </c>
+      <c r="O10" t="s">
+        <v>71</v>
+      </c>
+      <c r="P10" t="s">
         <v>17</v>
       </c>
-      <c r="K10" t="s">
-        <v>48</v>
-      </c>
-      <c r="L10" t="s">
-        <v>74</v>
-      </c>
-      <c r="M10" t="s">
-        <v>71</v>
-      </c>
-      <c r="N10" t="s">
-        <v>17</v>
-      </c>
-      <c r="O10" t="b">
+      <c r="Q10" t="b">
         <v>1</v>
       </c>
-      <c r="P10" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="R10" t="s">
+        <v>127</v>
+      </c>
+      <c r="S10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>31932165</v>
       </c>
@@ -1969,49 +2100,55 @@
         <v>69</v>
       </c>
       <c r="D11" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" t="s">
         <v>68</v>
       </c>
-      <c r="E11" t="s">
-        <v>15</v>
-      </c>
       <c r="F11" t="s">
         <v>15</v>
       </c>
       <c r="G11" t="s">
         <v>15</v>
       </c>
-      <c r="H11" t="b">
+      <c r="H11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" t="s">
+        <v>15</v>
+      </c>
+      <c r="J11" t="s">
+        <v>15</v>
+      </c>
+      <c r="K11" t="b">
         <v>0</v>
       </c>
-      <c r="I11" t="s">
+      <c r="L11" t="s">
         <v>85</v>
       </c>
-      <c r="J11" t="s">
-        <v>67</v>
-      </c>
-      <c r="K11" t="s">
+      <c r="M11" t="s">
         <v>48</v>
       </c>
-      <c r="L11" t="s">
+      <c r="N11" t="s">
         <v>74</v>
       </c>
-      <c r="M11" t="s">
+      <c r="O11" t="s">
         <v>70</v>
       </c>
-      <c r="N11" t="s">
+      <c r="P11" t="s">
         <v>17</v>
       </c>
-      <c r="O11" t="b">
+      <c r="Q11" t="b">
         <v>1</v>
       </c>
-      <c r="P11" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="R11" t="s">
+        <v>127</v>
+      </c>
+      <c r="S11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>31932165</v>
       </c>
@@ -2022,49 +2159,55 @@
         <v>77</v>
       </c>
       <c r="D12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" t="s">
         <v>76</v>
       </c>
-      <c r="E12" t="s">
-        <v>15</v>
-      </c>
       <c r="F12" t="s">
         <v>15</v>
       </c>
       <c r="G12" t="s">
         <v>15</v>
       </c>
-      <c r="H12" t="b">
+      <c r="H12" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" t="s">
+        <v>15</v>
+      </c>
+      <c r="J12" t="s">
+        <v>15</v>
+      </c>
+      <c r="K12" t="b">
         <v>0</v>
       </c>
-      <c r="I12" t="s">
+      <c r="L12" t="s">
         <v>85</v>
       </c>
-      <c r="J12" t="s">
-        <v>67</v>
-      </c>
-      <c r="K12" t="s">
+      <c r="M12" t="s">
         <v>48</v>
       </c>
-      <c r="L12" t="s">
+      <c r="N12" t="s">
         <v>63</v>
       </c>
-      <c r="M12" t="s">
+      <c r="O12" t="s">
         <v>80</v>
       </c>
-      <c r="N12" t="s">
+      <c r="P12" t="s">
         <v>17</v>
       </c>
-      <c r="O12" t="b">
+      <c r="Q12" t="b">
         <v>1</v>
       </c>
-      <c r="P12" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q12" t="s">
+      <c r="R12" t="s">
+        <v>127</v>
+      </c>
+      <c r="S12" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>31932165</v>
       </c>
@@ -2075,49 +2218,55 @@
         <v>15</v>
       </c>
       <c r="D13" t="s">
-        <v>15</v>
+        <v>67</v>
       </c>
       <c r="E13" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="F13" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G13" t="s">
         <v>45</v>
       </c>
-      <c r="H13" t="b">
+      <c r="H13" t="s">
+        <v>45</v>
+      </c>
+      <c r="I13" t="s">
+        <v>15</v>
+      </c>
+      <c r="J13" t="s">
+        <v>45</v>
+      </c>
+      <c r="K13" t="b">
         <v>0</v>
       </c>
-      <c r="I13" t="s">
+      <c r="L13" t="s">
         <v>81</v>
       </c>
-      <c r="J13" t="s">
-        <v>67</v>
-      </c>
-      <c r="K13" t="s">
+      <c r="M13" t="s">
         <v>48</v>
       </c>
-      <c r="L13" t="s">
+      <c r="N13" t="s">
         <v>63</v>
       </c>
-      <c r="M13" t="s">
+      <c r="O13" t="s">
         <v>80</v>
       </c>
-      <c r="N13" t="s">
+      <c r="P13" t="s">
         <v>17</v>
       </c>
-      <c r="O13" t="b">
+      <c r="Q13" t="b">
         <v>1</v>
       </c>
-      <c r="P13" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q13" t="s">
+      <c r="R13" t="s">
+        <v>127</v>
+      </c>
+      <c r="S13" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>31932165</v>
       </c>
@@ -2128,7 +2277,7 @@
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>15</v>
+        <v>82</v>
       </c>
       <c r="E14" t="s">
         <v>15</v>
@@ -2137,40 +2286,46 @@
         <v>15</v>
       </c>
       <c r="G14" t="s">
-        <v>86</v>
-      </c>
-      <c r="H14" t="b">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" t="s">
+        <v>15</v>
+      </c>
+      <c r="J14" t="s">
+        <v>172</v>
+      </c>
+      <c r="K14" t="b">
         <v>0</v>
       </c>
-      <c r="I14" t="s">
+      <c r="L14" t="s">
         <v>81</v>
       </c>
-      <c r="J14" t="s">
-        <v>82</v>
-      </c>
-      <c r="K14" t="s">
+      <c r="M14" t="s">
         <v>48</v>
       </c>
-      <c r="L14" t="s">
+      <c r="N14" t="s">
         <v>63</v>
       </c>
-      <c r="M14" t="s">
+      <c r="O14" t="s">
         <v>80</v>
       </c>
-      <c r="N14" t="s">
+      <c r="P14" t="s">
         <v>17</v>
       </c>
-      <c r="O14" t="b">
+      <c r="Q14" t="b">
         <v>1</v>
       </c>
-      <c r="P14" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q14" t="s">
+      <c r="R14" t="s">
+        <v>127</v>
+      </c>
+      <c r="S14" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>32559405</v>
       </c>
@@ -2187,26 +2342,26 @@
         <v>45</v>
       </c>
       <c r="F15" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G15" t="s">
         <v>45</v>
       </c>
-      <c r="H15" t="b">
+      <c r="H15" t="s">
+        <v>45</v>
+      </c>
+      <c r="I15" t="s">
+        <v>15</v>
+      </c>
+      <c r="J15" t="s">
+        <v>45</v>
+      </c>
+      <c r="K15" t="b">
         <v>0</v>
       </c>
-      <c r="I15" t="s">
+      <c r="L15" t="s">
         <v>14</v>
       </c>
-      <c r="J15" t="s">
-        <v>45</v>
-      </c>
-      <c r="K15" t="s">
-        <v>45</v>
-      </c>
-      <c r="L15" t="s">
-        <v>45</v>
-      </c>
       <c r="M15" t="s">
         <v>45</v>
       </c>
@@ -2217,13 +2372,19 @@
         <v>45</v>
       </c>
       <c r="P15" t="s">
-        <v>128</v>
+        <v>45</v>
       </c>
       <c r="Q15" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="R15" t="s">
+        <v>127</v>
+      </c>
+      <c r="S15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>32839535</v>
       </c>
@@ -2240,187 +2401,205 @@
         <v>45</v>
       </c>
       <c r="F16" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G16" t="s">
         <v>45</v>
       </c>
-      <c r="H16" t="b">
+      <c r="H16" t="s">
+        <v>45</v>
+      </c>
+      <c r="I16" t="s">
+        <v>15</v>
+      </c>
+      <c r="J16" t="s">
+        <v>45</v>
+      </c>
+      <c r="K16" t="b">
         <v>0</v>
       </c>
-      <c r="I16" t="s">
+      <c r="L16" t="s">
         <v>50</v>
       </c>
-      <c r="J16" t="s">
-        <v>45</v>
-      </c>
-      <c r="K16" t="s">
+      <c r="M16" t="s">
         <v>48</v>
       </c>
-      <c r="L16" t="s">
+      <c r="N16" t="s">
         <v>63</v>
       </c>
-      <c r="M16" t="s">
-        <v>15</v>
-      </c>
-      <c r="N16" t="s">
-        <v>15</v>
-      </c>
-      <c r="O16" t="b">
+      <c r="O16" t="s">
+        <v>15</v>
+      </c>
+      <c r="P16" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q16" t="b">
         <v>0</v>
       </c>
-      <c r="P16" t="s">
-        <v>130</v>
-      </c>
-      <c r="Q16" t="s">
+      <c r="R16" t="s">
+        <v>129</v>
+      </c>
+      <c r="S16" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>39208803</v>
       </c>
       <c r="B17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C17" t="s">
+        <v>114</v>
+      </c>
+      <c r="D17" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17" t="s">
+        <v>111</v>
+      </c>
+      <c r="F17" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" t="s">
+        <v>112</v>
+      </c>
+      <c r="H17" t="s">
         <v>115</v>
       </c>
-      <c r="D17" t="s">
-        <v>112</v>
-      </c>
-      <c r="E17" t="s">
-        <v>113</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="I17" t="s">
+        <v>15</v>
+      </c>
+      <c r="J17" t="s">
         <v>116</v>
       </c>
-      <c r="G17" t="s">
+      <c r="K17" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" t="s">
+        <v>50</v>
+      </c>
+      <c r="M17" t="s">
         <v>117</v>
       </c>
-      <c r="H17" t="b">
-        <v>0</v>
-      </c>
-      <c r="I17" t="s">
-        <v>50</v>
-      </c>
-      <c r="J17" t="s">
-        <v>114</v>
-      </c>
-      <c r="K17" t="s">
+      <c r="N17" t="s">
+        <v>15</v>
+      </c>
+      <c r="O17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P17" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>15</v>
+      </c>
+      <c r="R17" t="s">
+        <v>129</v>
+      </c>
+      <c r="S17" t="s">
         <v>118</v>
       </c>
-      <c r="L17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M17" t="s">
-        <v>15</v>
-      </c>
-      <c r="N17" t="s">
-        <v>15</v>
-      </c>
-      <c r="O17" t="s">
-        <v>15</v>
-      </c>
-      <c r="P17" t="s">
-        <v>130</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>39208803</v>
       </c>
       <c r="B18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D18" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="E18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H18" t="s">
+        <v>15</v>
+      </c>
+      <c r="I18" t="s">
+        <v>15</v>
+      </c>
+      <c r="J18" t="s">
+        <v>15</v>
+      </c>
+      <c r="K18" t="b">
+        <v>0</v>
+      </c>
+      <c r="L18" t="s">
+        <v>120</v>
+      </c>
+      <c r="M18" t="s">
+        <v>108</v>
+      </c>
+      <c r="N18" t="s">
+        <v>15</v>
+      </c>
+      <c r="O18" t="s">
+        <v>15</v>
+      </c>
+      <c r="P18" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>15</v>
+      </c>
+      <c r="R18" t="s">
+        <v>129</v>
+      </c>
+      <c r="S18" t="s">
         <v>105</v>
       </c>
-      <c r="F18" t="s">
-        <v>15</v>
-      </c>
-      <c r="G18" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" t="b">
-        <v>0</v>
-      </c>
-      <c r="I18" t="s">
-        <v>121</v>
-      </c>
-      <c r="J18" t="s">
-        <v>45</v>
-      </c>
-      <c r="K18" t="s">
-        <v>109</v>
-      </c>
-      <c r="L18" t="s">
-        <v>15</v>
-      </c>
-      <c r="M18" t="s">
-        <v>15</v>
-      </c>
-      <c r="N18" t="s">
-        <v>15</v>
-      </c>
-      <c r="O18" t="s">
-        <v>15</v>
-      </c>
-      <c r="P18" t="s">
-        <v>130</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>39208803</v>
       </c>
       <c r="B19" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D19" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" t="s">
+        <v>99</v>
+      </c>
+      <c r="H19" t="s">
+        <v>93</v>
+      </c>
+      <c r="I19" t="s">
+        <v>15</v>
+      </c>
+      <c r="J19" t="s">
         <v>100</v>
       </c>
-      <c r="F19" t="s">
-        <v>94</v>
-      </c>
-      <c r="G19" t="s">
-        <v>101</v>
-      </c>
-      <c r="H19" t="b">
+      <c r="K19" t="b">
         <v>0</v>
       </c>
-      <c r="I19" t="s">
+      <c r="L19" t="s">
         <v>81</v>
       </c>
-      <c r="J19" t="s">
-        <v>17</v>
-      </c>
-      <c r="K19" t="s">
-        <v>109</v>
-      </c>
-      <c r="L19" t="s">
-        <v>15</v>
-      </c>
       <c r="M19" t="s">
-        <v>15</v>
+        <v>108</v>
       </c>
       <c r="N19" t="s">
         <v>15</v>
@@ -2429,48 +2608,54 @@
         <v>15</v>
       </c>
       <c r="P19" t="s">
-        <v>130</v>
+        <v>15</v>
       </c>
       <c r="Q19" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R19" t="s">
+        <v>129</v>
+      </c>
+      <c r="S19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>39208803</v>
       </c>
       <c r="B20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C20" t="s">
-        <v>107</v>
-      </c>
-      <c r="D20" t="s">
-        <v>45</v>
+        <v>106</v>
       </c>
       <c r="E20" t="s">
-        <v>102</v>
+        <v>45</v>
       </c>
       <c r="F20" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G20" t="s">
-        <v>45</v>
-      </c>
-      <c r="H20" t="b">
+        <v>101</v>
+      </c>
+      <c r="H20" t="s">
+        <v>45</v>
+      </c>
+      <c r="I20" t="s">
+        <v>15</v>
+      </c>
+      <c r="J20" t="s">
+        <v>45</v>
+      </c>
+      <c r="K20" t="b">
         <v>0</v>
       </c>
-      <c r="I20" t="s">
-        <v>121</v>
-      </c>
-      <c r="K20" t="s">
-        <v>104</v>
-      </c>
       <c r="L20" t="s">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="M20" t="s">
-        <v>15</v>
+        <v>103</v>
       </c>
       <c r="N20" t="s">
         <v>15</v>
@@ -2479,49 +2664,55 @@
         <v>15</v>
       </c>
       <c r="P20" t="s">
-        <v>130</v>
+        <v>15</v>
       </c>
       <c r="Q20" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R20" t="s">
+        <v>129</v>
+      </c>
+      <c r="S20" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>39208803</v>
       </c>
       <c r="B21" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C21" t="s">
-        <v>108</v>
-      </c>
-      <c r="D21" t="s">
-        <v>45</v>
+        <v>107</v>
       </c>
       <c r="E21" t="s">
+        <v>45</v>
+      </c>
+      <c r="F21" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" t="s">
+        <v>102</v>
+      </c>
+      <c r="H21" t="s">
+        <v>45</v>
+      </c>
+      <c r="I21" t="s">
+        <v>15</v>
+      </c>
+      <c r="J21" t="s">
+        <v>45</v>
+      </c>
+      <c r="K21" t="b">
+        <v>0</v>
+      </c>
+      <c r="L21" t="s">
+        <v>120</v>
+      </c>
+      <c r="M21" t="s">
         <v>103</v>
       </c>
-      <c r="F21" t="s">
-        <v>45</v>
-      </c>
-      <c r="G21" t="s">
-        <v>45</v>
-      </c>
-      <c r="H21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I21" t="s">
-        <v>121</v>
-      </c>
-      <c r="K21" t="s">
-        <v>104</v>
-      </c>
-      <c r="L21" t="s">
-        <v>15</v>
-      </c>
-      <c r="M21" t="s">
-        <v>15</v>
-      </c>
       <c r="N21" t="s">
         <v>15</v>
       </c>
@@ -2529,27 +2720,33 @@
         <v>15</v>
       </c>
       <c r="P21" t="s">
-        <v>130</v>
+        <v>15</v>
       </c>
       <c r="Q21" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R21" t="s">
+        <v>129</v>
+      </c>
+      <c r="S21" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>35164550</v>
       </c>
       <c r="B22" t="s">
+        <v>122</v>
+      </c>
+      <c r="C22" t="s">
         <v>123</v>
-      </c>
-      <c r="C22" t="s">
-        <v>124</v>
       </c>
       <c r="D22" t="s">
         <v>125</v>
       </c>
       <c r="E22" t="s">
-        <v>15</v>
+        <v>124</v>
       </c>
       <c r="F22" t="s">
         <v>15</v>
@@ -2557,21 +2754,21 @@
       <c r="G22" t="s">
         <v>15</v>
       </c>
-      <c r="H22" t="b">
+      <c r="H22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" t="s">
+        <v>15</v>
+      </c>
+      <c r="J22" t="s">
+        <v>15</v>
+      </c>
+      <c r="K22" t="b">
         <v>0</v>
       </c>
-      <c r="I22" t="s">
+      <c r="L22" t="s">
         <v>85</v>
       </c>
-      <c r="J22" t="s">
-        <v>126</v>
-      </c>
-      <c r="K22" t="s">
-        <v>45</v>
-      </c>
-      <c r="L22" t="s">
-        <v>45</v>
-      </c>
       <c r="M22" t="s">
         <v>45</v>
       </c>
@@ -2582,737 +2779,821 @@
         <v>45</v>
       </c>
       <c r="P22" t="s">
-        <v>129</v>
+        <v>45</v>
       </c>
       <c r="Q22" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
+        <v>45</v>
+      </c>
+      <c r="R22" t="s">
+        <v>128</v>
+      </c>
+      <c r="S22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>40705877</v>
       </c>
       <c r="B23" t="s">
+        <v>130</v>
+      </c>
+      <c r="C23" t="s">
+        <v>143</v>
+      </c>
+      <c r="D23" t="s">
+        <v>137</v>
+      </c>
+      <c r="E23" t="s">
+        <v>144</v>
+      </c>
+      <c r="F23" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" t="s">
         <v>131</v>
       </c>
-      <c r="C23" t="s">
-        <v>144</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="H23" t="s">
+        <v>133</v>
+      </c>
+      <c r="I23" t="s">
+        <v>15</v>
+      </c>
+      <c r="J23" t="s">
+        <v>158</v>
+      </c>
+      <c r="K23" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" t="s">
+        <v>132</v>
+      </c>
+      <c r="M23" t="s">
+        <v>146</v>
+      </c>
+      <c r="N23" t="s">
         <v>145</v>
       </c>
-      <c r="E23" t="s">
-        <v>132</v>
-      </c>
-      <c r="F23" t="s">
-        <v>134</v>
-      </c>
-      <c r="G23" t="s">
-        <v>159</v>
-      </c>
-      <c r="H23" t="b">
-        <v>1</v>
-      </c>
-      <c r="I23" t="s">
-        <v>133</v>
-      </c>
-      <c r="J23" t="s">
-        <v>138</v>
-      </c>
-      <c r="K23" t="s">
-        <v>147</v>
-      </c>
-      <c r="L23" t="s">
-        <v>146</v>
-      </c>
-      <c r="M23" t="s">
-        <v>15</v>
-      </c>
-      <c r="N23" t="s">
-        <v>15</v>
-      </c>
       <c r="O23" t="s">
         <v>15</v>
       </c>
       <c r="P23" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="Q23" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R23" t="s">
+        <v>128</v>
+      </c>
+      <c r="S23" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>32499527</v>
       </c>
       <c r="B24" t="s">
+        <v>147</v>
+      </c>
+      <c r="C24" t="s">
+        <v>143</v>
+      </c>
+      <c r="D24" t="s">
+        <v>137</v>
+      </c>
+      <c r="E24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F24" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="s">
+        <v>15</v>
+      </c>
+      <c r="I24" t="s">
+        <v>15</v>
+      </c>
+      <c r="J24" t="s">
+        <v>15</v>
+      </c>
+      <c r="K24" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" t="s">
+        <v>171</v>
+      </c>
+      <c r="M24" t="s">
+        <v>15</v>
+      </c>
+      <c r="N24" t="s">
+        <v>15</v>
+      </c>
+      <c r="O24" t="s">
         <v>148</v>
       </c>
-      <c r="C24" t="s">
-        <v>144</v>
-      </c>
-      <c r="D24" t="s">
-        <v>145</v>
-      </c>
-      <c r="E24" t="s">
-        <v>15</v>
-      </c>
-      <c r="F24" t="s">
-        <v>15</v>
-      </c>
-      <c r="G24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H24" t="b">
+      <c r="P24" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q24" t="b">
         <v>1</v>
       </c>
-      <c r="I24" t="s">
-        <v>172</v>
-      </c>
-      <c r="J24" t="s">
-        <v>138</v>
-      </c>
-      <c r="K24" t="s">
-        <v>15</v>
-      </c>
-      <c r="L24" t="s">
-        <v>15</v>
-      </c>
-      <c r="M24" t="s">
+      <c r="R24" t="s">
+        <v>128</v>
+      </c>
+      <c r="S24" t="s">
         <v>149</v>
       </c>
-      <c r="N24" t="s">
-        <v>17</v>
-      </c>
-      <c r="O24" t="b">
-        <v>1</v>
-      </c>
-      <c r="P24" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>40705877</v>
       </c>
       <c r="B25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C25" t="s">
+        <v>143</v>
+      </c>
+      <c r="D25" t="s">
+        <v>137</v>
+      </c>
+      <c r="E25" t="s">
         <v>144</v>
       </c>
-      <c r="D25" t="s">
+      <c r="F25" t="s">
+        <v>15</v>
+      </c>
+      <c r="G25" t="s">
+        <v>159</v>
+      </c>
+      <c r="H25" t="s">
+        <v>165</v>
+      </c>
+      <c r="I25" t="s">
+        <v>15</v>
+      </c>
+      <c r="J25" t="s">
+        <v>15</v>
+      </c>
+      <c r="K25" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" t="s">
+        <v>132</v>
+      </c>
+      <c r="M25" t="s">
+        <v>146</v>
+      </c>
+      <c r="N25" t="s">
         <v>145</v>
       </c>
-      <c r="E25" t="s">
-        <v>160</v>
-      </c>
-      <c r="F25" t="s">
-        <v>166</v>
-      </c>
-      <c r="G25" t="s">
-        <v>15</v>
-      </c>
-      <c r="H25" t="b">
-        <v>1</v>
-      </c>
-      <c r="I25" t="s">
-        <v>133</v>
-      </c>
-      <c r="J25" t="s">
-        <v>138</v>
-      </c>
-      <c r="K25" t="s">
-        <v>147</v>
-      </c>
-      <c r="L25" t="s">
-        <v>146</v>
-      </c>
-      <c r="M25" t="s">
-        <v>15</v>
-      </c>
-      <c r="N25" t="s">
-        <v>15</v>
-      </c>
       <c r="O25" t="s">
         <v>15</v>
       </c>
       <c r="P25" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="Q25" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R25" t="s">
+        <v>128</v>
+      </c>
+      <c r="S25" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>32499527</v>
       </c>
       <c r="B26" t="s">
+        <v>147</v>
+      </c>
+      <c r="C26" t="s">
+        <v>143</v>
+      </c>
+      <c r="D26" t="s">
+        <v>137</v>
+      </c>
+      <c r="E26" t="s">
+        <v>144</v>
+      </c>
+      <c r="F26" t="s">
+        <v>15</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="s">
+        <v>15</v>
+      </c>
+      <c r="I26" t="s">
+        <v>15</v>
+      </c>
+      <c r="J26" t="s">
+        <v>15</v>
+      </c>
+      <c r="K26" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" t="s">
+        <v>171</v>
+      </c>
+      <c r="M26" t="s">
+        <v>15</v>
+      </c>
+      <c r="N26" t="s">
+        <v>15</v>
+      </c>
+      <c r="O26" t="s">
         <v>148</v>
       </c>
-      <c r="C26" t="s">
-        <v>144</v>
-      </c>
-      <c r="D26" t="s">
-        <v>145</v>
-      </c>
-      <c r="E26" t="s">
-        <v>15</v>
-      </c>
-      <c r="F26" t="s">
-        <v>15</v>
-      </c>
-      <c r="G26" t="s">
-        <v>15</v>
-      </c>
-      <c r="H26" t="b">
+      <c r="P26" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q26" t="b">
         <v>1</v>
       </c>
-      <c r="I26" t="s">
-        <v>172</v>
-      </c>
-      <c r="J26" t="s">
-        <v>138</v>
-      </c>
-      <c r="K26" t="s">
-        <v>15</v>
-      </c>
-      <c r="L26" t="s">
-        <v>15</v>
-      </c>
-      <c r="M26" t="s">
+      <c r="R26" t="s">
+        <v>128</v>
+      </c>
+      <c r="S26" t="s">
         <v>149</v>
       </c>
-      <c r="N26" t="s">
-        <v>17</v>
-      </c>
-      <c r="O26" t="b">
-        <v>1</v>
-      </c>
-      <c r="P26" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q26" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>40705877</v>
       </c>
       <c r="B27" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C27" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" t="s">
+        <v>137</v>
+      </c>
+      <c r="E27" t="s">
         <v>144</v>
       </c>
-      <c r="D27" t="s">
+      <c r="F27" t="s">
+        <v>15</v>
+      </c>
+      <c r="G27" t="s">
+        <v>160</v>
+      </c>
+      <c r="H27" t="s">
+        <v>166</v>
+      </c>
+      <c r="I27" t="s">
+        <v>15</v>
+      </c>
+      <c r="J27" t="s">
+        <v>15</v>
+      </c>
+      <c r="K27" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" t="s">
+        <v>132</v>
+      </c>
+      <c r="M27" t="s">
+        <v>146</v>
+      </c>
+      <c r="N27" t="s">
         <v>145</v>
       </c>
-      <c r="E27" t="s">
-        <v>161</v>
-      </c>
-      <c r="F27" t="s">
-        <v>167</v>
-      </c>
-      <c r="G27" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" t="b">
-        <v>1</v>
-      </c>
-      <c r="I27" t="s">
-        <v>133</v>
-      </c>
-      <c r="J27" t="s">
-        <v>138</v>
-      </c>
-      <c r="K27" t="s">
-        <v>147</v>
-      </c>
-      <c r="L27" t="s">
-        <v>146</v>
-      </c>
-      <c r="M27" t="s">
-        <v>15</v>
-      </c>
-      <c r="N27" t="s">
-        <v>15</v>
-      </c>
       <c r="O27" t="s">
         <v>15</v>
       </c>
       <c r="P27" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="Q27" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R27" t="s">
+        <v>128</v>
+      </c>
+      <c r="S27" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>32499527</v>
       </c>
       <c r="B28" t="s">
+        <v>147</v>
+      </c>
+      <c r="C28" t="s">
+        <v>143</v>
+      </c>
+      <c r="D28" t="s">
+        <v>137</v>
+      </c>
+      <c r="E28" t="s">
+        <v>144</v>
+      </c>
+      <c r="F28" t="s">
+        <v>15</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" t="s">
+        <v>15</v>
+      </c>
+      <c r="I28" t="s">
+        <v>15</v>
+      </c>
+      <c r="J28" t="s">
+        <v>15</v>
+      </c>
+      <c r="K28" t="b">
+        <v>1</v>
+      </c>
+      <c r="L28" t="s">
+        <v>171</v>
+      </c>
+      <c r="M28" t="s">
+        <v>15</v>
+      </c>
+      <c r="N28" t="s">
+        <v>15</v>
+      </c>
+      <c r="O28" t="s">
         <v>148</v>
       </c>
-      <c r="C28" t="s">
-        <v>144</v>
-      </c>
-      <c r="D28" t="s">
-        <v>145</v>
-      </c>
-      <c r="E28" t="s">
-        <v>15</v>
-      </c>
-      <c r="F28" t="s">
-        <v>15</v>
-      </c>
-      <c r="G28" t="s">
-        <v>15</v>
-      </c>
-      <c r="H28" t="b">
+      <c r="P28" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q28" t="b">
         <v>1</v>
       </c>
-      <c r="I28" t="s">
-        <v>172</v>
-      </c>
-      <c r="J28" t="s">
-        <v>138</v>
-      </c>
-      <c r="K28" t="s">
-        <v>15</v>
-      </c>
-      <c r="L28" t="s">
-        <v>15</v>
-      </c>
-      <c r="M28" t="s">
+      <c r="R28" t="s">
+        <v>128</v>
+      </c>
+      <c r="S28" t="s">
         <v>149</v>
       </c>
-      <c r="N28" t="s">
-        <v>17</v>
-      </c>
-      <c r="O28" t="b">
-        <v>1</v>
-      </c>
-      <c r="P28" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>40705877</v>
       </c>
       <c r="B29" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C29" t="s">
+        <v>143</v>
+      </c>
+      <c r="D29" t="s">
+        <v>137</v>
+      </c>
+      <c r="E29" t="s">
         <v>144</v>
       </c>
-      <c r="D29" t="s">
+      <c r="F29" t="s">
+        <v>15</v>
+      </c>
+      <c r="G29" t="s">
+        <v>161</v>
+      </c>
+      <c r="H29" t="s">
+        <v>170</v>
+      </c>
+      <c r="I29" t="s">
+        <v>15</v>
+      </c>
+      <c r="J29" t="s">
+        <v>15</v>
+      </c>
+      <c r="K29" t="b">
+        <v>1</v>
+      </c>
+      <c r="L29" t="s">
+        <v>132</v>
+      </c>
+      <c r="M29" t="s">
+        <v>146</v>
+      </c>
+      <c r="N29" t="s">
         <v>145</v>
       </c>
-      <c r="E29" t="s">
-        <v>162</v>
-      </c>
-      <c r="F29" t="s">
-        <v>171</v>
-      </c>
-      <c r="G29" t="s">
-        <v>15</v>
-      </c>
-      <c r="H29" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" t="s">
-        <v>133</v>
-      </c>
-      <c r="J29" t="s">
-        <v>138</v>
-      </c>
-      <c r="K29" t="s">
-        <v>147</v>
-      </c>
-      <c r="L29" t="s">
-        <v>146</v>
-      </c>
-      <c r="M29" t="s">
-        <v>15</v>
-      </c>
-      <c r="N29" t="s">
-        <v>15</v>
-      </c>
       <c r="O29" t="s">
         <v>15</v>
       </c>
       <c r="P29" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="Q29" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R29" t="s">
+        <v>128</v>
+      </c>
+      <c r="S29" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>32499527</v>
       </c>
       <c r="B30" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" t="s">
+        <v>143</v>
+      </c>
+      <c r="D30" t="s">
+        <v>137</v>
+      </c>
+      <c r="E30" t="s">
+        <v>144</v>
+      </c>
+      <c r="F30" t="s">
+        <v>15</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" t="s">
+        <v>15</v>
+      </c>
+      <c r="I30" t="s">
+        <v>15</v>
+      </c>
+      <c r="J30" t="s">
+        <v>15</v>
+      </c>
+      <c r="K30" t="b">
+        <v>1</v>
+      </c>
+      <c r="L30" t="s">
+        <v>171</v>
+      </c>
+      <c r="M30" t="s">
+        <v>15</v>
+      </c>
+      <c r="N30" t="s">
+        <v>15</v>
+      </c>
+      <c r="O30" t="s">
         <v>148</v>
       </c>
-      <c r="C30" t="s">
-        <v>144</v>
-      </c>
-      <c r="D30" t="s">
-        <v>145</v>
-      </c>
-      <c r="E30" t="s">
-        <v>15</v>
-      </c>
-      <c r="F30" t="s">
-        <v>15</v>
-      </c>
-      <c r="G30" t="s">
-        <v>15</v>
-      </c>
-      <c r="H30" t="b">
+      <c r="P30" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q30" t="b">
         <v>1</v>
       </c>
-      <c r="I30" t="s">
-        <v>172</v>
-      </c>
-      <c r="J30" t="s">
-        <v>138</v>
-      </c>
-      <c r="K30" t="s">
-        <v>15</v>
-      </c>
-      <c r="L30" t="s">
-        <v>15</v>
-      </c>
-      <c r="M30" t="s">
+      <c r="R30" t="s">
+        <v>128</v>
+      </c>
+      <c r="S30" t="s">
         <v>149</v>
       </c>
-      <c r="N30" t="s">
-        <v>17</v>
-      </c>
-      <c r="O30" t="b">
-        <v>1</v>
-      </c>
-      <c r="P30" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q30" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>40705877</v>
       </c>
       <c r="B31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C31" t="s">
+        <v>143</v>
+      </c>
+      <c r="D31" t="s">
+        <v>137</v>
+      </c>
+      <c r="E31" t="s">
         <v>144</v>
       </c>
-      <c r="D31" t="s">
+      <c r="F31" t="s">
+        <v>15</v>
+      </c>
+      <c r="G31" t="s">
+        <v>162</v>
+      </c>
+      <c r="H31" t="s">
+        <v>167</v>
+      </c>
+      <c r="I31" t="s">
+        <v>15</v>
+      </c>
+      <c r="J31" t="s">
+        <v>15</v>
+      </c>
+      <c r="K31" t="b">
+        <v>1</v>
+      </c>
+      <c r="L31" t="s">
+        <v>132</v>
+      </c>
+      <c r="M31" t="s">
+        <v>146</v>
+      </c>
+      <c r="N31" t="s">
         <v>145</v>
       </c>
-      <c r="E31" t="s">
-        <v>163</v>
-      </c>
-      <c r="F31" t="s">
-        <v>168</v>
-      </c>
-      <c r="G31" t="s">
-        <v>15</v>
-      </c>
-      <c r="H31" t="b">
-        <v>1</v>
-      </c>
-      <c r="I31" t="s">
-        <v>133</v>
-      </c>
-      <c r="J31" t="s">
-        <v>138</v>
-      </c>
-      <c r="K31" t="s">
-        <v>147</v>
-      </c>
-      <c r="L31" t="s">
-        <v>146</v>
-      </c>
-      <c r="M31" t="s">
-        <v>15</v>
-      </c>
-      <c r="N31" t="s">
-        <v>15</v>
-      </c>
       <c r="O31" t="s">
         <v>15</v>
       </c>
       <c r="P31" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="Q31" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R31" t="s">
+        <v>128</v>
+      </c>
+      <c r="S31" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>32499527</v>
       </c>
       <c r="B32" t="s">
+        <v>147</v>
+      </c>
+      <c r="C32" t="s">
+        <v>143</v>
+      </c>
+      <c r="D32" t="s">
+        <v>137</v>
+      </c>
+      <c r="E32" t="s">
+        <v>144</v>
+      </c>
+      <c r="F32" t="s">
+        <v>15</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" t="s">
+        <v>15</v>
+      </c>
+      <c r="I32" t="s">
+        <v>15</v>
+      </c>
+      <c r="J32" t="s">
+        <v>15</v>
+      </c>
+      <c r="K32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L32" t="s">
+        <v>171</v>
+      </c>
+      <c r="M32" t="s">
+        <v>15</v>
+      </c>
+      <c r="N32" t="s">
+        <v>15</v>
+      </c>
+      <c r="O32" t="s">
         <v>148</v>
       </c>
-      <c r="C32" t="s">
-        <v>144</v>
-      </c>
-      <c r="D32" t="s">
-        <v>145</v>
-      </c>
-      <c r="E32" t="s">
-        <v>15</v>
-      </c>
-      <c r="F32" t="s">
-        <v>15</v>
-      </c>
-      <c r="G32" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" t="b">
+      <c r="P32" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q32" t="b">
         <v>1</v>
       </c>
-      <c r="I32" t="s">
-        <v>172</v>
-      </c>
-      <c r="J32" t="s">
-        <v>138</v>
-      </c>
-      <c r="K32" t="s">
-        <v>15</v>
-      </c>
-      <c r="L32" t="s">
-        <v>15</v>
-      </c>
-      <c r="M32" t="s">
+      <c r="R32" t="s">
+        <v>128</v>
+      </c>
+      <c r="S32" t="s">
         <v>149</v>
       </c>
-      <c r="N32" t="s">
-        <v>17</v>
-      </c>
-      <c r="O32" t="b">
-        <v>1</v>
-      </c>
-      <c r="P32" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>40705877</v>
       </c>
       <c r="B33" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C33" t="s">
+        <v>143</v>
+      </c>
+      <c r="D33" t="s">
+        <v>137</v>
+      </c>
+      <c r="E33" t="s">
         <v>144</v>
       </c>
-      <c r="D33" t="s">
+      <c r="F33" t="s">
+        <v>15</v>
+      </c>
+      <c r="G33" t="s">
+        <v>163</v>
+      </c>
+      <c r="H33" t="s">
+        <v>169</v>
+      </c>
+      <c r="I33" t="s">
+        <v>15</v>
+      </c>
+      <c r="J33" t="s">
+        <v>15</v>
+      </c>
+      <c r="K33" t="b">
+        <v>1</v>
+      </c>
+      <c r="L33" t="s">
+        <v>132</v>
+      </c>
+      <c r="M33" t="s">
+        <v>146</v>
+      </c>
+      <c r="N33" t="s">
         <v>145</v>
       </c>
-      <c r="E33" t="s">
-        <v>164</v>
-      </c>
-      <c r="F33" t="s">
-        <v>170</v>
-      </c>
-      <c r="G33" t="s">
-        <v>15</v>
-      </c>
-      <c r="H33" t="b">
-        <v>1</v>
-      </c>
-      <c r="I33" t="s">
-        <v>133</v>
-      </c>
-      <c r="J33" t="s">
-        <v>138</v>
-      </c>
-      <c r="K33" t="s">
-        <v>147</v>
-      </c>
-      <c r="L33" t="s">
-        <v>146</v>
-      </c>
-      <c r="M33" t="s">
-        <v>15</v>
-      </c>
-      <c r="N33" t="s">
-        <v>15</v>
-      </c>
       <c r="O33" t="s">
         <v>15</v>
       </c>
       <c r="P33" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="Q33" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R33" t="s">
+        <v>128</v>
+      </c>
+      <c r="S33" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>32499527</v>
       </c>
       <c r="B34" t="s">
+        <v>147</v>
+      </c>
+      <c r="C34" t="s">
+        <v>143</v>
+      </c>
+      <c r="D34" t="s">
+        <v>137</v>
+      </c>
+      <c r="E34" t="s">
+        <v>144</v>
+      </c>
+      <c r="F34" t="s">
+        <v>15</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" t="s">
+        <v>15</v>
+      </c>
+      <c r="I34" t="s">
+        <v>15</v>
+      </c>
+      <c r="J34" t="s">
+        <v>15</v>
+      </c>
+      <c r="K34" t="b">
+        <v>1</v>
+      </c>
+      <c r="L34" t="s">
+        <v>171</v>
+      </c>
+      <c r="M34" t="s">
+        <v>15</v>
+      </c>
+      <c r="N34" t="s">
+        <v>15</v>
+      </c>
+      <c r="O34" t="s">
         <v>148</v>
       </c>
-      <c r="C34" t="s">
-        <v>144</v>
-      </c>
-      <c r="D34" t="s">
-        <v>145</v>
-      </c>
-      <c r="E34" t="s">
-        <v>15</v>
-      </c>
-      <c r="F34" t="s">
-        <v>15</v>
-      </c>
-      <c r="G34" t="s">
-        <v>15</v>
-      </c>
-      <c r="H34" t="b">
+      <c r="P34" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q34" t="b">
         <v>1</v>
       </c>
-      <c r="I34" t="s">
-        <v>172</v>
-      </c>
-      <c r="J34" t="s">
-        <v>138</v>
-      </c>
-      <c r="K34" t="s">
-        <v>15</v>
-      </c>
-      <c r="L34" t="s">
-        <v>15</v>
-      </c>
-      <c r="M34" t="s">
+      <c r="R34" t="s">
+        <v>128</v>
+      </c>
+      <c r="S34" t="s">
         <v>149</v>
       </c>
-      <c r="N34" t="s">
-        <v>17</v>
-      </c>
-      <c r="O34" t="b">
-        <v>1</v>
-      </c>
-      <c r="P34" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q34" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>40705877</v>
       </c>
       <c r="B35" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C35" t="s">
+        <v>143</v>
+      </c>
+      <c r="D35" t="s">
+        <v>137</v>
+      </c>
+      <c r="E35" t="s">
         <v>144</v>
       </c>
-      <c r="D35" t="s">
+      <c r="F35" t="s">
+        <v>15</v>
+      </c>
+      <c r="G35" t="s">
+        <v>164</v>
+      </c>
+      <c r="H35" t="s">
+        <v>168</v>
+      </c>
+      <c r="I35" t="s">
+        <v>15</v>
+      </c>
+      <c r="J35" t="s">
+        <v>15</v>
+      </c>
+      <c r="K35" t="b">
+        <v>1</v>
+      </c>
+      <c r="L35" t="s">
+        <v>132</v>
+      </c>
+      <c r="M35" t="s">
+        <v>146</v>
+      </c>
+      <c r="N35" t="s">
         <v>145</v>
       </c>
-      <c r="E35" t="s">
-        <v>165</v>
-      </c>
-      <c r="F35" t="s">
-        <v>169</v>
-      </c>
-      <c r="G35" t="s">
-        <v>15</v>
-      </c>
-      <c r="H35" t="b">
-        <v>1</v>
-      </c>
-      <c r="I35" t="s">
-        <v>133</v>
-      </c>
-      <c r="J35" t="s">
-        <v>138</v>
-      </c>
-      <c r="K35" t="s">
-        <v>147</v>
-      </c>
-      <c r="L35" t="s">
-        <v>146</v>
-      </c>
-      <c r="M35" t="s">
-        <v>15</v>
-      </c>
-      <c r="N35" t="s">
-        <v>15</v>
-      </c>
       <c r="O35" t="s">
         <v>15</v>
       </c>
       <c r="P35" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="Q35" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R35" t="s">
+        <v>128</v>
+      </c>
+      <c r="S35" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>40705877</v>
       </c>
       <c r="B36" t="s">
+        <v>130</v>
+      </c>
+      <c r="C36" t="s">
+        <v>134</v>
+      </c>
+      <c r="D36" t="s">
+        <v>135</v>
+      </c>
+      <c r="E36" t="s">
+        <v>15</v>
+      </c>
+      <c r="F36" t="s">
+        <v>15</v>
+      </c>
+      <c r="G36" t="s">
         <v>131</v>
       </c>
-      <c r="C36" t="s">
-        <v>135</v>
-      </c>
-      <c r="D36" t="s">
-        <v>15</v>
-      </c>
-      <c r="E36" t="s">
-        <v>132</v>
-      </c>
-      <c r="F36" t="s">
-        <v>134</v>
-      </c>
-      <c r="G36" t="s">
-        <v>15</v>
-      </c>
-      <c r="H36" t="b">
+      <c r="H36" t="s">
+        <v>133</v>
+      </c>
+      <c r="I36" t="s">
+        <v>15</v>
+      </c>
+      <c r="J36" t="s">
+        <v>15</v>
+      </c>
+      <c r="K36" t="b">
         <v>0</v>
       </c>
-      <c r="I36" t="s">
-        <v>155</v>
-      </c>
-      <c r="J36" t="s">
-        <v>136</v>
-      </c>
-      <c r="K36" t="s">
-        <v>15</v>
-      </c>
       <c r="L36" t="s">
-        <v>15</v>
+        <v>154</v>
       </c>
       <c r="M36" t="s">
         <v>15</v>
@@ -3324,101 +3605,113 @@
         <v>15</v>
       </c>
       <c r="P36" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="Q36" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R36" t="s">
+        <v>128</v>
+      </c>
+      <c r="S36" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>40705877</v>
       </c>
       <c r="B37" t="s">
+        <v>130</v>
+      </c>
+      <c r="C37" t="s">
+        <v>141</v>
+      </c>
+      <c r="D37" t="s">
+        <v>136</v>
+      </c>
+      <c r="E37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F37" t="s">
+        <v>15</v>
+      </c>
+      <c r="G37" t="s">
         <v>131</v>
       </c>
-      <c r="C37" t="s">
-        <v>142</v>
-      </c>
-      <c r="D37" t="s">
-        <v>15</v>
-      </c>
-      <c r="E37" t="s">
-        <v>132</v>
-      </c>
-      <c r="F37" t="s">
-        <v>134</v>
-      </c>
-      <c r="G37" t="s">
-        <v>15</v>
-      </c>
-      <c r="H37" t="b">
+      <c r="H37" t="s">
+        <v>133</v>
+      </c>
+      <c r="I37" t="s">
+        <v>15</v>
+      </c>
+      <c r="J37" t="s">
+        <v>15</v>
+      </c>
+      <c r="K37" t="b">
         <v>0</v>
       </c>
-      <c r="I37" t="s">
+      <c r="L37" t="s">
+        <v>154</v>
+      </c>
+      <c r="M37" t="s">
+        <v>44</v>
+      </c>
+      <c r="N37" t="s">
+        <v>45</v>
+      </c>
+      <c r="O37" t="s">
+        <v>45</v>
+      </c>
+      <c r="P37" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>45</v>
+      </c>
+      <c r="R37" t="s">
+        <v>128</v>
+      </c>
+      <c r="S37" t="s">
         <v>155</v>
       </c>
-      <c r="J37" t="s">
-        <v>137</v>
-      </c>
-      <c r="K37" t="s">
-        <v>44</v>
-      </c>
-      <c r="L37" t="s">
-        <v>45</v>
-      </c>
-      <c r="M37" t="s">
-        <v>45</v>
-      </c>
-      <c r="N37" t="s">
-        <v>45</v>
-      </c>
-      <c r="O37" t="s">
-        <v>45</v>
-      </c>
-      <c r="P37" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q37" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>40705877</v>
       </c>
       <c r="B38" t="s">
+        <v>130</v>
+      </c>
+      <c r="C38" t="s">
+        <v>142</v>
+      </c>
+      <c r="D38" t="s">
+        <v>139</v>
+      </c>
+      <c r="E38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F38" t="s">
+        <v>15</v>
+      </c>
+      <c r="G38" t="s">
         <v>131</v>
       </c>
-      <c r="C38" t="s">
-        <v>143</v>
-      </c>
-      <c r="D38" t="s">
-        <v>15</v>
-      </c>
-      <c r="E38" t="s">
-        <v>132</v>
-      </c>
-      <c r="F38" t="s">
-        <v>134</v>
-      </c>
-      <c r="G38" t="s">
-        <v>15</v>
-      </c>
-      <c r="H38" t="b">
+      <c r="H38" t="s">
+        <v>133</v>
+      </c>
+      <c r="I38" t="s">
+        <v>15</v>
+      </c>
+      <c r="J38" t="s">
+        <v>15</v>
+      </c>
+      <c r="K38" t="b">
         <v>0</v>
       </c>
-      <c r="I38" t="s">
-        <v>155</v>
-      </c>
-      <c r="J38" t="s">
-        <v>140</v>
-      </c>
-      <c r="K38" t="s">
-        <v>15</v>
-      </c>
       <c r="L38" t="s">
-        <v>15</v>
+        <v>154</v>
       </c>
       <c r="M38" t="s">
         <v>15</v>
@@ -3430,63 +3723,252 @@
         <v>15</v>
       </c>
       <c r="P38" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="Q38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="R38" t="s">
+        <v>128</v>
+      </c>
+      <c r="S38" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>40705877</v>
       </c>
       <c r="B39" t="s">
+        <v>130</v>
+      </c>
+      <c r="C39" t="s">
+        <v>140</v>
+      </c>
+      <c r="D39" t="s">
+        <v>138</v>
+      </c>
+      <c r="E39" t="s">
+        <v>151</v>
+      </c>
+      <c r="F39" t="s">
+        <v>15</v>
+      </c>
+      <c r="G39" t="s">
         <v>131</v>
       </c>
-      <c r="C39" t="s">
-        <v>141</v>
-      </c>
-      <c r="D39" t="s">
+      <c r="H39" t="s">
+        <v>133</v>
+      </c>
+      <c r="I39" t="s">
+        <v>15</v>
+      </c>
+      <c r="J39" t="s">
+        <v>15</v>
+      </c>
+      <c r="K39" t="b">
+        <v>0</v>
+      </c>
+      <c r="L39" t="s">
         <v>152</v>
       </c>
-      <c r="E39" t="s">
-        <v>132</v>
-      </c>
-      <c r="F39" t="s">
-        <v>134</v>
-      </c>
-      <c r="G39" t="s">
-        <v>15</v>
-      </c>
-      <c r="H39" t="b">
+      <c r="M39" t="s">
+        <v>15</v>
+      </c>
+      <c r="N39" t="s">
+        <v>15</v>
+      </c>
+      <c r="O39" t="s">
+        <v>15</v>
+      </c>
+      <c r="P39" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>15</v>
+      </c>
+      <c r="R39" t="s">
+        <v>128</v>
+      </c>
+      <c r="S39" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>32937646</v>
+      </c>
+      <c r="B43" t="s">
+        <v>174</v>
+      </c>
+      <c r="C43" t="s">
+        <v>15</v>
+      </c>
+      <c r="D43" t="s">
+        <v>181</v>
+      </c>
+      <c r="E43" t="s">
+        <v>182</v>
+      </c>
+      <c r="F43" t="s">
+        <v>188</v>
+      </c>
+      <c r="G43" t="s">
+        <v>175</v>
+      </c>
+      <c r="H43" t="s">
+        <v>173</v>
+      </c>
+      <c r="I43" t="s">
+        <v>192</v>
+      </c>
+      <c r="J43" t="s">
+        <v>193</v>
+      </c>
+      <c r="K43" t="b">
+        <v>1</v>
+      </c>
+      <c r="L43" t="s">
+        <v>15</v>
+      </c>
+      <c r="M43" t="s">
+        <v>176</v>
+      </c>
+      <c r="N43" t="s">
+        <v>177</v>
+      </c>
+      <c r="O43" t="s">
+        <v>194</v>
+      </c>
+      <c r="P43" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>15</v>
+      </c>
+      <c r="R43" t="s">
+        <v>129</v>
+      </c>
+      <c r="S43" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>32937646</v>
+      </c>
+      <c r="B44" t="s">
+        <v>174</v>
+      </c>
+      <c r="C44" t="s">
+        <v>15</v>
+      </c>
+      <c r="D44" t="s">
+        <v>186</v>
+      </c>
+      <c r="E44" t="s">
+        <v>185</v>
+      </c>
+      <c r="F44" t="s">
+        <v>189</v>
+      </c>
+      <c r="G44" t="s">
+        <v>175</v>
+      </c>
+      <c r="H44" t="s">
+        <v>173</v>
+      </c>
+      <c r="I44" t="s">
+        <v>192</v>
+      </c>
+      <c r="J44" t="s">
+        <v>183</v>
+      </c>
+      <c r="K44" t="b">
         <v>0</v>
       </c>
-      <c r="I39" t="s">
-        <v>153</v>
-      </c>
-      <c r="J39" t="s">
-        <v>139</v>
-      </c>
-      <c r="K39" t="s">
-        <v>15</v>
-      </c>
-      <c r="L39" t="s">
-        <v>15</v>
-      </c>
-      <c r="M39" t="s">
-        <v>15</v>
-      </c>
-      <c r="N39" t="s">
-        <v>15</v>
-      </c>
-      <c r="O39" t="s">
-        <v>15</v>
-      </c>
-      <c r="P39" t="s">
+      <c r="L44" t="s">
+        <v>180</v>
+      </c>
+      <c r="M44" t="s">
+        <v>176</v>
+      </c>
+      <c r="N44" t="s">
+        <v>177</v>
+      </c>
+      <c r="O44" t="s">
+        <v>194</v>
+      </c>
+      <c r="P44" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R44" t="s">
         <v>129</v>
       </c>
-      <c r="Q39" t="s">
-        <v>158</v>
+      <c r="S44" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>32937646</v>
+      </c>
+      <c r="B47" t="s">
+        <v>174</v>
+      </c>
+      <c r="C47" t="s">
+        <v>15</v>
+      </c>
+      <c r="D47" t="s">
+        <v>186</v>
+      </c>
+      <c r="E47" t="s">
+        <v>185</v>
+      </c>
+      <c r="F47" t="s">
+        <v>190</v>
+      </c>
+      <c r="G47" t="s">
+        <v>175</v>
+      </c>
+      <c r="H47" t="s">
+        <v>173</v>
+      </c>
+      <c r="I47" t="s">
+        <v>192</v>
+      </c>
+      <c r="J47" t="s">
+        <v>183</v>
+      </c>
+      <c r="K47" t="b">
+        <v>0</v>
+      </c>
+      <c r="L47" t="s">
+        <v>180</v>
+      </c>
+      <c r="M47" t="s">
+        <v>176</v>
+      </c>
+      <c r="N47" t="s">
+        <v>177</v>
+      </c>
+      <c r="O47" t="s">
+        <v>194</v>
+      </c>
+      <c r="P47" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>15</v>
+      </c>
+      <c r="R47" t="s">
+        <v>129</v>
+      </c>
+      <c r="S47" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrected annotations from 32499527.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45B5BB3B-DAC7-4484-BB79-219AE9DEB743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27232C86-856F-40E4-9447-20F326E0937E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="202">
   <si>
     <t>PMID</t>
   </si>
@@ -570,24 +570,21 @@
     <t>antiphage; RNA polymerase inihibition</t>
   </si>
   <si>
+    <t>Fill</t>
+  </si>
+  <si>
     <t>Cloned_into_organism</t>
   </si>
   <si>
     <t>Did_structural_validation</t>
   </si>
   <si>
-    <t>No human homology; claim is there but evidence is absent</t>
-  </si>
-  <si>
     <t>Lutibacter oricola</t>
   </si>
   <si>
     <t>A0A1H3CMF9</t>
   </si>
   <si>
-    <t>Authors claim human homology but provide no evidence; BLASTp of AA sequence and 30 to 60% identity filter yields no human matches</t>
-  </si>
-  <si>
     <t>From fig 1 description: "Homologues of human viperin are shown in red, genes annotated as nucleotide kinase are brown, genes known to be involved in defence are yellow and genes with mobile genetic elements are dark grey"; "We first performed a profile-based search for viperin homologues in a database of more than 38,000 bacterial and archaeal genomes. This search yielded 1,724 genes (1,112 non-redundant sequences) homologous to the human viperin gene (RSAD2)"</t>
   </si>
   <si>
@@ -619,6 +616,30 @@
   </si>
   <si>
     <t>T7 plaque assay; mutation assay</t>
+  </si>
+  <si>
+    <t>Template</t>
+  </si>
+  <si>
+    <t>Annotations</t>
+  </si>
+  <si>
+    <t>MAYKVNLHITQKCNYACKYCFAHFDHHNDLTLGQWKHIIDNLKTSGLVDAINFAGGEPVLHRDFAAIVNYAYDQGFKLSIITNGSLMLNPKLMPPELFAKFDTLGISVDSINPKTLIALGACNNSQEVLSYDKLSHLITLARSVNPTIRIKLNTVITNLNADEDLTIIGQELDIARWKMLRMKLFIHEGFNNAPLLVSQADFDGFVERHAEVSHDIVPENDLTRSYIMVDNQGRLLDDETEEYKVVGSLLAEDFGTVFDRYHFDEATYASRYAG</t>
+  </si>
+  <si>
+    <t>vip6</t>
+  </si>
+  <si>
+    <t>A0A1H0NKS3</t>
+  </si>
+  <si>
+    <t>Selenomonas ruminantium</t>
+  </si>
+  <si>
+    <t>J0S9F5</t>
+  </si>
+  <si>
+    <t>Methanofollis liminatans</t>
   </si>
 </sst>
 </file>
@@ -1485,7 +1506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:S47"/>
+  <dimension ref="A1:S60"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="17.6328125" customWidth="1"/>
@@ -1516,7 +1537,7 @@
         <v>92</v>
       </c>
       <c r="F1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G1" t="s">
         <v>97</v>
@@ -1525,7 +1546,7 @@
         <v>96</v>
       </c>
       <c r="I1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J1" t="s">
         <v>84</v>
@@ -1546,10 +1567,10 @@
         <v>8</v>
       </c>
       <c r="P1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Q1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="R1" t="s">
         <v>126</v>
@@ -2870,10 +2891,10 @@
         <v>15</v>
       </c>
       <c r="G24" t="s">
-        <v>15</v>
+        <v>131</v>
       </c>
       <c r="H24" t="s">
-        <v>15</v>
+        <v>133</v>
       </c>
       <c r="I24" t="s">
         <v>15</v>
@@ -2988,10 +3009,10 @@
         <v>15</v>
       </c>
       <c r="G26" t="s">
-        <v>15</v>
+        <v>159</v>
       </c>
       <c r="H26" t="s">
-        <v>15</v>
+        <v>165</v>
       </c>
       <c r="I26" t="s">
         <v>15</v>
@@ -3106,10 +3127,10 @@
         <v>15</v>
       </c>
       <c r="G28" t="s">
-        <v>15</v>
+        <v>160</v>
       </c>
       <c r="H28" t="s">
-        <v>15</v>
+        <v>166</v>
       </c>
       <c r="I28" t="s">
         <v>15</v>
@@ -3224,10 +3245,10 @@
         <v>15</v>
       </c>
       <c r="G30" t="s">
-        <v>15</v>
+        <v>161</v>
       </c>
       <c r="H30" t="s">
-        <v>15</v>
+        <v>170</v>
       </c>
       <c r="I30" t="s">
         <v>15</v>
@@ -3342,10 +3363,10 @@
         <v>15</v>
       </c>
       <c r="G32" t="s">
-        <v>15</v>
+        <v>162</v>
       </c>
       <c r="H32" t="s">
-        <v>15</v>
+        <v>167</v>
       </c>
       <c r="I32" t="s">
         <v>15</v>
@@ -3460,10 +3481,10 @@
         <v>15</v>
       </c>
       <c r="G34" t="s">
-        <v>15</v>
+        <v>163</v>
       </c>
       <c r="H34" t="s">
-        <v>15</v>
+        <v>169</v>
       </c>
       <c r="I34" t="s">
         <v>15</v>
@@ -3560,28 +3581,28 @@
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A36">
-        <v>40705877</v>
+        <v>32499527</v>
       </c>
       <c r="B36" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="C36" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="D36" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E36" t="s">
-        <v>15</v>
+        <v>144</v>
       </c>
       <c r="F36" t="s">
         <v>15</v>
       </c>
       <c r="G36" t="s">
-        <v>131</v>
+        <v>164</v>
       </c>
       <c r="H36" t="s">
-        <v>133</v>
+        <v>168</v>
       </c>
       <c r="I36" t="s">
         <v>15</v>
@@ -3590,10 +3611,10 @@
         <v>15</v>
       </c>
       <c r="K36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L36" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="M36" t="s">
         <v>15</v>
@@ -3602,19 +3623,19 @@
         <v>15</v>
       </c>
       <c r="O36" t="s">
-        <v>15</v>
+        <v>148</v>
       </c>
       <c r="P36" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q36" t="s">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="Q36" t="b">
+        <v>1</v>
       </c>
       <c r="R36" t="s">
         <v>128</v>
       </c>
       <c r="S36" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.35">
@@ -3625,10 +3646,10 @@
         <v>130</v>
       </c>
       <c r="C37" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D37" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E37" t="s">
         <v>15</v>
@@ -3655,25 +3676,25 @@
         <v>154</v>
       </c>
       <c r="M37" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="N37" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="O37" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="P37" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="Q37" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="R37" t="s">
         <v>128</v>
       </c>
       <c r="S37" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.35">
@@ -3684,10 +3705,10 @@
         <v>130</v>
       </c>
       <c r="C38" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D38" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E38" t="s">
         <v>15</v>
@@ -3714,25 +3735,25 @@
         <v>154</v>
       </c>
       <c r="M38" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="N38" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="O38" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="P38" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="Q38" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="R38" t="s">
         <v>128</v>
       </c>
       <c r="S38" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.35">
@@ -3743,13 +3764,13 @@
         <v>130</v>
       </c>
       <c r="C39" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D39" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E39" t="s">
-        <v>151</v>
+        <v>15</v>
       </c>
       <c r="F39" t="s">
         <v>15</v>
@@ -3770,7 +3791,7 @@
         <v>0</v>
       </c>
       <c r="L39" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="M39" t="s">
         <v>15</v>
@@ -3791,7 +3812,184 @@
         <v>128</v>
       </c>
       <c r="S39" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>40705877</v>
+      </c>
+      <c r="B40" t="s">
+        <v>130</v>
+      </c>
+      <c r="C40" t="s">
+        <v>140</v>
+      </c>
+      <c r="D40" t="s">
+        <v>138</v>
+      </c>
+      <c r="E40" t="s">
+        <v>151</v>
+      </c>
+      <c r="F40" t="s">
+        <v>15</v>
+      </c>
+      <c r="G40" t="s">
+        <v>131</v>
+      </c>
+      <c r="H40" t="s">
+        <v>133</v>
+      </c>
+      <c r="I40" t="s">
+        <v>15</v>
+      </c>
+      <c r="J40" t="s">
+        <v>15</v>
+      </c>
+      <c r="K40" t="b">
+        <v>0</v>
+      </c>
+      <c r="L40" t="s">
+        <v>152</v>
+      </c>
+      <c r="M40" t="s">
+        <v>15</v>
+      </c>
+      <c r="N40" t="s">
+        <v>15</v>
+      </c>
+      <c r="O40" t="s">
+        <v>15</v>
+      </c>
+      <c r="P40" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>15</v>
+      </c>
+      <c r="R40" t="s">
+        <v>128</v>
+      </c>
+      <c r="S40" t="s">
         <v>157</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>32937646</v>
+      </c>
+      <c r="B41" t="s">
+        <v>174</v>
+      </c>
+      <c r="C41" t="s">
+        <v>15</v>
+      </c>
+      <c r="D41" t="s">
+        <v>181</v>
+      </c>
+      <c r="E41" t="s">
+        <v>182</v>
+      </c>
+      <c r="F41" t="s">
+        <v>187</v>
+      </c>
+      <c r="G41" t="s">
+        <v>175</v>
+      </c>
+      <c r="H41" t="s">
+        <v>173</v>
+      </c>
+      <c r="I41" t="s">
+        <v>191</v>
+      </c>
+      <c r="J41" t="s">
+        <v>192</v>
+      </c>
+      <c r="K41" t="b">
+        <v>1</v>
+      </c>
+      <c r="L41" t="s">
+        <v>15</v>
+      </c>
+      <c r="M41" t="s">
+        <v>176</v>
+      </c>
+      <c r="N41" t="s">
+        <v>177</v>
+      </c>
+      <c r="O41" t="s">
+        <v>193</v>
+      </c>
+      <c r="P41" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>15</v>
+      </c>
+      <c r="R41" t="s">
+        <v>129</v>
+      </c>
+      <c r="S41" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>32937646</v>
+      </c>
+      <c r="B42" t="s">
+        <v>174</v>
+      </c>
+      <c r="C42" t="s">
+        <v>15</v>
+      </c>
+      <c r="D42" t="s">
+        <v>185</v>
+      </c>
+      <c r="E42" t="s">
+        <v>184</v>
+      </c>
+      <c r="F42" t="s">
+        <v>188</v>
+      </c>
+      <c r="G42" t="s">
+        <v>175</v>
+      </c>
+      <c r="H42" t="s">
+        <v>173</v>
+      </c>
+      <c r="I42" t="s">
+        <v>191</v>
+      </c>
+      <c r="J42" t="s">
+        <v>192</v>
+      </c>
+      <c r="K42" t="b">
+        <v>1</v>
+      </c>
+      <c r="L42" t="s">
+        <v>15</v>
+      </c>
+      <c r="M42" t="s">
+        <v>176</v>
+      </c>
+      <c r="N42" t="s">
+        <v>177</v>
+      </c>
+      <c r="O42" t="s">
+        <v>193</v>
+      </c>
+      <c r="P42" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>15</v>
+      </c>
+      <c r="R42" t="s">
+        <v>129</v>
+      </c>
+      <c r="S42" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.35">
@@ -3805,13 +4003,13 @@
         <v>15</v>
       </c>
       <c r="D43" t="s">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="E43" t="s">
-        <v>182</v>
+        <v>200</v>
       </c>
       <c r="F43" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G43" t="s">
         <v>175</v>
@@ -3820,10 +4018,10 @@
         <v>173</v>
       </c>
       <c r="I43" t="s">
+        <v>191</v>
+      </c>
+      <c r="J43" t="s">
         <v>192</v>
-      </c>
-      <c r="J43" t="s">
-        <v>193</v>
       </c>
       <c r="K43" t="b">
         <v>1</v>
@@ -3838,7 +4036,7 @@
         <v>177</v>
       </c>
       <c r="O43" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P43" t="s">
         <v>17</v>
@@ -3850,7 +4048,7 @@
         <v>129</v>
       </c>
       <c r="S43" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.35">
@@ -3861,16 +4059,16 @@
         <v>174</v>
       </c>
       <c r="C44" t="s">
-        <v>15</v>
+        <v>197</v>
       </c>
       <c r="D44" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="E44" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="F44" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="G44" t="s">
         <v>175</v>
@@ -3879,16 +4077,16 @@
         <v>173</v>
       </c>
       <c r="I44" t="s">
+        <v>191</v>
+      </c>
+      <c r="J44" t="s">
         <v>192</v>
       </c>
-      <c r="J44" t="s">
-        <v>183</v>
-      </c>
-      <c r="K44" t="b">
-        <v>0</v>
+      <c r="K44" t="s">
+        <v>178</v>
       </c>
       <c r="L44" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="M44" t="s">
         <v>176</v>
@@ -3897,7 +4095,7 @@
         <v>177</v>
       </c>
       <c r="O44" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P44" t="s">
         <v>17</v>
@@ -3909,66 +4107,67 @@
         <v>129</v>
       </c>
       <c r="S44" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A47">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A57">
         <v>32937646</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B57" t="s">
         <v>174</v>
       </c>
-      <c r="C47" t="s">
-        <v>15</v>
-      </c>
-      <c r="D47" t="s">
-        <v>186</v>
-      </c>
-      <c r="E47" t="s">
-        <v>185</v>
-      </c>
-      <c r="F47" t="s">
-        <v>190</v>
-      </c>
-      <c r="G47" t="s">
+      <c r="C57" t="s">
+        <v>15</v>
+      </c>
+      <c r="G57" t="s">
         <v>175</v>
       </c>
-      <c r="H47" t="s">
+      <c r="H57" t="s">
         <v>173</v>
       </c>
-      <c r="I47" t="s">
+      <c r="I57" t="s">
+        <v>191</v>
+      </c>
+      <c r="J57" t="s">
         <v>192</v>
       </c>
-      <c r="J47" t="s">
+      <c r="K57" t="s">
+        <v>178</v>
+      </c>
+      <c r="L57" t="s">
+        <v>178</v>
+      </c>
+      <c r="M57" t="s">
+        <v>176</v>
+      </c>
+      <c r="N57" t="s">
+        <v>177</v>
+      </c>
+      <c r="O57" t="s">
+        <v>193</v>
+      </c>
+      <c r="P57" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>15</v>
+      </c>
+      <c r="R57" t="s">
+        <v>129</v>
+      </c>
+      <c r="S57" t="s">
         <v>183</v>
       </c>
-      <c r="K47" t="b">
-        <v>0</v>
-      </c>
-      <c r="L47" t="s">
-        <v>180</v>
-      </c>
-      <c r="M47" t="s">
-        <v>176</v>
-      </c>
-      <c r="N47" t="s">
-        <v>177</v>
-      </c>
-      <c r="O47" t="s">
-        <v>194</v>
-      </c>
-      <c r="P47" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q47" t="s">
-        <v>15</v>
-      </c>
-      <c r="R47" t="s">
-        <v>129</v>
-      </c>
-      <c r="S47" t="s">
-        <v>184</v>
+    </row>
+    <row r="60" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Second round of extractions for PMID 32937646.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27232C86-856F-40E4-9447-20F326E0937E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA7B06C-5041-4D3F-B693-9386F33872CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="229">
   <si>
     <t>PMID</t>
   </si>
@@ -640,6 +640,87 @@
   </si>
   <si>
     <t>Methanofollis liminatans</t>
+  </si>
+  <si>
+    <t>vip8</t>
+  </si>
+  <si>
+    <t>MHNHNKIANKELVVNWHITEACNYRCGYCFAKWGKQKGELIQDVASISQLMDAISGLPAVLNQMHAANFEGVRLNLVGGETFLNYRKIKEVVKQAKKRGLKLSAITNGSRINNDFINLIANNFASIGFSVDSVDNSTNLNIGRVEKNAVMNPEKIIHTIASIRAINPKIEIKVNTVVSDLNKSEDLSDFIGQVMPNKWKIFKVLPVVANHHLISEEQFTRFLRRHQRFGEIIYAEDNTEMVDSYIMIDPIGRFFQNSDFNNGYYYSRPILQVGIHQAFNEINFNANKFYSRYKRASLN</t>
+  </si>
+  <si>
+    <t>Psychrobacter lutiphocae</t>
+  </si>
+  <si>
+    <t>P0DW49</t>
+  </si>
+  <si>
+    <t>D5EID4</t>
+  </si>
+  <si>
+    <t>vip15</t>
+  </si>
+  <si>
+    <t>Coraliomargarita akajimensis</t>
+  </si>
+  <si>
+    <t>MKPAIPPTINLHTIRACNYGCKYCFAGFQDCDTGVMPQADLHEILRQFAATTGMAIHPAKVNFAGGEPMLSPTFVEDICYAKSLGLTTSLVTNGSLLSERLLDKLSGQLDLLTISIDSLKPGTNRAIGRTNRQNPLTVSEYLDRILKARTRGITVKLNTVVNRLNLDEDMTDFIREAQPIRWKLFKVLKIQNENSAHFDSWAIRDEEFVHFVERHRKVESSGVTLVPESNEQMYGTYGIISPDGRFIDNSQGTHRYSPRIVDVGITQAFADVNFSMAGFQQRGGIYSIKRSTTNRSLQTSALHPKRELTK</t>
+  </si>
+  <si>
+    <t>Methanoplanus limicola</t>
+  </si>
+  <si>
+    <t>H1Z1K5</t>
+  </si>
+  <si>
+    <t>MPMHSTIKSVNWHITPRCNYRCRFCFAQNFHDGTVPYDKGLEILEILADAGMTKINFAGGEPLLHPGILDYCRESKKLGMTVSITTNGSKLNPSKIRKMAGIVDWIGLSIDSSLDTVEAELGRGTGNHVSNCLESAIYLHQAGIKLKVNTCVTALTFQENMIPLIRMLNPDRWKVLQMMHIDGENDFARDLEISAGDFRYFVERHRNVLLENGTSPVFESADDMESSYFMLTPGGFVKSDAGRKVTLYPLDEVIEKGIDNFVSEMKYQER</t>
+  </si>
+  <si>
+    <t>P0DW52</t>
+  </si>
+  <si>
+    <t>vip21</t>
+  </si>
+  <si>
+    <t>Lewinella persica</t>
+  </si>
+  <si>
+    <t>MTTPSFIPSVNFHLIKPCNMGCKYCFARFNDVASKSLTRGGLPKEDALAVVSALADFGFEKITFAGGEPTLYPWLTDVIELAKNKGMTTMLVTNGSRLNEAFYLRHAGLLDWITVSIDSLSVGTNLAIGRAKHGNQVFAREDYEVIAAMIHDYSYRLKINTVVSRYNHEEDMNDFIAHAKPERWKVFQALPIVGENDEYLEEFEITAEEFQQFLGRHGSQAKLVKENNDEMRGSYAMVDPKGCFFTNVNGQLEASSPILTVGCDAALREMNYDLTKFHDRGGRYDW</t>
+  </si>
+  <si>
+    <t>vip47</t>
+  </si>
+  <si>
+    <t>A0A1S1YUU1</t>
+  </si>
+  <si>
+    <t>Flammeovirga pacifica</t>
+  </si>
+  <si>
+    <t>MNKLVSGNNIIPSVNFHLWEPCNMRCKFCFAKFQDVKSTILPKGHLKKEQTLEIVEQLAEYGFQKITFVGGEPTLCPWISELIKKANLLGMTTMIVTNGSNLSKDFLVQNQSYLDWITLSIDSINSSTNKVVGRSTNSIHPDRIYYNQLIQTIYEYGYRLKINTVVTKANLNEDLNDFVNDAKPERWKVFQVLPVRGQNDNDIDELLISEKEFNEYVNRHSKNKFLITETNTDMTNTYVMVDPAGRFFNNQNGNYMYSDHILEVGVQKAFEEMGYNYDKFIDRKGIYQWK</t>
+  </si>
+  <si>
+    <t>vip50</t>
+  </si>
+  <si>
+    <t>Thermoplasmatales archaeon</t>
+  </si>
+  <si>
+    <t>MNTETTSVRKFRSANIHIYGKCNYRCEHCFDRCLTKNYMRPSDWVDTLTFLKEYGVEKINLAGGEPTLYPFLDQMCYLVKGMGFKLSIVSNGSLITEDWMARMEGVVDWIGLSIDSIDEADEIQIGRGRGGHLENIVQVADMAHRHGIKVKLNITVVRRSWMKDFRPFIEKVRPERVKCFRALTLKNANDDVPDTWSITDKQFEDFRRRHEDIGCIVFEDNEDMVSSYVMFDPMGRWMVDSGYEKRFISFEVLRREGLDREVDVEKYFGR</t>
+  </si>
+  <si>
+    <t>A0A110A2W7</t>
+  </si>
+  <si>
+    <t>vip56</t>
+  </si>
+  <si>
+    <t>Fibrobacter sp.</t>
+  </si>
+  <si>
+    <t>A0A1M7D0R2</t>
+  </si>
+  <si>
+    <t>MNIKTIVINWHITESCNYKCKYCFAKWNRVKEIWTNPDNVRKILENLKSIRLEDCLFTQKRLNIVGGEPILQQERLWQVIKMAHEMDFEISIITNGSHLEYICPFVHLISQVGVSIDSFDHKTNVRIGRECNGKTISFQQLKEKLEELRTLNPGLNIKINTVVNEYNFNEILVDRMAELKIDKWKILRQLPFDGKEGISDFKFNTFLFNNLKEEKMPKKDPLSNFLAAFSAPQKQNNVIFVEDNDVMTESYLMIAPDGRLFQNGHKEYEYSHPLTEISIDEALEEINFDQEKFNNRYENYATEEAKYRMEEFFLMNEYEDVSFDCCCPFGDKD</t>
   </si>
 </sst>
 </file>
@@ -1506,7 +1587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:S60"/>
+  <dimension ref="A1:S70"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="17.6328125" customWidth="1"/>
@@ -4082,11 +4163,11 @@
       <c r="J44" t="s">
         <v>192</v>
       </c>
-      <c r="K44" t="s">
-        <v>178</v>
+      <c r="K44" t="b">
+        <v>1</v>
       </c>
       <c r="L44" t="s">
-        <v>178</v>
+        <v>15</v>
       </c>
       <c r="M44" t="s">
         <v>176</v>
@@ -4107,6 +4188,419 @@
         <v>129</v>
       </c>
       <c r="S44" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>32937646</v>
+      </c>
+      <c r="B45" t="s">
+        <v>174</v>
+      </c>
+      <c r="C45" t="s">
+        <v>202</v>
+      </c>
+      <c r="D45" t="s">
+        <v>204</v>
+      </c>
+      <c r="E45" t="s">
+        <v>205</v>
+      </c>
+      <c r="F45" t="s">
+        <v>203</v>
+      </c>
+      <c r="G45" t="s">
+        <v>175</v>
+      </c>
+      <c r="H45" t="s">
+        <v>173</v>
+      </c>
+      <c r="I45" t="s">
+        <v>191</v>
+      </c>
+      <c r="J45" t="s">
+        <v>192</v>
+      </c>
+      <c r="K45" t="b">
+        <v>1</v>
+      </c>
+      <c r="L45" t="s">
+        <v>15</v>
+      </c>
+      <c r="M45" t="s">
+        <v>176</v>
+      </c>
+      <c r="N45" t="s">
+        <v>177</v>
+      </c>
+      <c r="O45" t="s">
+        <v>193</v>
+      </c>
+      <c r="P45" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>15</v>
+      </c>
+      <c r="R45" t="s">
+        <v>129</v>
+      </c>
+      <c r="S45" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>32937646</v>
+      </c>
+      <c r="B46" t="s">
+        <v>174</v>
+      </c>
+      <c r="C46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D46" t="s">
+        <v>208</v>
+      </c>
+      <c r="E46" t="s">
+        <v>206</v>
+      </c>
+      <c r="F46" t="s">
+        <v>209</v>
+      </c>
+      <c r="G46" t="s">
+        <v>175</v>
+      </c>
+      <c r="H46" t="s">
+        <v>173</v>
+      </c>
+      <c r="I46" t="s">
+        <v>191</v>
+      </c>
+      <c r="J46" t="s">
+        <v>192</v>
+      </c>
+      <c r="K46" t="b">
+        <v>1</v>
+      </c>
+      <c r="L46" t="s">
+        <v>15</v>
+      </c>
+      <c r="M46" t="s">
+        <v>176</v>
+      </c>
+      <c r="N46" t="s">
+        <v>177</v>
+      </c>
+      <c r="O46" t="s">
+        <v>193</v>
+      </c>
+      <c r="P46" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>15</v>
+      </c>
+      <c r="R46" t="s">
+        <v>129</v>
+      </c>
+      <c r="S46" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>32937646</v>
+      </c>
+      <c r="B47" t="s">
+        <v>174</v>
+      </c>
+      <c r="C47" t="s">
+        <v>15</v>
+      </c>
+      <c r="D47" t="s">
+        <v>210</v>
+      </c>
+      <c r="E47" t="s">
+        <v>211</v>
+      </c>
+      <c r="F47" t="s">
+        <v>212</v>
+      </c>
+      <c r="G47" t="s">
+        <v>175</v>
+      </c>
+      <c r="H47" t="s">
+        <v>173</v>
+      </c>
+      <c r="I47" t="s">
+        <v>191</v>
+      </c>
+      <c r="J47" t="s">
+        <v>192</v>
+      </c>
+      <c r="K47" t="b">
+        <v>1</v>
+      </c>
+      <c r="L47" t="s">
+        <v>15</v>
+      </c>
+      <c r="M47" t="s">
+        <v>176</v>
+      </c>
+      <c r="N47" t="s">
+        <v>177</v>
+      </c>
+      <c r="O47" t="s">
+        <v>193</v>
+      </c>
+      <c r="P47" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>15</v>
+      </c>
+      <c r="R47" t="s">
+        <v>129</v>
+      </c>
+      <c r="S47" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>32937646</v>
+      </c>
+      <c r="B48" t="s">
+        <v>174</v>
+      </c>
+      <c r="C48" t="s">
+        <v>214</v>
+      </c>
+      <c r="D48" t="s">
+        <v>215</v>
+      </c>
+      <c r="E48" t="s">
+        <v>213</v>
+      </c>
+      <c r="F48" t="s">
+        <v>216</v>
+      </c>
+      <c r="G48" t="s">
+        <v>175</v>
+      </c>
+      <c r="H48" t="s">
+        <v>173</v>
+      </c>
+      <c r="I48" t="s">
+        <v>191</v>
+      </c>
+      <c r="J48" t="s">
+        <v>192</v>
+      </c>
+      <c r="K48" t="b">
+        <v>1</v>
+      </c>
+      <c r="L48" t="s">
+        <v>15</v>
+      </c>
+      <c r="M48" t="s">
+        <v>176</v>
+      </c>
+      <c r="N48" t="s">
+        <v>177</v>
+      </c>
+      <c r="O48" t="s">
+        <v>193</v>
+      </c>
+      <c r="P48" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>15</v>
+      </c>
+      <c r="R48" t="s">
+        <v>129</v>
+      </c>
+      <c r="S48" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>32937646</v>
+      </c>
+      <c r="B49" t="s">
+        <v>174</v>
+      </c>
+      <c r="C49" t="s">
+        <v>217</v>
+      </c>
+      <c r="D49" t="s">
+        <v>219</v>
+      </c>
+      <c r="E49" t="s">
+        <v>218</v>
+      </c>
+      <c r="F49" t="s">
+        <v>220</v>
+      </c>
+      <c r="G49" t="s">
+        <v>175</v>
+      </c>
+      <c r="H49" t="s">
+        <v>173</v>
+      </c>
+      <c r="I49" t="s">
+        <v>191</v>
+      </c>
+      <c r="J49" t="s">
+        <v>192</v>
+      </c>
+      <c r="K49" t="b">
+        <v>1</v>
+      </c>
+      <c r="L49" t="s">
+        <v>15</v>
+      </c>
+      <c r="M49" t="s">
+        <v>176</v>
+      </c>
+      <c r="N49" t="s">
+        <v>177</v>
+      </c>
+      <c r="O49" t="s">
+        <v>193</v>
+      </c>
+      <c r="P49" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>15</v>
+      </c>
+      <c r="R49" t="s">
+        <v>129</v>
+      </c>
+      <c r="S49" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>32937646</v>
+      </c>
+      <c r="B50" t="s">
+        <v>174</v>
+      </c>
+      <c r="C50" t="s">
+        <v>221</v>
+      </c>
+      <c r="D50" t="s">
+        <v>222</v>
+      </c>
+      <c r="E50" t="s">
+        <v>224</v>
+      </c>
+      <c r="F50" t="s">
+        <v>223</v>
+      </c>
+      <c r="G50" t="s">
+        <v>175</v>
+      </c>
+      <c r="H50" t="s">
+        <v>173</v>
+      </c>
+      <c r="I50" t="s">
+        <v>191</v>
+      </c>
+      <c r="J50" t="s">
+        <v>192</v>
+      </c>
+      <c r="K50" t="b">
+        <v>1</v>
+      </c>
+      <c r="L50" t="s">
+        <v>15</v>
+      </c>
+      <c r="M50" t="s">
+        <v>176</v>
+      </c>
+      <c r="N50" t="s">
+        <v>177</v>
+      </c>
+      <c r="O50" t="s">
+        <v>193</v>
+      </c>
+      <c r="P50" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>15</v>
+      </c>
+      <c r="R50" t="s">
+        <v>129</v>
+      </c>
+      <c r="S50" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>32937646</v>
+      </c>
+      <c r="B51" t="s">
+        <v>174</v>
+      </c>
+      <c r="C51" t="s">
+        <v>225</v>
+      </c>
+      <c r="D51" t="s">
+        <v>226</v>
+      </c>
+      <c r="E51" t="s">
+        <v>227</v>
+      </c>
+      <c r="F51" t="s">
+        <v>228</v>
+      </c>
+      <c r="G51" t="s">
+        <v>175</v>
+      </c>
+      <c r="H51" t="s">
+        <v>173</v>
+      </c>
+      <c r="I51" t="s">
+        <v>191</v>
+      </c>
+      <c r="J51" t="s">
+        <v>192</v>
+      </c>
+      <c r="K51" t="b">
+        <v>1</v>
+      </c>
+      <c r="L51" t="s">
+        <v>15</v>
+      </c>
+      <c r="M51" t="s">
+        <v>176</v>
+      </c>
+      <c r="N51" t="s">
+        <v>177</v>
+      </c>
+      <c r="O51" t="s">
+        <v>193</v>
+      </c>
+      <c r="P51" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>15</v>
+      </c>
+      <c r="R51" t="s">
+        <v>129</v>
+      </c>
+      <c r="S51" t="s">
         <v>183</v>
       </c>
     </row>
@@ -4123,7 +4617,7 @@
         <v>174</v>
       </c>
       <c r="C57" t="s">
-        <v>15</v>
+        <v>178</v>
       </c>
       <c r="G57" t="s">
         <v>175</v>
@@ -4138,9 +4632,6 @@
         <v>192</v>
       </c>
       <c r="K57" t="s">
-        <v>178</v>
-      </c>
-      <c r="L57" t="s">
         <v>178</v>
       </c>
       <c r="M57" t="s">
@@ -4168,6 +4659,194 @@
     <row r="60" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>195</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>32937646</v>
+      </c>
+      <c r="B61" t="s">
+        <v>174</v>
+      </c>
+      <c r="C61" t="s">
+        <v>178</v>
+      </c>
+      <c r="G61" t="s">
+        <v>175</v>
+      </c>
+      <c r="H61" t="s">
+        <v>173</v>
+      </c>
+      <c r="I61" t="s">
+        <v>191</v>
+      </c>
+      <c r="J61" t="s">
+        <v>192</v>
+      </c>
+      <c r="K61" t="s">
+        <v>178</v>
+      </c>
+      <c r="M61" t="s">
+        <v>176</v>
+      </c>
+      <c r="N61" t="s">
+        <v>177</v>
+      </c>
+      <c r="O61" t="s">
+        <v>193</v>
+      </c>
+      <c r="P61" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>15</v>
+      </c>
+      <c r="R61" t="s">
+        <v>129</v>
+      </c>
+      <c r="S61" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>32937646</v>
+      </c>
+      <c r="B64" t="s">
+        <v>174</v>
+      </c>
+      <c r="C64" t="s">
+        <v>178</v>
+      </c>
+      <c r="G64" t="s">
+        <v>175</v>
+      </c>
+      <c r="H64" t="s">
+        <v>173</v>
+      </c>
+      <c r="I64" t="s">
+        <v>191</v>
+      </c>
+      <c r="J64" t="s">
+        <v>192</v>
+      </c>
+      <c r="K64" t="s">
+        <v>178</v>
+      </c>
+      <c r="M64" t="s">
+        <v>176</v>
+      </c>
+      <c r="N64" t="s">
+        <v>177</v>
+      </c>
+      <c r="O64" t="s">
+        <v>193</v>
+      </c>
+      <c r="P64" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q64" t="s">
+        <v>15</v>
+      </c>
+      <c r="R64" t="s">
+        <v>129</v>
+      </c>
+      <c r="S64" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="67" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>32937646</v>
+      </c>
+      <c r="B67" t="s">
+        <v>174</v>
+      </c>
+      <c r="C67" t="s">
+        <v>178</v>
+      </c>
+      <c r="G67" t="s">
+        <v>175</v>
+      </c>
+      <c r="H67" t="s">
+        <v>173</v>
+      </c>
+      <c r="I67" t="s">
+        <v>191</v>
+      </c>
+      <c r="J67" t="s">
+        <v>192</v>
+      </c>
+      <c r="K67" t="s">
+        <v>178</v>
+      </c>
+      <c r="M67" t="s">
+        <v>176</v>
+      </c>
+      <c r="N67" t="s">
+        <v>177</v>
+      </c>
+      <c r="O67" t="s">
+        <v>193</v>
+      </c>
+      <c r="P67" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q67" t="s">
+        <v>15</v>
+      </c>
+      <c r="R67" t="s">
+        <v>129</v>
+      </c>
+      <c r="S67" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="70" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>32937646</v>
+      </c>
+      <c r="B70" t="s">
+        <v>174</v>
+      </c>
+      <c r="C70" t="s">
+        <v>178</v>
+      </c>
+      <c r="G70" t="s">
+        <v>175</v>
+      </c>
+      <c r="H70" t="s">
+        <v>173</v>
+      </c>
+      <c r="I70" t="s">
+        <v>191</v>
+      </c>
+      <c r="J70" t="s">
+        <v>192</v>
+      </c>
+      <c r="K70" t="s">
+        <v>178</v>
+      </c>
+      <c r="M70" t="s">
+        <v>176</v>
+      </c>
+      <c r="N70" t="s">
+        <v>177</v>
+      </c>
+      <c r="O70" t="s">
+        <v>193</v>
+      </c>
+      <c r="P70" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q70" t="s">
+        <v>15</v>
+      </c>
+      <c r="R70" t="s">
+        <v>129</v>
+      </c>
+      <c r="S70" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed round 3 of extractions from PMID 32937646.
</commit_message>
<xml_diff>
--- a/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
+++ b/lit_review_manual/bacterial_immuneSystem_goldStandard_manual.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\lit_review_manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA7B06C-5041-4D3F-B693-9386F33872CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{728F943E-37C1-4816-8E27-41DA44DCDB3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{496E9F6B-74A8-4433-8D34-1A5B1F540F7A}"/>
   </bookViews>
   <sheets>
     <sheet name="gold_standard_manual" sheetId="1" r:id="rId1"/>
-    <sheet name="notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,26 +33,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="215">
   <si>
     <t>PMID</t>
   </si>
   <si>
-    <t>Gene_name</t>
-  </si>
-  <si>
     <t>Include</t>
   </si>
   <si>
     <t>Inclusion_reason</t>
   </si>
   <si>
-    <t>Refseq_NCBI_accession</t>
-  </si>
-  <si>
-    <t>Uniprot_or_uniparc_accession</t>
-  </si>
-  <si>
     <t>Bacterial_species</t>
   </si>
   <si>
@@ -63,12 +53,6 @@
     <t>Functional_assay</t>
   </si>
   <si>
-    <t>Cloned_into_plasmid</t>
-  </si>
-  <si>
-    <t>Did_structural_validation?</t>
-  </si>
-  <si>
     <t>Function_in_bacteria</t>
   </si>
   <si>
@@ -108,48 +92,6 @@
     <t>Streptococcus pyogenes serotype M1</t>
   </si>
   <si>
-    <t>Data_source</t>
-  </si>
-  <si>
-    <t>Data_source_notes</t>
-  </si>
-  <si>
-    <t>2020_Bernheim.pdf</t>
-  </si>
-  <si>
-    <t>E. coli</t>
-  </si>
-  <si>
-    <t>Antiphage</t>
-  </si>
-  <si>
-    <t>Abortive infection</t>
-  </si>
-  <si>
-    <t>Plasmid defense</t>
-  </si>
-  <si>
-    <t># If coming from same paper, please make sure is same organism</t>
-  </si>
-  <si>
-    <t>Transposon defense</t>
-  </si>
-  <si>
-    <t>Extracellular infection signalling; Intracellular pathogen sensing</t>
-  </si>
-  <si>
-    <t>Pore-forming</t>
-  </si>
-  <si>
-    <t>Transmembrane domain</t>
-  </si>
-  <si>
-    <t>Intracellular pathogen sensing</t>
-  </si>
-  <si>
-    <t>Antiphage; Nuclease</t>
-  </si>
-  <si>
     <t>Paper_title</t>
   </si>
   <si>
@@ -570,9 +512,6 @@
     <t>antiphage; RNA polymerase inihibition</t>
   </si>
   <si>
-    <t>Fill</t>
-  </si>
-  <si>
     <t>Cloned_into_organism</t>
   </si>
   <si>
@@ -618,12 +557,6 @@
     <t>T7 plaque assay; mutation assay</t>
   </si>
   <si>
-    <t>Template</t>
-  </si>
-  <si>
-    <t>Annotations</t>
-  </si>
-  <si>
     <t>MAYKVNLHITQKCNYACKYCFAHFDHHNDLTLGQWKHIIDNLKTSGLVDAINFAGGEPVLHRDFAAIVNYAYDQGFKLSIITNGSLMLNPKLMPPELFAKFDTLGISVDSINPKTLIALGACNNSQEVLSYDKLSHLITLARSVNPTIRIKLNTVITNLNADEDLTIIGQELDIARWKMLRMKLFIHEGFNNAPLLVSQADFDGFVERHAEVSHDIVPENDLTRSYIMVDNQGRLLDDETEEYKVVGSLLAEDFGTVFDRYHFDEATYASRYAG</t>
   </si>
   <si>
@@ -721,6 +654,30 @@
   </si>
   <si>
     <t>MNIKTIVINWHITESCNYKCKYCFAKWNRVKEIWTNPDNVRKILENLKSIRLEDCLFTQKRLNIVGGEPILQQERLWQVIKMAHEMDFEISIITNGSHLEYICPFVHLISQVGVSIDSFDHKTNVRIGRECNGKTISFQQLKEKLEELRTLNPGLNIKINTVVNEYNFNEILVDRMAELKIDKWKILRQLPFDGKEGISDFKFNTFLFNNLKEEKMPKKDPLSNFLAAFSAPQKQNNVIFVEDNDVMTESYLMIAPDGRLFQNGHKEYEYSHPLTEISIDEALEEINFDQEKFNNRYENYATEEAKYRMEEFFLMNEYEDVSFDCCCPFGDKD</t>
+  </si>
+  <si>
+    <t>Pseudoalteromonas ulvae</t>
+  </si>
+  <si>
+    <t>vip58</t>
+  </si>
+  <si>
+    <t>A0A244CMP</t>
+  </si>
+  <si>
+    <t>MEIHMTSIQELVINFHMTEACNYRCGYCYATWQDNSSDTELHHASENIHSLLLKLADYFFADNSLRQTLKYQSVRINFAGGEPVMLGSRFIDAILFAKQLGFATSIITNGHLLSTVMLKKIAVHLDMLGISFDTGDYLIAQSIGRVDRKKSWLSPARVLDVVTQYRALNPKGKVKINTVVNAYNWRENLTQTITQLKPDKWKLLRVLPVYSKEMTVLQWQYESYVHKHQVHADVIVVEDNDDMWQSYLMINPEGRFYQNAGACKGLTYSPPVLEVGVEEALKYINFNAEAFSKRYQSIHLPLAMSAGA</t>
+  </si>
+  <si>
+    <t>vip60</t>
+  </si>
+  <si>
+    <t>Lacinutrix mariniflava</t>
+  </si>
+  <si>
+    <t>P0DW53</t>
+  </si>
+  <si>
+    <t>MKTKITLSGFAGTGKSTVGKRIQEQLNFEFVSVGNYSRQYAMEKYGLTINEFQEQCKAQPELDNEIDEKFRLECNSKENLVIDYRLGFHFIKNAFHVLLKVSDESASKRIRLANRSDEVTSTKAIQQRNQKMRDRFQDNYGVDFTNDKNYDLVIDTDDLTANEVADLIIEHYQKSNAVSKIPSVNFHLWQPCNMRCKFCFATFLDVKQEYVPKGHLPEDEALEVVRKIAAAGFEKITFAGGEPLLCKWLPKLIKTAKQLGMTTMIVTNGSKLTDSFLKENKAYLDWIAVSIDSLDEENNIKIGRAITGKKPLSKAFYYDLIDKIHQYGYGLKINTVVNKVNYKDNLASFIAKAKPKRWKVLQVLPIKGQNDNKIDAFKITDEEYANFLDTHKDVETIVPESNDEIKGSYVMVDPAGRFFDNAAGTHNYSKPILEVGIQEALKTMNYDLDKFLNRGGVYNWNTNKNQDLRKEEVSYE</t>
   </si>
 </sst>
 </file>
@@ -1587,7 +1544,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F713C0BE-76CC-4F2B-96EE-4618258E5622}">
-  <dimension ref="A1:S70"/>
+  <dimension ref="A1:S53"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="17.6328125" customWidth="1"/>
@@ -1606,58 +1563,58 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I1" t="s">
+        <v>170</v>
+      </c>
+      <c r="J1" t="s">
+        <v>65</v>
+      </c>
+      <c r="K1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L1" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H1" t="s">
-        <v>96</v>
-      </c>
-      <c r="I1" t="s">
-        <v>190</v>
-      </c>
-      <c r="J1" t="s">
-        <v>84</v>
-      </c>
-      <c r="K1" t="s">
-        <v>2</v>
-      </c>
-      <c r="L1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P1" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>160</v>
+      </c>
+      <c r="R1" t="s">
+        <v>107</v>
+      </c>
+      <c r="S1" t="s">
         <v>7</v>
-      </c>
-      <c r="N1" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" t="s">
-        <v>8</v>
-      </c>
-      <c r="P1" t="s">
-        <v>179</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>180</v>
-      </c>
-      <c r="R1" t="s">
-        <v>126</v>
-      </c>
-      <c r="S1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.35">
@@ -1665,58 +1622,58 @@
         <v>12110595</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J2" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="K2" t="b">
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="M2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N2" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="O2" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="P2" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="Q2" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="R2" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S2" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.35">
@@ -1724,58 +1681,58 @@
         <v>30787435</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="H3" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="I3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J3" t="s">
-        <v>119</v>
+        <v>100</v>
       </c>
       <c r="K3" t="b">
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="M3" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="N3" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="O3" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="P3" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="Q3" t="b">
         <v>1</v>
       </c>
       <c r="R3" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S3" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.35">
@@ -1783,58 +1740,58 @@
         <v>30787435</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="H4" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="I4" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J4" t="s">
-        <v>119</v>
+        <v>100</v>
       </c>
       <c r="K4" t="b">
         <v>1</v>
       </c>
       <c r="L4" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="M4" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="N4" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="O4" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="P4" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q4" t="b">
         <v>1</v>
       </c>
       <c r="R4" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S4" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.35">
@@ -1842,58 +1799,58 @@
         <v>30787435</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="E5" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="H5" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J5" t="s">
-        <v>119</v>
+        <v>100</v>
       </c>
       <c r="K5" t="b">
         <v>1</v>
       </c>
       <c r="L5" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="M5" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="N5" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="O5" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="P5" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q5" t="b">
         <v>1</v>
       </c>
       <c r="R5" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S5" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.35">
@@ -1901,58 +1858,58 @@
         <v>31695182</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="I6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J6" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="K6" t="b">
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M6" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="N6" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="O6" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="P6" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="Q6" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="R6" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S6" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.35">
@@ -1960,58 +1917,58 @@
         <v>31695182</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="I7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J7" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="K7" t="b">
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M7" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="N7" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="O7" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="P7" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="Q7" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="R7" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S7" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.35">
@@ -2019,58 +1976,58 @@
         <v>31695182</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="H8" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="I8" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J8" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="K8" t="b">
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M8" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="N8" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="O8" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="P8" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="Q8" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="R8" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S8" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.35">
@@ -2078,58 +2035,58 @@
         <v>31695182</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="I9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="K9" t="b">
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="N9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="O9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="P9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="Q9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="R9" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S9" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.35">
@@ -2137,58 +2094,58 @@
         <v>31932165</v>
       </c>
       <c r="B10" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="F10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K10" t="b">
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="M10" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="N10" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="O10" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="P10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q10" t="b">
         <v>1</v>
       </c>
       <c r="R10" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.35">
@@ -2196,58 +2153,58 @@
         <v>31932165</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="F11" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H11" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I11" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J11" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K11" t="b">
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="M11" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="N11" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="O11" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="P11" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q11" t="b">
         <v>1</v>
       </c>
       <c r="R11" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S11" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.35">
@@ -2255,58 +2212,58 @@
         <v>31932165</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="D12" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="E12" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="F12" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H12" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J12" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K12" t="b">
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="M12" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="N12" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="O12" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="P12" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
       </c>
       <c r="R12" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S12" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.35">
@@ -2314,58 +2271,58 @@
         <v>31932165</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="E13" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F13" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="H13" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="I13" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J13" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="K13" t="b">
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="M13" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="N13" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="O13" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="P13" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q13" t="b">
         <v>1</v>
       </c>
       <c r="R13" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S13" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.35">
@@ -2373,58 +2330,58 @@
         <v>31932165</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D14" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="E14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J14" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="K14" t="b">
         <v>0</v>
       </c>
       <c r="L14" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="M14" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="N14" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="O14" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="P14" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q14" t="b">
         <v>1</v>
       </c>
       <c r="R14" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S14" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.35">
@@ -2432,58 +2389,58 @@
         <v>32559405</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="D15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="F15" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="H15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="I15" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="K15" t="b">
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="N15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="O15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="P15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="Q15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="R15" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="S15" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.35">
@@ -2491,58 +2448,58 @@
         <v>32839535</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="D16" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E16" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="F16" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G16" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="H16" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="I16" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J16" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="K16" t="b">
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="M16" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="N16" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="O16" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P16" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S16" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.35">
@@ -2550,58 +2507,58 @@
         <v>39208803</v>
       </c>
       <c r="B17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" t="s">
         <v>95</v>
       </c>
-      <c r="C17" t="s">
-        <v>114</v>
-      </c>
       <c r="D17" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="E17" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="F17" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G17" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="H17" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="I17" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J17" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="K17" t="b">
         <v>0</v>
       </c>
       <c r="L17" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="M17" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="N17" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O17" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P17" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q17" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R17" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S17" t="s">
-        <v>118</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.35">
@@ -2609,58 +2566,58 @@
         <v>39208803</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="C18" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E18" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G18" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="H18" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I18" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J18" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K18" t="b">
         <v>0</v>
       </c>
       <c r="L18" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="M18" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="N18" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O18" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P18" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q18" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R18" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S18" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.35">
@@ -2668,58 +2625,58 @@
         <v>39208803</v>
       </c>
       <c r="B19" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F19" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G19" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="H19" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="I19" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J19" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="K19" t="b">
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="M19" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="N19" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O19" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P19" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q19" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R19" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S19" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.35">
@@ -2727,55 +2684,55 @@
         <v>39208803</v>
       </c>
       <c r="B20" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="E20" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="F20" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G20" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="H20" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="I20" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J20" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="K20" t="b">
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="M20" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="N20" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O20" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P20" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q20" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R20" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S20" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.35">
@@ -2783,55 +2740,55 @@
         <v>39208803</v>
       </c>
       <c r="B21" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="C21" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="E21" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="F21" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G21" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="H21" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="I21" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J21" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="K21" t="b">
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="M21" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="N21" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O21" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P21" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q21" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R21" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S21" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.35">
@@ -2839,58 +2796,58 @@
         <v>35164550</v>
       </c>
       <c r="B22" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="C22" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="D22" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="E22" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="F22" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G22" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H22" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I22" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J22" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K22" t="b">
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="M22" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="N22" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="O22" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="P22" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="Q22" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="R22" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S22" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.35">
@@ -2898,58 +2855,58 @@
         <v>40705877</v>
       </c>
       <c r="B23" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C23" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D23" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E23" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F23" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G23" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="H23" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="I23" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J23" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="K23" t="b">
         <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="M23" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="N23" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="O23" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P23" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q23" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R23" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S23" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.35">
@@ -2957,58 +2914,58 @@
         <v>32499527</v>
       </c>
       <c r="B24" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="C24" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D24" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E24" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F24" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G24" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="H24" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="I24" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J24" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K24" t="b">
         <v>1</v>
       </c>
       <c r="L24" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="M24" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N24" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O24" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="P24" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q24" t="b">
         <v>1</v>
       </c>
       <c r="R24" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S24" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.35">
@@ -3016,58 +2973,58 @@
         <v>40705877</v>
       </c>
       <c r="B25" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C25" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D25" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E25" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F25" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G25" t="s">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="H25" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="I25" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J25" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K25" t="b">
         <v>1</v>
       </c>
       <c r="L25" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="M25" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="N25" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="O25" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P25" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q25" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R25" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S25" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.35">
@@ -3075,58 +3032,58 @@
         <v>32499527</v>
       </c>
       <c r="B26" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="C26" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D26" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E26" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F26" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G26" t="s">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="H26" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="I26" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J26" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K26" t="b">
         <v>1</v>
       </c>
       <c r="L26" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="M26" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N26" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O26" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="P26" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q26" t="b">
         <v>1</v>
       </c>
       <c r="R26" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S26" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.35">
@@ -3134,58 +3091,58 @@
         <v>40705877</v>
       </c>
       <c r="B27" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C27" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D27" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E27" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F27" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G27" t="s">
-        <v>160</v>
+        <v>141</v>
       </c>
       <c r="H27" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
       <c r="I27" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J27" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K27" t="b">
         <v>1</v>
       </c>
       <c r="L27" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="M27" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="N27" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="O27" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P27" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q27" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R27" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S27" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.35">
@@ -3193,58 +3150,58 @@
         <v>32499527</v>
       </c>
       <c r="B28" t="s">
+        <v>128</v>
+      </c>
+      <c r="C28" t="s">
+        <v>124</v>
+      </c>
+      <c r="D28" t="s">
+        <v>118</v>
+      </c>
+      <c r="E28" t="s">
+        <v>125</v>
+      </c>
+      <c r="F28" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" t="s">
+        <v>141</v>
+      </c>
+      <c r="H28" t="s">
         <v>147</v>
       </c>
-      <c r="C28" t="s">
-        <v>143</v>
-      </c>
-      <c r="D28" t="s">
-        <v>137</v>
-      </c>
-      <c r="E28" t="s">
-        <v>144</v>
-      </c>
-      <c r="F28" t="s">
-        <v>15</v>
-      </c>
-      <c r="G28" t="s">
-        <v>160</v>
-      </c>
-      <c r="H28" t="s">
-        <v>166</v>
-      </c>
       <c r="I28" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J28" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K28" t="b">
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="M28" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N28" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O28" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="P28" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q28" t="b">
         <v>1</v>
       </c>
       <c r="R28" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S28" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.35">
@@ -3252,58 +3209,58 @@
         <v>40705877</v>
       </c>
       <c r="B29" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C29" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D29" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E29" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F29" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G29" t="s">
-        <v>161</v>
+        <v>142</v>
       </c>
       <c r="H29" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="I29" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J29" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K29" t="b">
         <v>1</v>
       </c>
       <c r="L29" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="M29" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="N29" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="O29" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P29" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q29" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R29" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S29" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.35">
@@ -3311,58 +3268,58 @@
         <v>32499527</v>
       </c>
       <c r="B30" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="C30" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D30" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E30" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F30" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G30" t="s">
-        <v>161</v>
+        <v>142</v>
       </c>
       <c r="H30" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="I30" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J30" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K30" t="b">
         <v>1</v>
       </c>
       <c r="L30" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="M30" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N30" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O30" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="P30" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q30" t="b">
         <v>1</v>
       </c>
       <c r="R30" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S30" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.35">
@@ -3370,58 +3327,58 @@
         <v>40705877</v>
       </c>
       <c r="B31" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C31" t="s">
+        <v>124</v>
+      </c>
+      <c r="D31" t="s">
+        <v>118</v>
+      </c>
+      <c r="E31" t="s">
+        <v>125</v>
+      </c>
+      <c r="F31" t="s">
+        <v>10</v>
+      </c>
+      <c r="G31" t="s">
         <v>143</v>
       </c>
-      <c r="D31" t="s">
-        <v>137</v>
-      </c>
-      <c r="E31" t="s">
-        <v>144</v>
-      </c>
-      <c r="F31" t="s">
-        <v>15</v>
-      </c>
-      <c r="G31" t="s">
-        <v>162</v>
-      </c>
       <c r="H31" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
       <c r="I31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K31" t="b">
         <v>1</v>
       </c>
       <c r="L31" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="M31" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="N31" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="O31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R31" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S31" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.35">
@@ -3429,58 +3386,58 @@
         <v>32499527</v>
       </c>
       <c r="B32" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="C32" t="s">
+        <v>124</v>
+      </c>
+      <c r="D32" t="s">
+        <v>118</v>
+      </c>
+      <c r="E32" t="s">
+        <v>125</v>
+      </c>
+      <c r="F32" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32" t="s">
         <v>143</v>
       </c>
-      <c r="D32" t="s">
-        <v>137</v>
-      </c>
-      <c r="E32" t="s">
-        <v>144</v>
-      </c>
-      <c r="F32" t="s">
-        <v>15</v>
-      </c>
-      <c r="G32" t="s">
-        <v>162</v>
-      </c>
       <c r="H32" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
       <c r="I32" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J32" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K32" t="b">
         <v>1</v>
       </c>
       <c r="L32" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="M32" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N32" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O32" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="P32" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q32" t="b">
         <v>1</v>
       </c>
       <c r="R32" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S32" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.35">
@@ -3488,58 +3445,58 @@
         <v>40705877</v>
       </c>
       <c r="B33" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C33" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D33" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E33" t="s">
+        <v>125</v>
+      </c>
+      <c r="F33" t="s">
+        <v>10</v>
+      </c>
+      <c r="G33" t="s">
         <v>144</v>
       </c>
-      <c r="F33" t="s">
-        <v>15</v>
-      </c>
-      <c r="G33" t="s">
-        <v>163</v>
-      </c>
       <c r="H33" t="s">
-        <v>169</v>
+        <v>150</v>
       </c>
       <c r="I33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K33" t="b">
         <v>1</v>
       </c>
       <c r="L33" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="M33" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="N33" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="O33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R33" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S33" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.35">
@@ -3547,58 +3504,58 @@
         <v>32499527</v>
       </c>
       <c r="B34" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="C34" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D34" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E34" t="s">
+        <v>125</v>
+      </c>
+      <c r="F34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" t="s">
         <v>144</v>
       </c>
-      <c r="F34" t="s">
-        <v>15</v>
-      </c>
-      <c r="G34" t="s">
-        <v>163</v>
-      </c>
       <c r="H34" t="s">
-        <v>169</v>
+        <v>150</v>
       </c>
       <c r="I34" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J34" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K34" t="b">
         <v>1</v>
       </c>
       <c r="L34" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="M34" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N34" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O34" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="P34" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q34" t="b">
         <v>1</v>
       </c>
       <c r="R34" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S34" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.35">
@@ -3606,58 +3563,58 @@
         <v>40705877</v>
       </c>
       <c r="B35" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C35" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D35" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E35" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G35" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="H35" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
       <c r="I35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K35" t="b">
         <v>1</v>
       </c>
       <c r="L35" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="M35" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="N35" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="O35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R35" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S35" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.35">
@@ -3665,58 +3622,58 @@
         <v>32499527</v>
       </c>
       <c r="B36" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="C36" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D36" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="E36" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F36" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G36" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="H36" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
       <c r="I36" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J36" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K36" t="b">
         <v>1</v>
       </c>
       <c r="L36" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="M36" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N36" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O36" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="P36" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q36" t="b">
         <v>1</v>
       </c>
       <c r="R36" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S36" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.35">
@@ -3724,58 +3681,58 @@
         <v>40705877</v>
       </c>
       <c r="B37" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C37" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="D37" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="E37" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F37" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G37" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="H37" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="I37" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J37" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K37" t="b">
         <v>0</v>
       </c>
       <c r="L37" t="s">
-        <v>154</v>
+        <v>135</v>
       </c>
       <c r="M37" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N37" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O37" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P37" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q37" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R37" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S37" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.35">
@@ -3783,58 +3740,58 @@
         <v>40705877</v>
       </c>
       <c r="B38" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C38" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
       <c r="D38" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="E38" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F38" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G38" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="H38" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="I38" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J38" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K38" t="b">
         <v>0</v>
       </c>
       <c r="L38" t="s">
-        <v>154</v>
+        <v>135</v>
       </c>
       <c r="M38" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="N38" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="O38" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="P38" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="Q38" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="R38" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S38" t="s">
-        <v>155</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.35">
@@ -3842,58 +3799,58 @@
         <v>40705877</v>
       </c>
       <c r="B39" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C39" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
       <c r="D39" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="E39" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F39" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G39" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="H39" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="I39" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J39" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K39" t="b">
         <v>0</v>
       </c>
       <c r="L39" t="s">
-        <v>154</v>
+        <v>135</v>
       </c>
       <c r="M39" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N39" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O39" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P39" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q39" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R39" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S39" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.35">
@@ -3901,58 +3858,58 @@
         <v>40705877</v>
       </c>
       <c r="B40" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C40" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
       <c r="D40" t="s">
-        <v>138</v>
+        <v>119</v>
       </c>
       <c r="E40" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
       <c r="F40" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G40" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="H40" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="I40" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J40" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K40" t="b">
         <v>0</v>
       </c>
       <c r="L40" t="s">
-        <v>152</v>
+        <v>133</v>
       </c>
       <c r="M40" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N40" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O40" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P40" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q40" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R40" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="S40" t="s">
-        <v>157</v>
+        <v>138</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.35">
@@ -3960,58 +3917,58 @@
         <v>32937646</v>
       </c>
       <c r="B41" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C41" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D41" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="E41" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
       <c r="F41" t="s">
-        <v>187</v>
+        <v>167</v>
       </c>
       <c r="G41" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H41" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I41" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J41" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K41" t="b">
         <v>1</v>
       </c>
       <c r="L41" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M41" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N41" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O41" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P41" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q41" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R41" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S41" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.35">
@@ -4019,58 +3976,58 @@
         <v>32937646</v>
       </c>
       <c r="B42" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C42" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D42" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="E42" t="s">
-        <v>184</v>
+        <v>164</v>
       </c>
       <c r="F42" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="G42" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H42" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I42" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J42" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K42" t="b">
         <v>1</v>
       </c>
       <c r="L42" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M42" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N42" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O42" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P42" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q42" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R42" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S42" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.35">
@@ -4078,58 +4035,58 @@
         <v>32937646</v>
       </c>
       <c r="B43" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C43" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="E43" t="s">
-        <v>200</v>
+        <v>178</v>
       </c>
       <c r="F43" t="s">
-        <v>189</v>
+        <v>169</v>
       </c>
       <c r="G43" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H43" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I43" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J43" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K43" t="b">
         <v>1</v>
       </c>
       <c r="L43" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M43" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N43" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O43" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P43" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q43" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R43" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S43" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.35">
@@ -4137,58 +4094,58 @@
         <v>32937646</v>
       </c>
       <c r="B44" t="s">
+        <v>155</v>
+      </c>
+      <c r="C44" t="s">
+        <v>175</v>
+      </c>
+      <c r="D44" t="s">
+        <v>177</v>
+      </c>
+      <c r="E44" t="s">
+        <v>176</v>
+      </c>
+      <c r="F44" t="s">
         <v>174</v>
       </c>
-      <c r="C44" t="s">
-        <v>197</v>
-      </c>
-      <c r="D44" t="s">
-        <v>199</v>
-      </c>
-      <c r="E44" t="s">
-        <v>198</v>
-      </c>
-      <c r="F44" t="s">
-        <v>196</v>
-      </c>
       <c r="G44" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H44" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I44" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J44" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K44" t="b">
         <v>1</v>
       </c>
       <c r="L44" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M44" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N44" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O44" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P44" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q44" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R44" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S44" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.35">
@@ -4196,58 +4153,58 @@
         <v>32937646</v>
       </c>
       <c r="B45" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C45" t="s">
-        <v>202</v>
+        <v>180</v>
       </c>
       <c r="D45" t="s">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="E45" t="s">
-        <v>205</v>
+        <v>183</v>
       </c>
       <c r="F45" t="s">
-        <v>203</v>
+        <v>181</v>
       </c>
       <c r="G45" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H45" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I45" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J45" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K45" t="b">
         <v>1</v>
       </c>
       <c r="L45" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M45" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N45" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O45" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P45" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q45" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R45" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S45" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.35">
@@ -4255,58 +4212,58 @@
         <v>32937646</v>
       </c>
       <c r="B46" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C46" t="s">
-        <v>207</v>
+        <v>185</v>
       </c>
       <c r="D46" t="s">
-        <v>208</v>
+        <v>186</v>
       </c>
       <c r="E46" t="s">
-        <v>206</v>
+        <v>184</v>
       </c>
       <c r="F46" t="s">
-        <v>209</v>
+        <v>187</v>
       </c>
       <c r="G46" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H46" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I46" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J46" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K46" t="b">
         <v>1</v>
       </c>
       <c r="L46" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M46" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N46" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O46" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P46" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q46" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R46" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S46" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.35">
@@ -4314,58 +4271,58 @@
         <v>32937646</v>
       </c>
       <c r="B47" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C47" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D47" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="E47" t="s">
-        <v>211</v>
+        <v>189</v>
       </c>
       <c r="F47" t="s">
-        <v>212</v>
+        <v>190</v>
       </c>
       <c r="G47" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H47" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I47" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J47" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K47" t="b">
         <v>1</v>
       </c>
       <c r="L47" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M47" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N47" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O47" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P47" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q47" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R47" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S47" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.35">
@@ -4373,58 +4330,58 @@
         <v>32937646</v>
       </c>
       <c r="B48" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C48" t="s">
-        <v>214</v>
+        <v>192</v>
       </c>
       <c r="D48" t="s">
-        <v>215</v>
+        <v>193</v>
       </c>
       <c r="E48" t="s">
-        <v>213</v>
+        <v>191</v>
       </c>
       <c r="F48" t="s">
-        <v>216</v>
+        <v>194</v>
       </c>
       <c r="G48" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H48" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I48" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J48" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K48" t="b">
         <v>1</v>
       </c>
       <c r="L48" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M48" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N48" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O48" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P48" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q48" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R48" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S48" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.35">
@@ -4432,58 +4389,58 @@
         <v>32937646</v>
       </c>
       <c r="B49" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C49" t="s">
-        <v>217</v>
+        <v>195</v>
       </c>
       <c r="D49" t="s">
-        <v>219</v>
+        <v>197</v>
       </c>
       <c r="E49" t="s">
-        <v>218</v>
+        <v>196</v>
       </c>
       <c r="F49" t="s">
-        <v>220</v>
+        <v>198</v>
       </c>
       <c r="G49" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H49" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I49" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J49" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K49" t="b">
         <v>1</v>
       </c>
       <c r="L49" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M49" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N49" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O49" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P49" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q49" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R49" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S49" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.35">
@@ -4491,58 +4448,58 @@
         <v>32937646</v>
       </c>
       <c r="B50" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C50" t="s">
-        <v>221</v>
+        <v>199</v>
       </c>
       <c r="D50" t="s">
-        <v>222</v>
+        <v>200</v>
       </c>
       <c r="E50" t="s">
-        <v>224</v>
+        <v>202</v>
       </c>
       <c r="F50" t="s">
-        <v>223</v>
+        <v>201</v>
       </c>
       <c r="G50" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H50" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I50" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J50" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K50" t="b">
         <v>1</v>
       </c>
       <c r="L50" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M50" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N50" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O50" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P50" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q50" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R50" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S50" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.35">
@@ -4550,502 +4507,180 @@
         <v>32937646</v>
       </c>
       <c r="B51" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C51" t="s">
-        <v>225</v>
+        <v>203</v>
       </c>
       <c r="D51" t="s">
-        <v>226</v>
+        <v>204</v>
       </c>
       <c r="E51" t="s">
-        <v>227</v>
+        <v>205</v>
       </c>
       <c r="F51" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="G51" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="H51" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="I51" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="J51" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K51" t="b">
         <v>1</v>
       </c>
       <c r="L51" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M51" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="N51" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="O51" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="P51" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q51" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R51" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="S51" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A57">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A52">
         <v>32937646</v>
       </c>
-      <c r="B57" t="s">
-        <v>174</v>
-      </c>
-      <c r="C57" t="s">
-        <v>178</v>
-      </c>
-      <c r="G57" t="s">
-        <v>175</v>
-      </c>
-      <c r="H57" t="s">
+      <c r="B52" t="s">
+        <v>155</v>
+      </c>
+      <c r="C52" t="s">
+        <v>208</v>
+      </c>
+      <c r="D52" t="s">
+        <v>207</v>
+      </c>
+      <c r="E52" t="s">
+        <v>209</v>
+      </c>
+      <c r="F52" t="s">
+        <v>210</v>
+      </c>
+      <c r="G52" t="s">
+        <v>156</v>
+      </c>
+      <c r="H52" t="s">
+        <v>154</v>
+      </c>
+      <c r="I52" t="s">
+        <v>171</v>
+      </c>
+      <c r="J52" t="s">
+        <v>172</v>
+      </c>
+      <c r="K52" t="b">
+        <v>1</v>
+      </c>
+      <c r="L52" t="s">
+        <v>10</v>
+      </c>
+      <c r="M52" t="s">
+        <v>157</v>
+      </c>
+      <c r="N52" t="s">
+        <v>158</v>
+      </c>
+      <c r="O52" t="s">
         <v>173</v>
       </c>
-      <c r="I57" t="s">
-        <v>191</v>
-      </c>
-      <c r="J57" t="s">
-        <v>192</v>
-      </c>
-      <c r="K57" t="s">
-        <v>178</v>
-      </c>
-      <c r="M57" t="s">
-        <v>176</v>
-      </c>
-      <c r="N57" t="s">
-        <v>177</v>
-      </c>
-      <c r="O57" t="s">
-        <v>193</v>
-      </c>
-      <c r="P57" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q57" t="s">
-        <v>15</v>
-      </c>
-      <c r="R57" t="s">
-        <v>129</v>
-      </c>
-      <c r="S57" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A61">
+      <c r="P52" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q52" t="s">
+        <v>10</v>
+      </c>
+      <c r="R52" t="s">
+        <v>110</v>
+      </c>
+      <c r="S52" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A53">
         <v>32937646</v>
       </c>
-      <c r="B61" t="s">
-        <v>174</v>
-      </c>
-      <c r="C61" t="s">
-        <v>178</v>
-      </c>
-      <c r="G61" t="s">
-        <v>175</v>
-      </c>
-      <c r="H61" t="s">
+      <c r="B53" t="s">
+        <v>155</v>
+      </c>
+      <c r="C53" t="s">
+        <v>211</v>
+      </c>
+      <c r="D53" t="s">
+        <v>212</v>
+      </c>
+      <c r="E53" t="s">
+        <v>213</v>
+      </c>
+      <c r="F53" t="s">
+        <v>214</v>
+      </c>
+      <c r="G53" t="s">
+        <v>156</v>
+      </c>
+      <c r="H53" t="s">
+        <v>154</v>
+      </c>
+      <c r="I53" t="s">
+        <v>171</v>
+      </c>
+      <c r="J53" t="s">
+        <v>172</v>
+      </c>
+      <c r="K53" t="b">
+        <v>1</v>
+      </c>
+      <c r="L53" t="s">
+        <v>10</v>
+      </c>
+      <c r="M53" t="s">
+        <v>157</v>
+      </c>
+      <c r="N53" t="s">
+        <v>158</v>
+      </c>
+      <c r="O53" t="s">
         <v>173</v>
       </c>
-      <c r="I61" t="s">
-        <v>191</v>
-      </c>
-      <c r="J61" t="s">
-        <v>192</v>
-      </c>
-      <c r="K61" t="s">
-        <v>178</v>
-      </c>
-      <c r="M61" t="s">
-        <v>176</v>
-      </c>
-      <c r="N61" t="s">
-        <v>177</v>
-      </c>
-      <c r="O61" t="s">
-        <v>193</v>
-      </c>
-      <c r="P61" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q61" t="s">
-        <v>15</v>
-      </c>
-      <c r="R61" t="s">
-        <v>129</v>
-      </c>
-      <c r="S61" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A64">
-        <v>32937646</v>
-      </c>
-      <c r="B64" t="s">
-        <v>174</v>
-      </c>
-      <c r="C64" t="s">
-        <v>178</v>
-      </c>
-      <c r="G64" t="s">
-        <v>175</v>
-      </c>
-      <c r="H64" t="s">
-        <v>173</v>
-      </c>
-      <c r="I64" t="s">
-        <v>191</v>
-      </c>
-      <c r="J64" t="s">
-        <v>192</v>
-      </c>
-      <c r="K64" t="s">
-        <v>178</v>
-      </c>
-      <c r="M64" t="s">
-        <v>176</v>
-      </c>
-      <c r="N64" t="s">
-        <v>177</v>
-      </c>
-      <c r="O64" t="s">
-        <v>193</v>
-      </c>
-      <c r="P64" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q64" t="s">
-        <v>15</v>
-      </c>
-      <c r="R64" t="s">
-        <v>129</v>
-      </c>
-      <c r="S64" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A67">
-        <v>32937646</v>
-      </c>
-      <c r="B67" t="s">
-        <v>174</v>
-      </c>
-      <c r="C67" t="s">
-        <v>178</v>
-      </c>
-      <c r="G67" t="s">
-        <v>175</v>
-      </c>
-      <c r="H67" t="s">
-        <v>173</v>
-      </c>
-      <c r="I67" t="s">
-        <v>191</v>
-      </c>
-      <c r="J67" t="s">
-        <v>192</v>
-      </c>
-      <c r="K67" t="s">
-        <v>178</v>
-      </c>
-      <c r="M67" t="s">
-        <v>176</v>
-      </c>
-      <c r="N67" t="s">
-        <v>177</v>
-      </c>
-      <c r="O67" t="s">
-        <v>193</v>
-      </c>
-      <c r="P67" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q67" t="s">
-        <v>15</v>
-      </c>
-      <c r="R67" t="s">
-        <v>129</v>
-      </c>
-      <c r="S67" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A70">
-        <v>32937646</v>
-      </c>
-      <c r="B70" t="s">
-        <v>174</v>
-      </c>
-      <c r="C70" t="s">
-        <v>178</v>
-      </c>
-      <c r="G70" t="s">
-        <v>175</v>
-      </c>
-      <c r="H70" t="s">
-        <v>173</v>
-      </c>
-      <c r="I70" t="s">
-        <v>191</v>
-      </c>
-      <c r="J70" t="s">
-        <v>192</v>
-      </c>
-      <c r="K70" t="s">
-        <v>178</v>
-      </c>
-      <c r="M70" t="s">
-        <v>176</v>
-      </c>
-      <c r="N70" t="s">
-        <v>177</v>
-      </c>
-      <c r="O70" t="s">
-        <v>193</v>
-      </c>
-      <c r="P70" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q70" t="s">
-        <v>15</v>
-      </c>
-      <c r="R70" t="s">
-        <v>129</v>
-      </c>
-      <c r="S70" t="s">
-        <v>183</v>
+      <c r="P53" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q53" t="s">
+        <v>10</v>
+      </c>
+      <c r="R53" t="s">
+        <v>110</v>
+      </c>
+      <c r="S53" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20763D68-EA66-4594-BAC3-0F2D52F0EB3F}">
-  <dimension ref="A1:K10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2" t="b">
-        <v>1</v>
-      </c>
-      <c r="K2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" t="b">
-        <v>0</v>
-      </c>
-      <c r="K3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" t="b">
-        <v>0</v>
-      </c>
-      <c r="K4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="D5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J5" t="s">
-        <v>15</v>
-      </c>
-      <c r="K5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="J6" t="b">
-        <v>0</v>
-      </c>
-      <c r="K6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="J7" t="b">
-        <v>0</v>
-      </c>
-      <c r="K7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="J8" t="s">
-        <v>15</v>
-      </c>
-      <c r="K8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="J9" t="b">
-        <v>0</v>
-      </c>
-      <c r="K9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="J10" t="b">
-        <v>0</v>
-      </c>
-      <c r="K10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>